<commit_message>
Add all current cards
Add src info for all the currently planned alpha cards from Justin's doc (name, element, description) - some descriptions are modified and shortened
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\Cards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{904E3C4A-3EF6-4EDE-8AA4-1DF25D224FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241F4646-90AE-4A88-A59D-33D1BCD66787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="15" r:id="rId1"/>
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="49">
   <si>
     <t>FIREBALL</t>
   </si>
@@ -142,28 +142,16 @@
     <t>Light</t>
   </si>
   <si>
-    <t>ricocheting / chain lightning on multiple targets within range</t>
-  </si>
-  <si>
     <t>Modify</t>
   </si>
   <si>
     <t>BG</t>
   </si>
   <si>
-    <t>SPARK</t>
-  </si>
-  <si>
     <t>TIDAL WAVE</t>
   </si>
   <si>
     <t>BRAMBLE SNARE</t>
-  </si>
-  <si>
-    <t>LIFE STEAL</t>
-  </si>
-  <si>
-    <t>VOID HOLE</t>
   </si>
   <si>
     <t>ASTRAL DAGGER</t>
@@ -178,23 +166,95 @@
     <t>Elements</t>
   </si>
   <si>
-    <t>fizzles on walls, explodes on enemies, stun (temp)</t>
+    <t>FROST NOVA</t>
   </si>
   <si>
-    <t>wave carries enemies to wall, deals damage continuously (temp)</t>
+    <t>Deals damage on contact. Explodes against surfaces</t>
   </si>
   <si>
-    <t>snare trap (temp)</t>
+    <t>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</t>
   </si>
   <si>
-    <t>Explodes on anything, Burn DOT (TEMP)</t>
+    <t>Ice</t>
+  </si>
+  <si>
+    <t>Summons a wave that pushes back all enemies it hits, accumulating damage</t>
+  </si>
+  <si>
+    <t>Flies to the nearest enemy in vision</t>
+  </si>
+  <si>
+    <t>Creates a trap area that slows + damages enemies as they move through it</t>
+  </si>
+  <si>
+    <t>BLACK HOLE</t>
+  </si>
+  <si>
+    <t>CHAIN LIGHTNING</t>
+  </si>
+  <si>
+    <t>DIVINE JUDGEMENT</t>
+  </si>
+  <si>
+    <t>Casts a bolt of lightning</t>
+  </si>
+  <si>
+    <t>Vacuums in nearby enemies</t>
+  </si>
+  <si>
+    <t>Casts a tracking bolt of lightning that can chain to close enemies</t>
+  </si>
+  <si>
+    <t>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</t>
+  </si>
+  <si>
+    <t>Haste</t>
+  </si>
+  <si>
+    <t>HINDER</t>
+  </si>
+  <si>
+    <t>MULLIGAN</t>
+  </si>
+  <si>
+    <t>BUT WAIT, THERE'S MORE</t>
+  </si>
+  <si>
+    <t>MANA SHIELD</t>
+  </si>
+  <si>
+    <t>RUNAWAY BULL</t>
+  </si>
+  <si>
+    <t>HOLY BLADE</t>
+  </si>
+  <si>
+    <t>Increases player movement speed for a set duration</t>
+  </si>
+  <si>
+    <t>Enemies are temporarily slowed on hit for a set duration.</t>
+  </si>
+  <si>
+    <t>Randomly swap two cards in the current hand with cards in the deck</t>
+  </si>
+  <si>
+    <t>Randomly shuffle two cards from the discard pile back into the deck</t>
+  </si>
+  <si>
+    <t>Negate x number of hits</t>
+  </si>
+  <si>
+    <t>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</t>
+  </si>
+  <si>
+    <t>Increase damage of your weapon by x for a certain amount of time</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,6 +311,12 @@
     </font>
     <font>
       <sz val="24"/>
+      <color theme="1"/>
+      <name val="Germania One"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="22"/>
       <color theme="1"/>
       <name val="Germania One"/>
       <family val="2"/>
@@ -462,7 +528,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="184">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -531,7 +597,173 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -543,11 +775,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -558,61 +787,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -645,43 +823,73 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -705,159 +913,20 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -915,7 +984,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6276"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6284"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -975,7 +1044,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6277"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6285"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1035,7 +1104,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6278"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6286"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1095,7 +1164,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6279"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6287"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -13108,141 +13177,141 @@
   <sheetData>
     <row r="1" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="170"/>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="172"/>
-      <c r="H2" s="129"/>
-      <c r="I2" s="130"/>
-      <c r="J2" s="130"/>
-      <c r="K2" s="130"/>
-      <c r="L2" s="131"/>
-      <c r="N2" s="143"/>
-      <c r="O2" s="144"/>
-      <c r="P2" s="144"/>
-      <c r="Q2" s="144"/>
-      <c r="R2" s="145"/>
+      <c r="B2" s="101"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="103"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="65"/>
+      <c r="N2" s="76"/>
+      <c r="O2" s="77"/>
+      <c r="P2" s="77"/>
+      <c r="Q2" s="77"/>
+      <c r="R2" s="78"/>
       <c r="T2" s="23"/>
       <c r="U2" s="24"/>
       <c r="V2" s="24"/>
       <c r="W2" s="24"/>
-      <c r="X2" s="157"/>
+      <c r="X2" s="89"/>
     </row>
     <row r="3" spans="2:24" s="58" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="173"/>
-      <c r="C3" s="174"/>
-      <c r="D3" s="174" t="str">
+      <c r="B3" s="104"/>
+      <c r="C3" s="105"/>
+      <c r="D3" s="105" t="str">
         <f>Src!$A5</f>
         <v>FIREBALL</v>
       </c>
-      <c r="E3" s="174"/>
-      <c r="F3" s="175"/>
-      <c r="H3" s="132"/>
-      <c r="I3" s="133"/>
-      <c r="J3" s="133" t="str">
+      <c r="E3" s="105"/>
+      <c r="F3" s="106"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67" t="str">
         <f>Src!A6</f>
-        <v>SPARK</v>
+        <v>FROST NOVA</v>
       </c>
-      <c r="K3" s="133"/>
-      <c r="L3" s="134"/>
-      <c r="N3" s="146"/>
-      <c r="O3" s="147"/>
-      <c r="P3" s="167" t="str">
+      <c r="K3" s="67"/>
+      <c r="L3" s="68"/>
+      <c r="N3" s="79"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="98" t="str">
         <f>Src!A7</f>
         <v>TIDAL WAVE</v>
       </c>
-      <c r="Q3" s="147"/>
-      <c r="R3" s="148"/>
-      <c r="T3" s="158"/>
-      <c r="U3" s="159"/>
-      <c r="V3" s="168" t="str">
+      <c r="Q3" s="80"/>
+      <c r="R3" s="81"/>
+      <c r="T3" s="90"/>
+      <c r="U3" s="91"/>
+      <c r="V3" s="99" t="str">
         <f>Src!A8</f>
         <v>BRAMBLE SNARE</v>
       </c>
-      <c r="W3" s="159"/>
-      <c r="X3" s="160"/>
+      <c r="W3" s="91"/>
+      <c r="X3" s="92"/>
     </row>
     <row r="4" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="176"/>
-      <c r="C4" s="177" t="e" vm="1">
+      <c r="B4" s="107"/>
+      <c r="C4" s="113" t="e" vm="1">
         <f>Src!F5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="177"/>
-      <c r="E4" s="177"/>
-      <c r="F4" s="178"/>
-      <c r="H4" s="135"/>
-      <c r="I4" s="136"/>
-      <c r="J4" s="136"/>
-      <c r="K4" s="136"/>
-      <c r="L4" s="137"/>
-      <c r="N4" s="149"/>
-      <c r="O4" s="150"/>
-      <c r="P4" s="150"/>
-      <c r="Q4" s="150"/>
-      <c r="R4" s="151"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="113"/>
+      <c r="F4" s="108"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="70"/>
+      <c r="J4" s="70"/>
+      <c r="K4" s="70"/>
+      <c r="L4" s="71"/>
+      <c r="N4" s="82"/>
+      <c r="O4" s="83"/>
+      <c r="P4" s="83"/>
+      <c r="Q4" s="83"/>
+      <c r="R4" s="84"/>
       <c r="T4" s="26"/>
-      <c r="U4" s="161"/>
-      <c r="V4" s="161"/>
-      <c r="W4" s="161"/>
-      <c r="X4" s="162"/>
+      <c r="U4" s="93"/>
+      <c r="V4" s="93"/>
+      <c r="W4" s="93"/>
+      <c r="X4" s="94"/>
     </row>
     <row r="5" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="176"/>
-      <c r="C5" s="179" t="str">
+      <c r="B5" s="107"/>
+      <c r="C5" s="181" t="str">
         <f>Src!$C5</f>
-        <v>Explodes on anything, Burn DOT (TEMP)</v>
+        <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="179"/>
-      <c r="E5" s="179"/>
-      <c r="F5" s="180"/>
-      <c r="H5" s="135"/>
-      <c r="I5" s="138" t="str">
+      <c r="D5" s="181"/>
+      <c r="E5" s="181"/>
+      <c r="F5" s="109"/>
+      <c r="H5" s="69"/>
+      <c r="I5" s="180" t="str">
         <f>Src!$C6</f>
-        <v>fizzles on walls, explodes on enemies, stun (temp)</v>
+        <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="J5" s="138"/>
-      <c r="K5" s="138"/>
-      <c r="L5" s="139"/>
-      <c r="N5" s="149"/>
-      <c r="O5" s="152" t="str">
+      <c r="J5" s="180"/>
+      <c r="K5" s="180"/>
+      <c r="L5" s="72"/>
+      <c r="N5" s="82"/>
+      <c r="O5" s="182" t="str">
         <f>Src!C7</f>
-        <v>wave carries enemies to wall, deals damage continuously (temp)</v>
+        <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="P5" s="152"/>
-      <c r="Q5" s="152"/>
-      <c r="R5" s="153"/>
+      <c r="P5" s="182"/>
+      <c r="Q5" s="182"/>
+      <c r="R5" s="85"/>
       <c r="T5" s="26"/>
-      <c r="U5" s="163" t="str">
+      <c r="U5" s="183" t="str">
         <f>Src!C8</f>
-        <v>snare trap (temp)</v>
+        <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="V5" s="163"/>
-      <c r="W5" s="163"/>
-      <c r="X5" s="164"/>
+      <c r="V5" s="183"/>
+      <c r="W5" s="183"/>
+      <c r="X5" s="95"/>
     </row>
     <row r="6" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="181"/>
-      <c r="C6" s="182"/>
-      <c r="D6" s="182"/>
-      <c r="E6" s="182"/>
-      <c r="F6" s="183"/>
-      <c r="H6" s="140"/>
-      <c r="I6" s="141"/>
-      <c r="J6" s="141"/>
-      <c r="K6" s="141"/>
-      <c r="L6" s="142"/>
-      <c r="N6" s="154"/>
-      <c r="O6" s="155"/>
-      <c r="P6" s="155"/>
-      <c r="Q6" s="155"/>
-      <c r="R6" s="156"/>
+      <c r="B6" s="110"/>
+      <c r="C6" s="111"/>
+      <c r="D6" s="111"/>
+      <c r="E6" s="111"/>
+      <c r="F6" s="112"/>
+      <c r="H6" s="73"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="74"/>
+      <c r="L6" s="75"/>
+      <c r="N6" s="86"/>
+      <c r="O6" s="87"/>
+      <c r="P6" s="87"/>
+      <c r="Q6" s="87"/>
+      <c r="R6" s="88"/>
       <c r="T6" s="28"/>
-      <c r="U6" s="165"/>
-      <c r="V6" s="165"/>
-      <c r="W6" s="165"/>
-      <c r="X6" s="166"/>
+      <c r="U6" s="96"/>
+      <c r="V6" s="96"/>
+      <c r="W6" s="96"/>
+      <c r="X6" s="97"/>
     </row>
     <row r="7" spans="2:24" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="8" spans="2:24" ht="393" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13262,7 +13331,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60AA5721-EBD9-4F1E-B70A-78151D63ED79}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.42578125" customWidth="1"/>
@@ -13278,10 +13347,10 @@
       </c>
       <c r="C1" s="58"/>
       <c r="E1" s="58" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G1" s="58" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H1" t="e" vm="2">
         <v>#VALUE!</v>
@@ -13311,7 +13380,7 @@
       </c>
       <c r="E4" s="60"/>
       <c r="F4" s="60" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="61" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
@@ -13321,10 +13390,10 @@
       <c r="B5" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="60" t="s">
-        <v>28</v>
+      <c r="C5" s="100" t="s">
+        <v>22</v>
       </c>
-      <c r="D5" s="60" t="s">
+      <c r="D5" s="184" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="60"/>
@@ -13332,101 +13401,237 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="169" t="s">
+    <row r="6" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="100" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="100" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="100" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="184" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="100" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="100" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="100" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="184" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="169" t="s">
+      <c r="B8" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="169" t="s">
-        <v>25</v>
+      <c r="C8" s="100" t="s">
+        <v>27</v>
       </c>
-      <c r="D6" s="169" t="s">
+      <c r="D8" s="184" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="100" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="100" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="100" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="184" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="169" t="s">
-        <v>17</v>
+    <row r="10" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="100" t="s">
+        <v>28</v>
       </c>
-      <c r="B7" s="169" t="s">
+      <c r="B10" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="169" t="s">
-        <v>26</v>
+      <c r="C10" s="100" t="s">
+        <v>32</v>
       </c>
-      <c r="D7" s="169" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="169" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="169" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="169" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="169" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="169" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="169" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="169" t="s">
+      <c r="D10" s="184" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="169" t="s">
-        <v>20</v>
+    <row r="11" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="100" t="s">
+        <v>17</v>
       </c>
-      <c r="B10" s="169" t="s">
+      <c r="B11" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="169" t="s">
-        <v>11</v>
+      <c r="C11" s="100" t="s">
+        <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="169" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="169" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="169" t="s">
+      <c r="D11" s="184" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="169" t="s">
-        <v>22</v>
+    <row r="12" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="100" t="s">
+        <v>29</v>
       </c>
-      <c r="B12" s="169" t="s">
+      <c r="B12" s="100" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="169" t="s">
+      <c r="C12" s="100" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="184" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="100" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="100" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="100" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="184" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="100" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="169" t="s">
-        <v>8</v>
+      <c r="C14" s="100" t="s">
+        <v>42</v>
       </c>
-      <c r="E12" s="169" t="s">
+      <c r="D14" s="184"/>
+    </row>
+    <row r="15" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="100" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="100" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="184"/>
+    </row>
+    <row r="16" spans="1:8" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="100" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="100" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="184"/>
+    </row>
+    <row r="17" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="100" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="100" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="184"/>
+    </row>
+    <row r="18" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="100" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="100" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="184"/>
+    </row>
+    <row r="19" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="100" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="184"/>
+    </row>
+    <row r="20" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="100" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="100" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="184"/>
+    </row>
+    <row r="21" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="184"/>
+    </row>
+    <row r="22" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="100" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="184"/>
+    </row>
+    <row r="23" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="100" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="169" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="169" t="s">
-        <v>14</v>
+    <row r="24" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="100" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="100" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="100" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="100" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="100" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -13461,7 +13666,7 @@
     <row r="3" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
-      <c r="E3" s="125" t="str">
+      <c r="E3" s="121" t="str">
         <f>Src!A5</f>
         <v>FIREBALL</v>
       </c>
@@ -13469,71 +13674,71 @@
       <c r="G3" s="11"/>
       <c r="K3" s="1"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="109"/>
+      <c r="M3" s="123"/>
       <c r="N3" s="2"/>
       <c r="O3" s="3"/>
     </row>
     <row r="4" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="12"/>
-      <c r="D4" s="111"/>
-      <c r="E4" s="126"/>
-      <c r="F4" s="111"/>
+      <c r="D4" s="125"/>
+      <c r="E4" s="122"/>
+      <c r="F4" s="125"/>
       <c r="G4" s="13"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="67"/>
-      <c r="M4" s="110"/>
-      <c r="N4" s="67"/>
+      <c r="L4" s="126"/>
+      <c r="M4" s="124"/>
+      <c r="N4" s="126"/>
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="12"/>
-      <c r="D5" s="111"/>
-      <c r="E5" s="126"/>
-      <c r="F5" s="111"/>
+      <c r="D5" s="125"/>
+      <c r="E5" s="122"/>
+      <c r="F5" s="125"/>
       <c r="G5" s="13"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="67"/>
-      <c r="M5" s="110"/>
-      <c r="N5" s="67"/>
+      <c r="L5" s="126"/>
+      <c r="M5" s="124"/>
+      <c r="N5" s="126"/>
       <c r="O5" s="5"/>
     </row>
     <row r="6" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C6" s="12"/>
-      <c r="D6" s="107"/>
-      <c r="E6" s="107"/>
-      <c r="F6" s="107"/>
+      <c r="D6" s="117"/>
+      <c r="E6" s="117"/>
+      <c r="F6" s="117"/>
       <c r="G6" s="13"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="108"/>
-      <c r="M6" s="108"/>
-      <c r="N6" s="108"/>
+      <c r="L6" s="118"/>
+      <c r="M6" s="118"/>
+      <c r="N6" s="118"/>
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="12"/>
-      <c r="D7" s="128" t="str">
+      <c r="D7" s="116" t="str">
         <f>Src!C5</f>
-        <v>Explodes on anything, Burn DOT (TEMP)</v>
+        <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="E7" s="128"/>
-      <c r="F7" s="128"/>
-      <c r="G7" s="127"/>
+      <c r="E7" s="116"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="62"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="78"/>
-      <c r="M7" s="78"/>
-      <c r="N7" s="78"/>
-      <c r="O7" s="79"/>
+      <c r="L7" s="119"/>
+      <c r="M7" s="119"/>
+      <c r="N7" s="119"/>
+      <c r="O7" s="120"/>
     </row>
     <row r="8" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="14"/>
-      <c r="D8" s="112"/>
-      <c r="E8" s="112"/>
-      <c r="F8" s="112"/>
+      <c r="D8" s="114"/>
+      <c r="E8" s="114"/>
+      <c r="F8" s="114"/>
       <c r="G8" s="15"/>
       <c r="K8" s="6"/>
-      <c r="L8" s="76"/>
-      <c r="M8" s="76"/>
-      <c r="N8" s="76"/>
+      <c r="L8" s="115"/>
+      <c r="M8" s="115"/>
+      <c r="N8" s="115"/>
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13541,73 +13746,73 @@
     <row r="12" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="16"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="105"/>
+      <c r="E12" s="138"/>
       <c r="F12" s="17"/>
       <c r="G12" s="18"/>
       <c r="K12" s="1"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="68"/>
+      <c r="M12" s="135"/>
       <c r="N12" s="2"/>
       <c r="O12" s="3"/>
     </row>
     <row r="13" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="19"/>
-      <c r="D13" s="103"/>
-      <c r="E13" s="106"/>
-      <c r="F13" s="103"/>
+      <c r="D13" s="130"/>
+      <c r="E13" s="139"/>
+      <c r="F13" s="130"/>
       <c r="G13" s="20"/>
       <c r="K13" s="4"/>
-      <c r="L13" s="67"/>
-      <c r="M13" s="69"/>
-      <c r="N13" s="67"/>
+      <c r="L13" s="126"/>
+      <c r="M13" s="136"/>
+      <c r="N13" s="126"/>
       <c r="O13" s="5"/>
     </row>
     <row r="14" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="19"/>
-      <c r="D14" s="103"/>
-      <c r="E14" s="106"/>
-      <c r="F14" s="103"/>
+      <c r="D14" s="130"/>
+      <c r="E14" s="139"/>
+      <c r="F14" s="130"/>
       <c r="G14" s="20"/>
       <c r="K14" s="4"/>
-      <c r="L14" s="67"/>
-      <c r="M14" s="70"/>
-      <c r="N14" s="67"/>
+      <c r="L14" s="126"/>
+      <c r="M14" s="137"/>
+      <c r="N14" s="126"/>
       <c r="O14" s="5"/>
     </row>
     <row r="15" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C15" s="19"/>
-      <c r="D15" s="104"/>
-      <c r="E15" s="104"/>
-      <c r="F15" s="104"/>
+      <c r="D15" s="134"/>
+      <c r="E15" s="134"/>
+      <c r="F15" s="134"/>
       <c r="G15" s="20"/>
       <c r="K15" s="4"/>
-      <c r="L15" s="63"/>
-      <c r="M15" s="64"/>
-      <c r="N15" s="65"/>
+      <c r="L15" s="131"/>
+      <c r="M15" s="132"/>
+      <c r="N15" s="133"/>
       <c r="O15" s="5"/>
     </row>
     <row r="16" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="19"/>
-      <c r="D16" s="101"/>
-      <c r="E16" s="101"/>
-      <c r="F16" s="101"/>
-      <c r="G16" s="102"/>
+      <c r="D16" s="128"/>
+      <c r="E16" s="128"/>
+      <c r="F16" s="128"/>
+      <c r="G16" s="129"/>
       <c r="K16" s="4"/>
-      <c r="L16" s="78"/>
-      <c r="M16" s="78"/>
-      <c r="N16" s="78"/>
-      <c r="O16" s="79"/>
+      <c r="L16" s="119"/>
+      <c r="M16" s="119"/>
+      <c r="N16" s="119"/>
+      <c r="O16" s="120"/>
     </row>
     <row r="17" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17" s="21"/>
-      <c r="D17" s="100"/>
-      <c r="E17" s="100"/>
-      <c r="F17" s="100"/>
+      <c r="D17" s="127"/>
+      <c r="E17" s="127"/>
+      <c r="F17" s="127"/>
       <c r="G17" s="22"/>
       <c r="K17" s="6"/>
-      <c r="L17" s="76"/>
-      <c r="M17" s="76"/>
-      <c r="N17" s="76"/>
+      <c r="L17" s="115"/>
+      <c r="M17" s="115"/>
+      <c r="N17" s="115"/>
       <c r="O17" s="7"/>
     </row>
     <row r="18" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13615,73 +13820,73 @@
     <row r="21" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="23"/>
       <c r="D21" s="24"/>
-      <c r="E21" s="91"/>
+      <c r="E21" s="141"/>
       <c r="F21" s="24"/>
       <c r="G21" s="25"/>
       <c r="K21" s="1"/>
       <c r="L21" s="2"/>
-      <c r="M21" s="68"/>
+      <c r="M21" s="135"/>
       <c r="N21" s="2"/>
       <c r="O21" s="3"/>
     </row>
     <row r="22" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="26"/>
-      <c r="D22" s="90"/>
-      <c r="E22" s="92"/>
-      <c r="F22" s="90"/>
+      <c r="D22" s="140"/>
+      <c r="E22" s="142"/>
+      <c r="F22" s="140"/>
       <c r="G22" s="27"/>
       <c r="K22" s="4"/>
-      <c r="L22" s="67"/>
-      <c r="M22" s="69"/>
-      <c r="N22" s="67"/>
+      <c r="L22" s="126"/>
+      <c r="M22" s="136"/>
+      <c r="N22" s="126"/>
       <c r="O22" s="5"/>
     </row>
     <row r="23" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="26"/>
-      <c r="D23" s="90"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="90"/>
+      <c r="D23" s="140"/>
+      <c r="E23" s="142"/>
+      <c r="F23" s="140"/>
       <c r="G23" s="27"/>
       <c r="K23" s="4"/>
-      <c r="L23" s="67"/>
-      <c r="M23" s="70"/>
-      <c r="N23" s="67"/>
+      <c r="L23" s="126"/>
+      <c r="M23" s="137"/>
+      <c r="N23" s="126"/>
       <c r="O23" s="5"/>
     </row>
     <row r="24" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C24" s="26"/>
-      <c r="D24" s="99"/>
-      <c r="E24" s="99"/>
-      <c r="F24" s="99"/>
+      <c r="D24" s="149"/>
+      <c r="E24" s="149"/>
+      <c r="F24" s="149"/>
       <c r="G24" s="27"/>
       <c r="K24" s="4"/>
-      <c r="L24" s="63"/>
-      <c r="M24" s="64"/>
-      <c r="N24" s="65"/>
+      <c r="L24" s="131"/>
+      <c r="M24" s="132"/>
+      <c r="N24" s="133"/>
       <c r="O24" s="5"/>
     </row>
     <row r="25" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="26"/>
-      <c r="D25" s="97"/>
-      <c r="E25" s="97"/>
-      <c r="F25" s="97"/>
-      <c r="G25" s="98"/>
+      <c r="D25" s="147"/>
+      <c r="E25" s="147"/>
+      <c r="F25" s="147"/>
+      <c r="G25" s="148"/>
       <c r="K25" s="4"/>
-      <c r="L25" s="78"/>
-      <c r="M25" s="78"/>
-      <c r="N25" s="78"/>
-      <c r="O25" s="79"/>
+      <c r="L25" s="119"/>
+      <c r="M25" s="119"/>
+      <c r="N25" s="119"/>
+      <c r="O25" s="120"/>
     </row>
     <row r="26" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C26" s="28"/>
-      <c r="D26" s="96"/>
-      <c r="E26" s="96"/>
-      <c r="F26" s="96"/>
+      <c r="D26" s="146"/>
+      <c r="E26" s="146"/>
+      <c r="F26" s="146"/>
       <c r="G26" s="29"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="76"/>
-      <c r="M26" s="76"/>
-      <c r="N26" s="76"/>
+      <c r="L26" s="115"/>
+      <c r="M26" s="115"/>
+      <c r="N26" s="115"/>
       <c r="O26" s="7"/>
     </row>
     <row r="27" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13689,73 +13894,73 @@
     <row r="30" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="37"/>
       <c r="D30" s="38"/>
-      <c r="E30" s="88"/>
+      <c r="E30" s="156"/>
       <c r="F30" s="38"/>
       <c r="G30" s="39"/>
       <c r="K30" s="1"/>
       <c r="L30" s="2"/>
-      <c r="M30" s="68"/>
+      <c r="M30" s="135"/>
       <c r="N30" s="2"/>
       <c r="O30" s="3"/>
     </row>
     <row r="31" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="40"/>
-      <c r="D31" s="82"/>
-      <c r="E31" s="89"/>
-      <c r="F31" s="82"/>
+      <c r="D31" s="150"/>
+      <c r="E31" s="157"/>
+      <c r="F31" s="150"/>
       <c r="G31" s="41"/>
       <c r="K31" s="4"/>
-      <c r="L31" s="67"/>
-      <c r="M31" s="69"/>
-      <c r="N31" s="67"/>
+      <c r="L31" s="126"/>
+      <c r="M31" s="136"/>
+      <c r="N31" s="126"/>
       <c r="O31" s="5"/>
     </row>
     <row r="32" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="40"/>
-      <c r="D32" s="82"/>
-      <c r="E32" s="89"/>
-      <c r="F32" s="82"/>
+      <c r="D32" s="150"/>
+      <c r="E32" s="157"/>
+      <c r="F32" s="150"/>
       <c r="G32" s="41"/>
       <c r="K32" s="4"/>
-      <c r="L32" s="67"/>
-      <c r="M32" s="70"/>
-      <c r="N32" s="67"/>
+      <c r="L32" s="126"/>
+      <c r="M32" s="137"/>
+      <c r="N32" s="126"/>
       <c r="O32" s="5"/>
     </row>
     <row r="33" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C33" s="40"/>
-      <c r="D33" s="87"/>
-      <c r="E33" s="87"/>
-      <c r="F33" s="87"/>
+      <c r="D33" s="155"/>
+      <c r="E33" s="155"/>
+      <c r="F33" s="155"/>
       <c r="G33" s="41"/>
       <c r="K33" s="4"/>
-      <c r="L33" s="63"/>
-      <c r="M33" s="64"/>
-      <c r="N33" s="65"/>
+      <c r="L33" s="131"/>
+      <c r="M33" s="132"/>
+      <c r="N33" s="133"/>
       <c r="O33" s="5"/>
     </row>
     <row r="34" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="40"/>
-      <c r="D34" s="94"/>
-      <c r="E34" s="94"/>
-      <c r="F34" s="94"/>
-      <c r="G34" s="95"/>
+      <c r="D34" s="144"/>
+      <c r="E34" s="144"/>
+      <c r="F34" s="144"/>
+      <c r="G34" s="145"/>
       <c r="K34" s="4"/>
-      <c r="L34" s="78"/>
-      <c r="M34" s="78"/>
-      <c r="N34" s="78"/>
-      <c r="O34" s="79"/>
+      <c r="L34" s="119"/>
+      <c r="M34" s="119"/>
+      <c r="N34" s="119"/>
+      <c r="O34" s="120"/>
     </row>
     <row r="35" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C35" s="42"/>
-      <c r="D35" s="93"/>
-      <c r="E35" s="93"/>
-      <c r="F35" s="93"/>
+      <c r="D35" s="143"/>
+      <c r="E35" s="143"/>
+      <c r="F35" s="143"/>
       <c r="G35" s="43"/>
       <c r="K35" s="6"/>
-      <c r="L35" s="76"/>
-      <c r="M35" s="76"/>
-      <c r="N35" s="76"/>
+      <c r="L35" s="115"/>
+      <c r="M35" s="115"/>
+      <c r="N35" s="115"/>
       <c r="O35" s="7"/>
     </row>
     <row r="36" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13763,73 +13968,73 @@
     <row r="39" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C39" s="44"/>
       <c r="D39" s="45"/>
-      <c r="E39" s="74"/>
+      <c r="E39" s="159"/>
       <c r="F39" s="45"/>
       <c r="G39" s="46"/>
       <c r="K39" s="1"/>
       <c r="L39" s="2"/>
-      <c r="M39" s="68"/>
+      <c r="M39" s="135"/>
       <c r="N39" s="2"/>
       <c r="O39" s="3"/>
     </row>
     <row r="40" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C40" s="47"/>
-      <c r="D40" s="73"/>
-      <c r="E40" s="75"/>
-      <c r="F40" s="73"/>
+      <c r="D40" s="158"/>
+      <c r="E40" s="160"/>
+      <c r="F40" s="158"/>
       <c r="G40" s="48"/>
       <c r="K40" s="4"/>
-      <c r="L40" s="67"/>
-      <c r="M40" s="69"/>
-      <c r="N40" s="67"/>
+      <c r="L40" s="126"/>
+      <c r="M40" s="136"/>
+      <c r="N40" s="126"/>
       <c r="O40" s="5"/>
     </row>
     <row r="41" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C41" s="47"/>
-      <c r="D41" s="73"/>
-      <c r="E41" s="75"/>
-      <c r="F41" s="73"/>
+      <c r="D41" s="158"/>
+      <c r="E41" s="160"/>
+      <c r="F41" s="158"/>
       <c r="G41" s="48"/>
       <c r="K41" s="4"/>
-      <c r="L41" s="67"/>
-      <c r="M41" s="70"/>
-      <c r="N41" s="67"/>
+      <c r="L41" s="126"/>
+      <c r="M41" s="137"/>
+      <c r="N41" s="126"/>
       <c r="O41" s="5"/>
     </row>
     <row r="42" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C42" s="47"/>
-      <c r="D42" s="86"/>
-      <c r="E42" s="86"/>
-      <c r="F42" s="86"/>
+      <c r="D42" s="154"/>
+      <c r="E42" s="154"/>
+      <c r="F42" s="154"/>
       <c r="G42" s="48"/>
       <c r="K42" s="4"/>
-      <c r="L42" s="63"/>
-      <c r="M42" s="64"/>
-      <c r="N42" s="65"/>
+      <c r="L42" s="131"/>
+      <c r="M42" s="132"/>
+      <c r="N42" s="133"/>
       <c r="O42" s="5"/>
     </row>
     <row r="43" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C43" s="47"/>
-      <c r="D43" s="84"/>
-      <c r="E43" s="84"/>
-      <c r="F43" s="84"/>
-      <c r="G43" s="85"/>
+      <c r="D43" s="152"/>
+      <c r="E43" s="152"/>
+      <c r="F43" s="152"/>
+      <c r="G43" s="153"/>
       <c r="K43" s="4"/>
-      <c r="L43" s="78"/>
-      <c r="M43" s="78"/>
-      <c r="N43" s="78"/>
-      <c r="O43" s="79"/>
+      <c r="L43" s="119"/>
+      <c r="M43" s="119"/>
+      <c r="N43" s="119"/>
+      <c r="O43" s="120"/>
     </row>
     <row r="44" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C44" s="49"/>
-      <c r="D44" s="83"/>
-      <c r="E44" s="83"/>
-      <c r="F44" s="83"/>
+      <c r="D44" s="151"/>
+      <c r="E44" s="151"/>
+      <c r="F44" s="151"/>
       <c r="G44" s="50"/>
       <c r="K44" s="6"/>
-      <c r="L44" s="76"/>
-      <c r="M44" s="76"/>
-      <c r="N44" s="76"/>
+      <c r="L44" s="115"/>
+      <c r="M44" s="115"/>
+      <c r="N44" s="115"/>
       <c r="O44" s="7"/>
     </row>
     <row r="45" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -13837,102 +14042,110 @@
     <row r="48" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C48" s="51"/>
       <c r="D48" s="52"/>
-      <c r="E48" s="71"/>
+      <c r="E48" s="166"/>
       <c r="F48" s="52"/>
       <c r="G48" s="53"/>
       <c r="K48" s="1"/>
       <c r="L48" s="2"/>
-      <c r="M48" s="68"/>
+      <c r="M48" s="135"/>
       <c r="N48" s="2"/>
       <c r="O48" s="3"/>
     </row>
     <row r="49" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C49" s="54"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="72"/>
-      <c r="F49" s="62"/>
+      <c r="D49" s="164"/>
+      <c r="E49" s="167"/>
+      <c r="F49" s="164"/>
       <c r="G49" s="55"/>
       <c r="K49" s="4"/>
-      <c r="L49" s="67"/>
-      <c r="M49" s="69"/>
-      <c r="N49" s="67"/>
+      <c r="L49" s="126"/>
+      <c r="M49" s="136"/>
+      <c r="N49" s="126"/>
       <c r="O49" s="5"/>
     </row>
     <row r="50" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C50" s="54"/>
-      <c r="D50" s="62"/>
-      <c r="E50" s="72"/>
-      <c r="F50" s="62"/>
+      <c r="D50" s="164"/>
+      <c r="E50" s="167"/>
+      <c r="F50" s="164"/>
       <c r="G50" s="55"/>
       <c r="K50" s="4"/>
-      <c r="L50" s="67"/>
-      <c r="M50" s="70"/>
-      <c r="N50" s="67"/>
+      <c r="L50" s="126"/>
+      <c r="M50" s="137"/>
+      <c r="N50" s="126"/>
       <c r="O50" s="5"/>
     </row>
     <row r="51" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C51" s="54"/>
-      <c r="D51" s="66"/>
-      <c r="E51" s="66"/>
-      <c r="F51" s="66"/>
+      <c r="D51" s="165"/>
+      <c r="E51" s="165"/>
+      <c r="F51" s="165"/>
       <c r="G51" s="55"/>
       <c r="K51" s="4"/>
-      <c r="L51" s="63"/>
-      <c r="M51" s="64"/>
-      <c r="N51" s="65"/>
+      <c r="L51" s="131"/>
+      <c r="M51" s="132"/>
+      <c r="N51" s="133"/>
       <c r="O51" s="5"/>
     </row>
     <row r="52" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C52" s="54"/>
-      <c r="D52" s="80"/>
-      <c r="E52" s="80"/>
-      <c r="F52" s="80"/>
-      <c r="G52" s="81"/>
+      <c r="D52" s="162"/>
+      <c r="E52" s="162"/>
+      <c r="F52" s="162"/>
+      <c r="G52" s="163"/>
       <c r="K52" s="4"/>
-      <c r="L52" s="78"/>
-      <c r="M52" s="78"/>
-      <c r="N52" s="78"/>
-      <c r="O52" s="79"/>
+      <c r="L52" s="119"/>
+      <c r="M52" s="119"/>
+      <c r="N52" s="119"/>
+      <c r="O52" s="120"/>
     </row>
     <row r="53" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C53" s="56"/>
-      <c r="D53" s="77"/>
-      <c r="E53" s="77"/>
-      <c r="F53" s="77"/>
+      <c r="D53" s="161"/>
+      <c r="E53" s="161"/>
+      <c r="F53" s="161"/>
       <c r="G53" s="57"/>
       <c r="K53" s="6"/>
-      <c r="L53" s="76"/>
-      <c r="M53" s="76"/>
-      <c r="N53" s="76"/>
+      <c r="L53" s="115"/>
+      <c r="M53" s="115"/>
+      <c r="N53" s="115"/>
       <c r="O53" s="7"/>
     </row>
     <row r="54" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="M3:M5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="L16:O16"/>
-    <mergeCell ref="D16:G16"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="L15:N15"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="M12:M14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="L53:N53"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="L52:O52"/>
+    <mergeCell ref="D52:G52"/>
+    <mergeCell ref="N40:N41"/>
+    <mergeCell ref="M39:M41"/>
+    <mergeCell ref="L40:L41"/>
+    <mergeCell ref="D49:D50"/>
+    <mergeCell ref="L51:N51"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="N49:N50"/>
+    <mergeCell ref="M48:M50"/>
+    <mergeCell ref="L49:L50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="L44:N44"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="L43:O43"/>
+    <mergeCell ref="D43:G43"/>
+    <mergeCell ref="L42:N42"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="N31:N32"/>
+    <mergeCell ref="M30:M32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="E30:E32"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="E39:E41"/>
     <mergeCell ref="F22:F23"/>
     <mergeCell ref="E21:E23"/>
     <mergeCell ref="D22:D23"/>
@@ -13949,38 +14162,30 @@
     <mergeCell ref="D25:G25"/>
     <mergeCell ref="L24:N24"/>
     <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="L43:O43"/>
-    <mergeCell ref="D43:G43"/>
-    <mergeCell ref="L42:N42"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="N31:N32"/>
-    <mergeCell ref="M30:M32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="E30:E32"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="E39:E41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="L53:N53"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="L52:O52"/>
-    <mergeCell ref="D52:G52"/>
-    <mergeCell ref="N40:N41"/>
-    <mergeCell ref="M39:M41"/>
-    <mergeCell ref="L40:L41"/>
-    <mergeCell ref="D49:D50"/>
-    <mergeCell ref="L51:N51"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="N49:N50"/>
-    <mergeCell ref="M48:M50"/>
-    <mergeCell ref="L49:L50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="L16:O16"/>
+    <mergeCell ref="D16:G16"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="L15:N15"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="M12:M14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="M3:M5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="L7:O7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -14028,7 +14233,7 @@
     <row r="3" spans="3:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="30"/>
       <c r="D3" s="31"/>
-      <c r="E3" s="114"/>
+      <c r="E3" s="174"/>
       <c r="F3" s="31"/>
       <c r="G3" s="32"/>
       <c r="K3" s="1"/>
@@ -14036,130 +14241,136 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="3"/>
-      <c r="R3" s="124"/>
-      <c r="S3" s="124"/>
-      <c r="T3" s="124"/>
-      <c r="U3" s="124"/>
-      <c r="V3" s="124"/>
+      <c r="R3" s="172"/>
+      <c r="S3" s="172"/>
+      <c r="T3" s="172"/>
+      <c r="U3" s="172"/>
+      <c r="V3" s="172"/>
       <c r="Z3" s="1"/>
       <c r="AA3" s="2"/>
-      <c r="AB3" s="68"/>
+      <c r="AB3" s="135"/>
       <c r="AC3" s="2"/>
       <c r="AD3" s="3"/>
     </row>
     <row r="4" spans="3:30" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="33"/>
-      <c r="D4" s="118"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="118"/>
+      <c r="D4" s="178"/>
+      <c r="E4" s="175"/>
+      <c r="F4" s="178"/>
       <c r="G4" s="34"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="67"/>
+      <c r="L4" s="126"/>
       <c r="M4" s="8"/>
-      <c r="N4" s="67"/>
+      <c r="N4" s="126"/>
       <c r="O4" s="5"/>
-      <c r="R4" s="124"/>
-      <c r="S4" s="124"/>
-      <c r="T4" s="124"/>
-      <c r="U4" s="124"/>
-      <c r="V4" s="124"/>
+      <c r="R4" s="172"/>
+      <c r="S4" s="172"/>
+      <c r="T4" s="172"/>
+      <c r="U4" s="172"/>
+      <c r="V4" s="172"/>
       <c r="Z4" s="4"/>
-      <c r="AA4" s="67"/>
-      <c r="AB4" s="69"/>
-      <c r="AC4" s="67"/>
+      <c r="AA4" s="126"/>
+      <c r="AB4" s="136"/>
+      <c r="AC4" s="126"/>
       <c r="AD4" s="5"/>
     </row>
     <row r="5" spans="3:30" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="33"/>
-      <c r="D5" s="118"/>
-      <c r="E5" s="115"/>
-      <c r="F5" s="118"/>
+      <c r="D5" s="178"/>
+      <c r="E5" s="175"/>
+      <c r="F5" s="178"/>
       <c r="G5" s="34"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="67"/>
+      <c r="L5" s="126"/>
       <c r="M5" s="8"/>
-      <c r="N5" s="67"/>
+      <c r="N5" s="126"/>
       <c r="O5" s="5"/>
-      <c r="R5" s="124"/>
-      <c r="S5" s="124"/>
-      <c r="T5" s="124"/>
-      <c r="U5" s="124"/>
-      <c r="V5" s="124"/>
+      <c r="R5" s="172"/>
+      <c r="S5" s="172"/>
+      <c r="T5" s="172"/>
+      <c r="U5" s="172"/>
+      <c r="V5" s="172"/>
       <c r="Z5" s="4"/>
-      <c r="AA5" s="67"/>
-      <c r="AB5" s="69"/>
-      <c r="AC5" s="67"/>
+      <c r="AA5" s="126"/>
+      <c r="AB5" s="136"/>
+      <c r="AC5" s="126"/>
       <c r="AD5" s="5"/>
     </row>
     <row r="6" spans="3:30" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C6" s="33"/>
-      <c r="D6" s="119"/>
-      <c r="E6" s="119"/>
-      <c r="F6" s="119"/>
+      <c r="D6" s="179"/>
+      <c r="E6" s="179"/>
+      <c r="F6" s="179"/>
       <c r="G6" s="34"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="120"/>
-      <c r="M6" s="121"/>
-      <c r="N6" s="122"/>
+      <c r="L6" s="168"/>
+      <c r="M6" s="169"/>
+      <c r="N6" s="170"/>
       <c r="O6" s="5"/>
-      <c r="R6" s="124"/>
-      <c r="S6" s="124"/>
-      <c r="T6" s="124"/>
-      <c r="U6" s="124"/>
-      <c r="V6" s="124"/>
+      <c r="R6" s="172"/>
+      <c r="S6" s="172"/>
+      <c r="T6" s="172"/>
+      <c r="U6" s="172"/>
+      <c r="V6" s="172"/>
       <c r="Z6" s="4"/>
-      <c r="AA6" s="108"/>
-      <c r="AB6" s="108"/>
-      <c r="AC6" s="108"/>
+      <c r="AA6" s="118"/>
+      <c r="AB6" s="118"/>
+      <c r="AC6" s="118"/>
       <c r="AD6" s="5"/>
     </row>
     <row r="7" spans="3:30" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="33"/>
-      <c r="D7" s="116"/>
-      <c r="E7" s="116"/>
-      <c r="F7" s="116"/>
-      <c r="G7" s="117"/>
+      <c r="D7" s="176"/>
+      <c r="E7" s="176"/>
+      <c r="F7" s="176"/>
+      <c r="G7" s="177"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="123"/>
-      <c r="M7" s="123"/>
-      <c r="N7" s="123"/>
+      <c r="L7" s="171"/>
+      <c r="M7" s="171"/>
+      <c r="N7" s="171"/>
       <c r="O7" s="5"/>
-      <c r="R7" s="124"/>
-      <c r="S7" s="124"/>
-      <c r="T7" s="124"/>
-      <c r="U7" s="124"/>
-      <c r="V7" s="124"/>
+      <c r="R7" s="172"/>
+      <c r="S7" s="172"/>
+      <c r="T7" s="172"/>
+      <c r="U7" s="172"/>
+      <c r="V7" s="172"/>
       <c r="Z7" s="4"/>
-      <c r="AA7" s="78"/>
-      <c r="AB7" s="78"/>
-      <c r="AC7" s="78"/>
-      <c r="AD7" s="79"/>
+      <c r="AA7" s="119"/>
+      <c r="AB7" s="119"/>
+      <c r="AC7" s="119"/>
+      <c r="AD7" s="120"/>
     </row>
     <row r="8" spans="3:30" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="35"/>
-      <c r="D8" s="113"/>
-      <c r="E8" s="113"/>
-      <c r="F8" s="113"/>
+      <c r="D8" s="173"/>
+      <c r="E8" s="173"/>
+      <c r="F8" s="173"/>
       <c r="G8" s="36"/>
       <c r="K8" s="6"/>
-      <c r="L8" s="76"/>
-      <c r="M8" s="76"/>
-      <c r="N8" s="76"/>
+      <c r="L8" s="115"/>
+      <c r="M8" s="115"/>
+      <c r="N8" s="115"/>
       <c r="O8" s="7"/>
-      <c r="R8" s="124"/>
-      <c r="S8" s="124"/>
-      <c r="T8" s="124"/>
-      <c r="U8" s="124"/>
-      <c r="V8" s="124"/>
+      <c r="R8" s="172"/>
+      <c r="S8" s="172"/>
+      <c r="T8" s="172"/>
+      <c r="U8" s="172"/>
+      <c r="V8" s="172"/>
       <c r="Z8" s="6"/>
-      <c r="AA8" s="76"/>
-      <c r="AB8" s="76"/>
-      <c r="AC8" s="76"/>
+      <c r="AA8" s="115"/>
+      <c r="AB8" s="115"/>
+      <c r="AC8" s="115"/>
       <c r="AD8" s="7"/>
     </row>
     <row r="9" spans="3:30" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="D6:F6"/>
     <mergeCell ref="N4:N5"/>
     <mergeCell ref="L6:N6"/>
     <mergeCell ref="L8:N8"/>
@@ -14172,12 +14383,6 @@
     <mergeCell ref="AA6:AC6"/>
     <mergeCell ref="AA7:AD7"/>
     <mergeCell ref="L4:L5"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="D6:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Attack card art WIP
Added brief temporary art for each attack card that will be changed as I work on them
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D08244B-30B6-4F20-9F92-2F74F44EBFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267C5140-6AF5-415C-979F-318696290F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="11">
+  <futureMetadata name="XLRICHVALUE" count="27">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -121,8 +121,120 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="11"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="12"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="13"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="14"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="15"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="16"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="17"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="18"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="19"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="20"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="21"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="22"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="23"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="24"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="25"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="26"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="11">
+  <valueMetadata count="27">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -155,6 +267,54 @@
     </bk>
     <bk>
       <rc t="1" v="10"/>
+    </bk>
+    <bk>
+      <rc t="1" v="11"/>
+    </bk>
+    <bk>
+      <rc t="1" v="12"/>
+    </bk>
+    <bk>
+      <rc t="1" v="13"/>
+    </bk>
+    <bk>
+      <rc t="1" v="14"/>
+    </bk>
+    <bk>
+      <rc t="1" v="15"/>
+    </bk>
+    <bk>
+      <rc t="1" v="16"/>
+    </bk>
+    <bk>
+      <rc t="1" v="17"/>
+    </bk>
+    <bk>
+      <rc t="1" v="18"/>
+    </bk>
+    <bk>
+      <rc t="1" v="19"/>
+    </bk>
+    <bk>
+      <rc t="1" v="20"/>
+    </bk>
+    <bk>
+      <rc t="1" v="21"/>
+    </bk>
+    <bk>
+      <rc t="1" v="22"/>
+    </bk>
+    <bk>
+      <rc t="1" v="23"/>
+    </bk>
+    <bk>
+      <rc t="1" v="24"/>
+    </bk>
+    <bk>
+      <rc t="1" v="25"/>
+    </bk>
+    <bk>
+      <rc t="1" v="26"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -220,9 +380,6 @@
     <t>Art</t>
   </si>
   <si>
-    <t>Elements</t>
-  </si>
-  <si>
     <t>FROST NOVA</t>
   </si>
   <si>
@@ -263,9 +420,6 @@
   </si>
   <si>
     <t>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</t>
-  </si>
-  <si>
-    <t>Haste</t>
   </si>
   <si>
     <t>HINDER</t>
@@ -311,6 +465,12 @@
   </si>
   <si>
     <t>Draw</t>
+  </si>
+  <si>
+    <t>HASTE</t>
+  </si>
+  <si>
+    <t>Icons</t>
   </si>
 </sst>
 </file>
@@ -403,7 +563,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -490,19 +650,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA9D08E"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFE699"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFD6DCE4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -645,7 +799,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="261">
+  <cellXfs count="247">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -714,18 +868,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -741,7 +883,6 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -784,9 +925,6 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -802,7 +940,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -829,7 +966,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -839,9 +975,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -855,7 +988,6 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -881,7 +1013,6 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -898,8 +1029,8 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -919,9 +1050,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -933,7 +1061,6 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -952,10 +1079,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1205,7 +1328,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -1234,11 +1356,21 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1247,6 +1379,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFD6DCE4"/>
       <color rgb="FFF2F2F2"/>
       <color rgb="FF37343E"/>
       <color rgb="FFFFE699"/>
@@ -1256,7 +1389,6 @@
       <color rgb="FFDDEBF7"/>
       <color rgb="FFFFFFCC"/>
       <color rgb="FFFF7373"/>
-      <color rgb="FFFF9999"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1295,7 +1427,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6592"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6856"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1410,7 +1542,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6593"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6857"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1470,7 +1602,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6594"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6858"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1530,7 +1662,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6595"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6859"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1590,7 +1722,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6596"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6860"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1650,7 +1782,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6597"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6861"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1710,7 +1842,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6598"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6862"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1770,7 +1902,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6599"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6863"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1830,7 +1962,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6600"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6864"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1895,7 +2027,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6601"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6865"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1960,7 +2092,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6602"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6866"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2025,7 +2157,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6603"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6867"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2090,7 +2222,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6604"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6868"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2155,7 +2287,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6605"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6869"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2220,7 +2352,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6606"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6870"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2285,7 +2417,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6607"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6871"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2350,7 +2482,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$K$1" spid="_x0000_s6608"/>
+                  <a14:cameraTool cellRange="Src!$J$1" spid="_x0000_s6872"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2415,7 +2547,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$K$1" spid="_x0000_s6609"/>
+                  <a14:cameraTool cellRange="Src!$J$1" spid="_x0000_s6873"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2480,7 +2612,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$L$1" spid="_x0000_s6610"/>
+                  <a14:cameraTool cellRange="Src!$K$1" spid="_x0000_s6874"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2545,7 +2677,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$I$1" spid="_x0000_s6611"/>
+                  <a14:cameraTool cellRange="Src!$H$1" spid="_x0000_s6875"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2610,7 +2742,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$J$1" spid="_x0000_s6612"/>
+                  <a14:cameraTool cellRange="Src!$I$1" spid="_x0000_s6876"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2675,7 +2807,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$M$1" spid="_x0000_s6613"/>
+                  <a14:cameraTool cellRange="Src!$L$1" spid="_x0000_s6877"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2740,7 +2872,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$N$1" spid="_x0000_s6614"/>
+                  <a14:cameraTool cellRange="Src!$M$1" spid="_x0000_s6878"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2805,7 +2937,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$N$1" spid="_x0000_s6615"/>
+                  <a14:cameraTool cellRange="Src!$M$1" spid="_x0000_s6879"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -13915,10 +14047,82 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="11">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="27">
   <rv s="0">
     <v>0</v>
     <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>8</v>
+    <v>4</v>
+  </rv>
+  <rv s="0">
+    <v>9</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>10</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>11</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>12</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>13</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>14</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>15</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>16</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>17</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
   </rv>
   <rv s="0">
     <v>1</v>
@@ -13952,14 +14156,6 @@
     <v>8</v>
     <v>5</v>
   </rv>
-  <rv s="0">
-    <v>9</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
 </rvData>
 </file>
 
@@ -13984,6 +14180,14 @@
   <rel r:id="rId8"/>
   <rel r:id="rId9"/>
   <rel r:id="rId10"/>
+  <rel r:id="rId11"/>
+  <rel r:id="rId12"/>
+  <rel r:id="rId13"/>
+  <rel r:id="rId14"/>
+  <rel r:id="rId15"/>
+  <rel r:id="rId16"/>
+  <rel r:id="rId17"/>
+  <rel r:id="rId18"/>
 </richValueRels>
 </file>
 
@@ -14280,150 +14484,150 @@
   <sheetData>
     <row r="1" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="78"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="80"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="92"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="92"/>
-      <c r="L2" s="93"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="75"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="86"/>
+      <c r="J2" s="86"/>
+      <c r="K2" s="86"/>
+      <c r="L2" s="87"/>
       <c r="N2" s="16"/>
       <c r="O2" s="17"/>
       <c r="P2" s="17"/>
       <c r="Q2" s="17"/>
-      <c r="R2" s="104"/>
+      <c r="R2" s="97"/>
       <c r="T2" s="23"/>
       <c r="U2" s="24"/>
       <c r="V2" s="24"/>
       <c r="W2" s="24"/>
-      <c r="X2" s="67"/>
+      <c r="X2" s="63"/>
     </row>
     <row r="3" spans="2:24" s="58" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="81"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82" t="str">
+      <c r="B3" s="76"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77" t="str">
         <f>Src!$A5</f>
         <v>FIREBALL</v>
       </c>
-      <c r="E3" s="82"/>
-      <c r="F3" s="83"/>
-      <c r="H3" s="94"/>
-      <c r="I3" s="95"/>
-      <c r="J3" s="134" t="str">
+      <c r="E3" s="77"/>
+      <c r="F3" s="78"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="123" t="str">
         <f>Src!A6</f>
         <v>FROST NOVA</v>
       </c>
-      <c r="K3" s="95"/>
-      <c r="L3" s="96"/>
-      <c r="N3" s="105"/>
-      <c r="O3" s="106"/>
-      <c r="P3" s="107" t="str">
+      <c r="K3" s="89"/>
+      <c r="L3" s="90"/>
+      <c r="N3" s="98"/>
+      <c r="O3" s="99"/>
+      <c r="P3" s="100" t="str">
         <f>Src!A7</f>
         <v>TIDAL WAVE</v>
       </c>
-      <c r="Q3" s="106"/>
-      <c r="R3" s="108"/>
-      <c r="T3" s="68"/>
-      <c r="U3" s="69"/>
-      <c r="V3" s="76" t="str">
+      <c r="Q3" s="99"/>
+      <c r="R3" s="101"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="71" t="str">
         <f>Src!A8</f>
         <v>BRAMBLE SNARE</v>
       </c>
-      <c r="W3" s="69"/>
-      <c r="X3" s="70"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="66"/>
     </row>
     <row r="4" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="84"/>
-      <c r="C4" s="170" t="e" vm="1">
-        <f>Src!F5</f>
+      <c r="B4" s="79"/>
+      <c r="C4" s="155" t="e" vm="1">
+        <f>Src!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="170"/>
-      <c r="E4" s="170"/>
-      <c r="F4" s="85"/>
-      <c r="H4" s="97"/>
-      <c r="I4" s="98"/>
-      <c r="J4" s="114">
-        <f>Src!F6</f>
-        <v>0</v>
+      <c r="D4" s="155"/>
+      <c r="E4" s="155"/>
+      <c r="F4" s="80"/>
+      <c r="H4" s="91"/>
+      <c r="I4" s="243" t="e" vm="2">
+        <f>Src!E6</f>
+        <v>#VALUE!</v>
       </c>
-      <c r="K4" s="98"/>
-      <c r="L4" s="99"/>
-      <c r="N4" s="246"/>
-      <c r="O4" s="109"/>
-      <c r="P4" s="65">
-        <f>Src!F7</f>
-        <v>0</v>
+      <c r="J4" s="243"/>
+      <c r="K4" s="243"/>
+      <c r="L4" s="92"/>
+      <c r="N4" s="231"/>
+      <c r="O4" s="179" t="e" vm="3">
+        <f>Src!E7</f>
+        <v>#VALUE!</v>
       </c>
-      <c r="Q4" s="109"/>
-      <c r="R4" s="110"/>
+      <c r="P4" s="179"/>
+      <c r="Q4" s="179"/>
+      <c r="R4" s="102"/>
       <c r="T4" s="26"/>
-      <c r="U4" s="247"/>
-      <c r="V4" s="64">
-        <f xml:space="preserve"> Src!F8</f>
-        <v>0</v>
+      <c r="U4" s="193" t="e" vm="4">
+        <f xml:space="preserve"> Src!E8</f>
+        <v>#VALUE!</v>
       </c>
-      <c r="W4" s="71"/>
-      <c r="X4" s="72"/>
+      <c r="V4" s="193"/>
+      <c r="W4" s="193"/>
+      <c r="X4" s="67"/>
     </row>
     <row r="5" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="84"/>
-      <c r="C5" s="171" t="str">
+      <c r="B5" s="79"/>
+      <c r="C5" s="156" t="str">
         <f>Src!$C5</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="171"/>
-      <c r="E5" s="171"/>
-      <c r="F5" s="86"/>
-      <c r="H5" s="97"/>
-      <c r="I5" s="172" t="str">
+      <c r="D5" s="156"/>
+      <c r="E5" s="156"/>
+      <c r="F5" s="81"/>
+      <c r="H5" s="91"/>
+      <c r="I5" s="157" t="str">
         <f>Src!$C6</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="J5" s="172"/>
-      <c r="K5" s="172"/>
-      <c r="L5" s="100"/>
+      <c r="J5" s="157"/>
+      <c r="K5" s="157"/>
+      <c r="L5" s="93"/>
       <c r="N5" s="19"/>
-      <c r="O5" s="173" t="str">
+      <c r="O5" s="158" t="str">
         <f>Src!C7</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="P5" s="173"/>
-      <c r="Q5" s="173"/>
-      <c r="R5" s="111"/>
+      <c r="P5" s="158"/>
+      <c r="Q5" s="158"/>
+      <c r="R5" s="103"/>
       <c r="T5" s="26"/>
-      <c r="U5" s="174" t="str">
+      <c r="U5" s="159" t="str">
         <f>Src!C8</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="V5" s="174"/>
-      <c r="W5" s="174"/>
-      <c r="X5" s="73"/>
+      <c r="V5" s="159"/>
+      <c r="W5" s="159"/>
+      <c r="X5" s="68"/>
     </row>
     <row r="6" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="87"/>
-      <c r="C6" s="88"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="89"/>
-      <c r="H6" s="101"/>
-      <c r="I6" s="102"/>
-      <c r="J6" s="102"/>
-      <c r="K6" s="102"/>
-      <c r="L6" s="103"/>
+      <c r="B6" s="82"/>
+      <c r="C6" s="83"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="84"/>
+      <c r="H6" s="94"/>
+      <c r="I6" s="95"/>
+      <c r="J6" s="95"/>
+      <c r="K6" s="95"/>
+      <c r="L6" s="96"/>
       <c r="N6" s="21"/>
-      <c r="O6" s="112"/>
-      <c r="P6" s="112"/>
-      <c r="Q6" s="112"/>
-      <c r="R6" s="113"/>
+      <c r="O6" s="104"/>
+      <c r="P6" s="104"/>
+      <c r="Q6" s="104"/>
+      <c r="R6" s="105"/>
       <c r="T6" s="28"/>
-      <c r="U6" s="74"/>
-      <c r="V6" s="74"/>
-      <c r="W6" s="74"/>
-      <c r="X6" s="75"/>
+      <c r="U6" s="69"/>
+      <c r="V6" s="69"/>
+      <c r="W6" s="69"/>
+      <c r="X6" s="70"/>
     </row>
     <row r="7" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -14431,146 +14635,146 @@
       <c r="C8" s="38"/>
       <c r="D8" s="38"/>
       <c r="E8" s="38"/>
-      <c r="F8" s="248"/>
+      <c r="F8" s="232"/>
       <c r="H8" s="44"/>
       <c r="I8" s="45"/>
       <c r="J8" s="45"/>
       <c r="K8" s="45"/>
-      <c r="L8" s="115"/>
+      <c r="L8" s="106"/>
       <c r="N8" s="51"/>
       <c r="O8" s="52"/>
       <c r="P8" s="52"/>
       <c r="Q8" s="52"/>
-      <c r="R8" s="124"/>
+      <c r="R8" s="114"/>
       <c r="T8" s="37"/>
       <c r="U8" s="38"/>
       <c r="V8" s="38"/>
       <c r="W8" s="38"/>
-      <c r="X8" s="248"/>
+      <c r="X8" s="232"/>
     </row>
     <row r="9" spans="2:24" s="58" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="249"/>
-      <c r="C9" s="250"/>
-      <c r="D9" s="251" t="str">
+      <c r="B9" s="233"/>
+      <c r="C9" s="234"/>
+      <c r="D9" s="235" t="str">
         <f>Src!$A9</f>
         <v>LIGHTNING BOLT</v>
       </c>
-      <c r="E9" s="250"/>
-      <c r="F9" s="252"/>
-      <c r="H9" s="116"/>
-      <c r="I9" s="117"/>
-      <c r="J9" s="135" t="str">
+      <c r="E9" s="234"/>
+      <c r="F9" s="236"/>
+      <c r="H9" s="107"/>
+      <c r="I9" s="108"/>
+      <c r="J9" s="124" t="str">
         <f>Src!A10</f>
         <v>BLACK HOLE</v>
       </c>
-      <c r="K9" s="117"/>
-      <c r="L9" s="118"/>
-      <c r="N9" s="125"/>
-      <c r="O9" s="126"/>
-      <c r="P9" s="127" t="str">
+      <c r="K9" s="108"/>
+      <c r="L9" s="109"/>
+      <c r="N9" s="115"/>
+      <c r="O9" s="116"/>
+      <c r="P9" s="117" t="str">
         <f>Src!A11</f>
         <v>ASTRAL DAGGER</v>
       </c>
-      <c r="Q9" s="126"/>
-      <c r="R9" s="128"/>
-      <c r="T9" s="249"/>
-      <c r="U9" s="250"/>
-      <c r="V9" s="251" t="str">
+      <c r="Q9" s="116"/>
+      <c r="R9" s="118"/>
+      <c r="T9" s="233"/>
+      <c r="U9" s="234"/>
+      <c r="V9" s="235" t="str">
         <f>Src!A12</f>
         <v>CHAIN LIGHTNING</v>
       </c>
-      <c r="W9" s="250"/>
-      <c r="X9" s="252"/>
+      <c r="W9" s="234"/>
+      <c r="X9" s="236"/>
     </row>
     <row r="10" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="40"/>
-      <c r="C10" s="218">
-        <f>Src!F9</f>
-        <v>0</v>
+      <c r="C10" s="203" t="e" vm="5">
+        <f>Src!E9</f>
+        <v>#VALUE!</v>
       </c>
-      <c r="D10" s="218"/>
-      <c r="E10" s="218"/>
-      <c r="F10" s="259"/>
+      <c r="D10" s="203"/>
+      <c r="E10" s="203"/>
+      <c r="F10" s="242"/>
       <c r="H10" s="47"/>
-      <c r="I10" s="119"/>
-      <c r="J10" s="63">
-        <f>Src!F10</f>
-        <v>0</v>
+      <c r="I10" s="211" t="e" vm="6">
+        <f>Src!E10</f>
+        <v>#VALUE!</v>
       </c>
-      <c r="K10" s="119"/>
-      <c r="L10" s="120"/>
+      <c r="J10" s="211"/>
+      <c r="K10" s="211"/>
+      <c r="L10" s="110"/>
       <c r="N10" s="54"/>
-      <c r="O10" s="260"/>
-      <c r="P10" s="62">
-        <f>Src!F11</f>
-        <v>0</v>
+      <c r="O10" s="162" t="e" vm="7">
+        <f>Src!E11</f>
+        <v>#VALUE!</v>
       </c>
-      <c r="Q10" s="129"/>
-      <c r="R10" s="130"/>
+      <c r="P10" s="162"/>
+      <c r="Q10" s="162"/>
+      <c r="R10" s="119"/>
       <c r="T10" s="40"/>
-      <c r="U10" s="258"/>
-      <c r="V10" s="136">
-        <f>Src!F12</f>
-        <v>0</v>
+      <c r="U10" s="203" t="e" vm="8">
+        <f>Src!E12</f>
+        <v>#VALUE!</v>
       </c>
-      <c r="W10" s="258"/>
-      <c r="X10" s="253"/>
+      <c r="V10" s="203"/>
+      <c r="W10" s="203"/>
+      <c r="X10" s="237"/>
     </row>
     <row r="11" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="40"/>
-      <c r="C11" s="254" t="str">
+      <c r="C11" s="238" t="str">
         <f>Src!$C9</f>
         <v>Casts a bolt of lightning</v>
       </c>
-      <c r="D11" s="254"/>
-      <c r="E11" s="254"/>
-      <c r="F11" s="255"/>
+      <c r="D11" s="238"/>
+      <c r="E11" s="238"/>
+      <c r="F11" s="239"/>
       <c r="H11" s="47"/>
-      <c r="I11" s="175" t="str">
+      <c r="I11" s="160" t="str">
         <f>Src!$C10</f>
         <v>Vacuums in nearby enemies</v>
       </c>
-      <c r="J11" s="175"/>
-      <c r="K11" s="175"/>
-      <c r="L11" s="121"/>
+      <c r="J11" s="160"/>
+      <c r="K11" s="160"/>
+      <c r="L11" s="111"/>
       <c r="N11" s="54"/>
-      <c r="O11" s="176" t="str">
+      <c r="O11" s="161" t="str">
         <f>Src!C11</f>
         <v>Flies to the nearest enemy in vision</v>
       </c>
-      <c r="P11" s="176"/>
-      <c r="Q11" s="176"/>
-      <c r="R11" s="131"/>
+      <c r="P11" s="161"/>
+      <c r="Q11" s="161"/>
+      <c r="R11" s="120"/>
       <c r="T11" s="40"/>
-      <c r="U11" s="254" t="str">
+      <c r="U11" s="238" t="str">
         <f>Src!C12</f>
         <v>Casts a tracking bolt of lightning that can chain to close enemies</v>
       </c>
-      <c r="V11" s="254"/>
-      <c r="W11" s="254"/>
-      <c r="X11" s="255"/>
+      <c r="V11" s="238"/>
+      <c r="W11" s="238"/>
+      <c r="X11" s="239"/>
     </row>
     <row r="12" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="42"/>
-      <c r="C12" s="256"/>
-      <c r="D12" s="256"/>
-      <c r="E12" s="256"/>
-      <c r="F12" s="257"/>
+      <c r="C12" s="240"/>
+      <c r="D12" s="240"/>
+      <c r="E12" s="240"/>
+      <c r="F12" s="241"/>
       <c r="H12" s="49"/>
-      <c r="I12" s="122"/>
-      <c r="J12" s="122"/>
-      <c r="K12" s="122"/>
-      <c r="L12" s="123"/>
+      <c r="I12" s="112"/>
+      <c r="J12" s="112"/>
+      <c r="K12" s="112"/>
+      <c r="L12" s="113"/>
       <c r="N12" s="56"/>
-      <c r="O12" s="132"/>
-      <c r="P12" s="132"/>
-      <c r="Q12" s="132"/>
-      <c r="R12" s="133"/>
+      <c r="O12" s="121"/>
+      <c r="P12" s="121"/>
+      <c r="Q12" s="121"/>
+      <c r="R12" s="122"/>
       <c r="T12" s="42"/>
-      <c r="U12" s="256"/>
-      <c r="V12" s="256"/>
-      <c r="W12" s="256"/>
-      <c r="X12" s="257"/>
+      <c r="U12" s="240"/>
+      <c r="V12" s="240"/>
+      <c r="W12" s="240"/>
+      <c r="X12" s="241"/>
     </row>
     <row r="13" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -14578,468 +14782,483 @@
       <c r="C14" s="52"/>
       <c r="D14" s="52"/>
       <c r="E14" s="52"/>
-      <c r="F14" s="124"/>
-      <c r="H14" s="152"/>
-      <c r="I14" s="153"/>
-      <c r="J14" s="153"/>
-      <c r="K14" s="153"/>
-      <c r="L14" s="154"/>
-      <c r="N14" s="152"/>
-      <c r="O14" s="153"/>
-      <c r="P14" s="153"/>
-      <c r="Q14" s="153"/>
-      <c r="R14" s="154"/>
-      <c r="T14" s="152"/>
-      <c r="U14" s="153"/>
-      <c r="V14" s="153"/>
-      <c r="W14" s="153"/>
-      <c r="X14" s="154"/>
+      <c r="F14" s="114"/>
+      <c r="H14" s="139"/>
+      <c r="I14" s="140"/>
+      <c r="J14" s="140"/>
+      <c r="K14" s="140"/>
+      <c r="L14" s="141"/>
+      <c r="N14" s="139"/>
+      <c r="O14" s="140"/>
+      <c r="P14" s="140"/>
+      <c r="Q14" s="140"/>
+      <c r="R14" s="141"/>
+      <c r="T14" s="139"/>
+      <c r="U14" s="140"/>
+      <c r="V14" s="140"/>
+      <c r="W14" s="140"/>
+      <c r="X14" s="141"/>
     </row>
     <row r="15" spans="2:24" s="58" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="125"/>
-      <c r="C15" s="126"/>
-      <c r="D15" s="127" t="str">
+      <c r="B15" s="115"/>
+      <c r="C15" s="116"/>
+      <c r="D15" s="117" t="str">
         <f>Src!$A13</f>
         <v>DIVINE JUDGEMENT</v>
       </c>
-      <c r="E15" s="126"/>
-      <c r="F15" s="128"/>
-      <c r="H15" s="155"/>
-      <c r="I15" s="156"/>
-      <c r="J15" s="157" t="str">
+      <c r="E15" s="116"/>
+      <c r="F15" s="118"/>
+      <c r="H15" s="142"/>
+      <c r="I15" s="143"/>
+      <c r="J15" s="144" t="str">
         <f>Src!A14</f>
-        <v>Haste</v>
+        <v>HASTE</v>
       </c>
-      <c r="K15" s="156"/>
-      <c r="L15" s="158"/>
-      <c r="N15" s="155"/>
-      <c r="O15" s="156"/>
-      <c r="P15" s="157" t="str">
+      <c r="K15" s="143"/>
+      <c r="L15" s="145"/>
+      <c r="N15" s="142"/>
+      <c r="O15" s="143"/>
+      <c r="P15" s="144" t="str">
         <f>Src!A15</f>
         <v>HINDER</v>
       </c>
-      <c r="Q15" s="156"/>
-      <c r="R15" s="158"/>
-      <c r="T15" s="155"/>
-      <c r="U15" s="156"/>
-      <c r="V15" s="168" t="str">
+      <c r="Q15" s="143"/>
+      <c r="R15" s="145"/>
+      <c r="T15" s="142"/>
+      <c r="U15" s="143"/>
+      <c r="V15" s="153" t="str">
         <f>Src!A16</f>
         <v>MULLIGAN</v>
       </c>
-      <c r="W15" s="156"/>
-      <c r="X15" s="158"/>
+      <c r="W15" s="143"/>
+      <c r="X15" s="145"/>
     </row>
     <row r="16" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="54"/>
-      <c r="C16" s="177">
-        <f>Src!F13</f>
+      <c r="C16" s="162" t="e" vm="9">
+        <f>Src!E13</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D16" s="162"/>
+      <c r="E16" s="162"/>
+      <c r="F16" s="119"/>
+      <c r="H16" s="146"/>
+      <c r="I16" s="246">
+        <f>Src!E14</f>
         <v>0</v>
       </c>
-      <c r="D16" s="177"/>
-      <c r="E16" s="177"/>
-      <c r="F16" s="130"/>
-      <c r="H16" s="159"/>
-      <c r="I16" s="160"/>
-      <c r="J16" s="161">
-        <f>Src!F14</f>
+      <c r="J16" s="246"/>
+      <c r="K16" s="246"/>
+      <c r="L16" s="147"/>
+      <c r="N16" s="146"/>
+      <c r="O16" s="164">
+        <f>Src!E15</f>
         <v>0</v>
       </c>
-      <c r="K16" s="160"/>
-      <c r="L16" s="162"/>
-      <c r="N16" s="159"/>
-      <c r="O16" s="160"/>
-      <c r="P16" s="161">
-        <f>Src!F15</f>
+      <c r="P16" s="164"/>
+      <c r="Q16" s="164"/>
+      <c r="R16" s="147"/>
+      <c r="T16" s="146"/>
+      <c r="U16" s="164">
+        <f xml:space="preserve"> Src!E16</f>
         <v>0</v>
       </c>
-      <c r="Q16" s="160"/>
-      <c r="R16" s="162"/>
-      <c r="T16" s="159"/>
-      <c r="U16" s="160"/>
-      <c r="V16" s="161">
-        <f xml:space="preserve"> Src!F16</f>
-        <v>0</v>
-      </c>
-      <c r="W16" s="160"/>
-      <c r="X16" s="162"/>
+      <c r="V16" s="164"/>
+      <c r="W16" s="164"/>
+      <c r="X16" s="147"/>
     </row>
     <row r="17" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="54"/>
-      <c r="C17" s="176" t="str">
+      <c r="C17" s="161" t="str">
         <f>Src!$C13</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D17" s="176"/>
-      <c r="E17" s="176"/>
-      <c r="F17" s="131"/>
-      <c r="H17" s="159"/>
-      <c r="I17" s="178" t="str">
+      <c r="D17" s="161"/>
+      <c r="E17" s="161"/>
+      <c r="F17" s="120"/>
+      <c r="H17" s="146"/>
+      <c r="I17" s="163" t="str">
         <f>Src!$C14</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="J17" s="178"/>
-      <c r="K17" s="178"/>
-      <c r="L17" s="164"/>
-      <c r="N17" s="159"/>
-      <c r="O17" s="178" t="str">
+      <c r="J17" s="163"/>
+      <c r="K17" s="163"/>
+      <c r="L17" s="149"/>
+      <c r="N17" s="146"/>
+      <c r="O17" s="163" t="str">
         <f>Src!C15</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="P17" s="178"/>
-      <c r="Q17" s="178"/>
-      <c r="R17" s="164"/>
-      <c r="T17" s="159"/>
-      <c r="U17" s="178" t="str">
+      <c r="P17" s="163"/>
+      <c r="Q17" s="163"/>
+      <c r="R17" s="149"/>
+      <c r="T17" s="146"/>
+      <c r="U17" s="163" t="str">
         <f>Src!C16</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="V17" s="178"/>
-      <c r="W17" s="178"/>
-      <c r="X17" s="164"/>
+      <c r="V17" s="163"/>
+      <c r="W17" s="163"/>
+      <c r="X17" s="149"/>
     </row>
     <row r="18" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="56"/>
-      <c r="C18" s="132"/>
-      <c r="D18" s="132"/>
-      <c r="E18" s="132"/>
-      <c r="F18" s="133"/>
-      <c r="H18" s="165"/>
-      <c r="I18" s="166"/>
-      <c r="J18" s="166"/>
-      <c r="K18" s="166"/>
-      <c r="L18" s="167"/>
-      <c r="N18" s="165"/>
-      <c r="O18" s="166"/>
-      <c r="P18" s="166"/>
-      <c r="Q18" s="166"/>
-      <c r="R18" s="167"/>
-      <c r="T18" s="165"/>
-      <c r="U18" s="166"/>
-      <c r="V18" s="166"/>
-      <c r="W18" s="166"/>
-      <c r="X18" s="167"/>
+      <c r="C18" s="121"/>
+      <c r="D18" s="121"/>
+      <c r="E18" s="121"/>
+      <c r="F18" s="122"/>
+      <c r="H18" s="150"/>
+      <c r="I18" s="151"/>
+      <c r="J18" s="151"/>
+      <c r="K18" s="151"/>
+      <c r="L18" s="152"/>
+      <c r="N18" s="150"/>
+      <c r="O18" s="151"/>
+      <c r="P18" s="151"/>
+      <c r="Q18" s="151"/>
+      <c r="R18" s="152"/>
+      <c r="T18" s="150"/>
+      <c r="U18" s="151"/>
+      <c r="V18" s="151"/>
+      <c r="W18" s="151"/>
+      <c r="X18" s="152"/>
     </row>
     <row r="19" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="20" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="152"/>
-      <c r="C20" s="153"/>
-      <c r="D20" s="153"/>
-      <c r="E20" s="153"/>
-      <c r="F20" s="154"/>
-      <c r="H20" s="152"/>
-      <c r="I20" s="153"/>
-      <c r="J20" s="153"/>
-      <c r="K20" s="153"/>
-      <c r="L20" s="154"/>
-      <c r="N20" s="152"/>
-      <c r="O20" s="153"/>
-      <c r="P20" s="153"/>
-      <c r="Q20" s="153"/>
-      <c r="R20" s="154"/>
-      <c r="T20" s="152"/>
-      <c r="U20" s="153"/>
-      <c r="V20" s="153"/>
-      <c r="W20" s="153"/>
-      <c r="X20" s="154"/>
+      <c r="B20" s="139"/>
+      <c r="C20" s="140"/>
+      <c r="D20" s="140"/>
+      <c r="E20" s="140"/>
+      <c r="F20" s="141"/>
+      <c r="H20" s="139"/>
+      <c r="I20" s="140"/>
+      <c r="J20" s="140"/>
+      <c r="K20" s="140"/>
+      <c r="L20" s="141"/>
+      <c r="N20" s="139"/>
+      <c r="O20" s="140"/>
+      <c r="P20" s="140"/>
+      <c r="Q20" s="140"/>
+      <c r="R20" s="141"/>
+      <c r="T20" s="139"/>
+      <c r="U20" s="140"/>
+      <c r="V20" s="140"/>
+      <c r="W20" s="140"/>
+      <c r="X20" s="141"/>
     </row>
     <row r="21" spans="2:24" s="58" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="155"/>
-      <c r="C21" s="156"/>
-      <c r="D21" s="163" t="str">
+      <c r="B21" s="142"/>
+      <c r="C21" s="143"/>
+      <c r="D21" s="148" t="str">
         <f>Src!$A17</f>
         <v>BUT WAIT, THERE'S MORE</v>
       </c>
-      <c r="E21" s="156"/>
-      <c r="F21" s="158"/>
-      <c r="H21" s="155"/>
-      <c r="I21" s="156"/>
-      <c r="J21" s="169" t="str">
+      <c r="E21" s="143"/>
+      <c r="F21" s="145"/>
+      <c r="H21" s="142"/>
+      <c r="I21" s="143"/>
+      <c r="J21" s="154" t="str">
         <f>Src!A18</f>
         <v>MANA SHIELD</v>
       </c>
-      <c r="K21" s="156"/>
-      <c r="L21" s="158"/>
-      <c r="N21" s="155"/>
-      <c r="O21" s="156"/>
-      <c r="P21" s="169" t="str">
+      <c r="K21" s="143"/>
+      <c r="L21" s="145"/>
+      <c r="N21" s="142"/>
+      <c r="O21" s="143"/>
+      <c r="P21" s="154" t="str">
         <f>Src!A19</f>
         <v>RUNAWAY BULL</v>
       </c>
-      <c r="Q21" s="156"/>
-      <c r="R21" s="158"/>
-      <c r="T21" s="155"/>
-      <c r="U21" s="156"/>
-      <c r="V21" s="169" t="str">
+      <c r="Q21" s="143"/>
+      <c r="R21" s="145"/>
+      <c r="T21" s="142"/>
+      <c r="U21" s="143"/>
+      <c r="V21" s="154" t="str">
         <f>Src!A20</f>
         <v>HOLY BLADE</v>
       </c>
-      <c r="W21" s="156"/>
-      <c r="X21" s="158"/>
+      <c r="W21" s="143"/>
+      <c r="X21" s="145"/>
     </row>
     <row r="22" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="159"/>
-      <c r="C22" s="179">
-        <f>Src!F17</f>
+      <c r="B22" s="146"/>
+      <c r="C22" s="164">
+        <f>Src!E17</f>
         <v>0</v>
       </c>
-      <c r="D22" s="179"/>
-      <c r="E22" s="179"/>
-      <c r="F22" s="162"/>
-      <c r="H22" s="159"/>
-      <c r="I22" s="160"/>
-      <c r="J22" s="161">
-        <f>Src!F18</f>
+      <c r="D22" s="164"/>
+      <c r="E22" s="164"/>
+      <c r="F22" s="147"/>
+      <c r="H22" s="146"/>
+      <c r="I22" s="164">
+        <f>Src!E18</f>
         <v>0</v>
       </c>
-      <c r="K22" s="160"/>
-      <c r="L22" s="162"/>
-      <c r="N22" s="159"/>
-      <c r="O22" s="160"/>
-      <c r="P22" s="161">
-        <f>Src!F19</f>
+      <c r="J22" s="164"/>
+      <c r="K22" s="164"/>
+      <c r="L22" s="147"/>
+      <c r="N22" s="146"/>
+      <c r="O22" s="164">
+        <f>Src!E19</f>
         <v>0</v>
       </c>
-      <c r="Q22" s="160"/>
-      <c r="R22" s="162"/>
-      <c r="T22" s="159"/>
-      <c r="U22" s="160"/>
-      <c r="V22" s="161">
-        <f xml:space="preserve"> Src!F20</f>
+      <c r="P22" s="164"/>
+      <c r="Q22" s="164"/>
+      <c r="R22" s="147"/>
+      <c r="T22" s="146"/>
+      <c r="U22" s="164">
+        <f xml:space="preserve"> Src!E20</f>
         <v>0</v>
       </c>
-      <c r="W22" s="160"/>
-      <c r="X22" s="162"/>
+      <c r="V22" s="164"/>
+      <c r="W22" s="164"/>
+      <c r="X22" s="147"/>
     </row>
     <row r="23" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="159"/>
-      <c r="C23" s="178" t="str">
+      <c r="B23" s="146"/>
+      <c r="C23" s="163" t="str">
         <f>Src!$C17</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D23" s="178"/>
-      <c r="E23" s="178"/>
-      <c r="F23" s="164"/>
-      <c r="H23" s="159"/>
-      <c r="I23" s="178" t="str">
+      <c r="D23" s="163"/>
+      <c r="E23" s="163"/>
+      <c r="F23" s="149"/>
+      <c r="H23" s="146"/>
+      <c r="I23" s="163" t="str">
         <f>Src!$C18</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="J23" s="178"/>
-      <c r="K23" s="178"/>
-      <c r="L23" s="164"/>
-      <c r="N23" s="159"/>
-      <c r="O23" s="178" t="str">
+      <c r="J23" s="163"/>
+      <c r="K23" s="163"/>
+      <c r="L23" s="149"/>
+      <c r="N23" s="146"/>
+      <c r="O23" s="163" t="str">
         <f>Src!C19</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="P23" s="178"/>
-      <c r="Q23" s="178"/>
-      <c r="R23" s="164"/>
-      <c r="T23" s="159"/>
-      <c r="U23" s="178" t="str">
+      <c r="P23" s="163"/>
+      <c r="Q23" s="163"/>
+      <c r="R23" s="149"/>
+      <c r="T23" s="146"/>
+      <c r="U23" s="163" t="str">
         <f>Src!C20</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="V23" s="178"/>
-      <c r="W23" s="178"/>
-      <c r="X23" s="164"/>
+      <c r="V23" s="163"/>
+      <c r="W23" s="163"/>
+      <c r="X23" s="149"/>
     </row>
     <row r="24" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="165"/>
-      <c r="C24" s="166"/>
-      <c r="D24" s="166"/>
-      <c r="E24" s="166"/>
-      <c r="F24" s="167"/>
-      <c r="H24" s="165"/>
-      <c r="I24" s="166"/>
-      <c r="J24" s="166"/>
-      <c r="K24" s="166"/>
-      <c r="L24" s="167"/>
-      <c r="N24" s="165"/>
-      <c r="O24" s="166"/>
-      <c r="P24" s="166"/>
-      <c r="Q24" s="166"/>
-      <c r="R24" s="167"/>
-      <c r="T24" s="165"/>
-      <c r="U24" s="166"/>
-      <c r="V24" s="166"/>
-      <c r="W24" s="166"/>
-      <c r="X24" s="167"/>
+      <c r="B24" s="150"/>
+      <c r="C24" s="151"/>
+      <c r="D24" s="151"/>
+      <c r="E24" s="151"/>
+      <c r="F24" s="152"/>
+      <c r="H24" s="150"/>
+      <c r="I24" s="151"/>
+      <c r="J24" s="151"/>
+      <c r="K24" s="151"/>
+      <c r="L24" s="152"/>
+      <c r="N24" s="150"/>
+      <c r="O24" s="151"/>
+      <c r="P24" s="151"/>
+      <c r="Q24" s="151"/>
+      <c r="R24" s="152"/>
+      <c r="T24" s="150"/>
+      <c r="U24" s="151"/>
+      <c r="V24" s="151"/>
+      <c r="W24" s="151"/>
+      <c r="X24" s="152"/>
     </row>
     <row r="25" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="137"/>
-      <c r="C26" s="138"/>
-      <c r="D26" s="138"/>
-      <c r="E26" s="138"/>
-      <c r="F26" s="139"/>
-      <c r="H26" s="137"/>
-      <c r="I26" s="138"/>
-      <c r="J26" s="138"/>
-      <c r="K26" s="138"/>
-      <c r="L26" s="139"/>
-      <c r="N26" s="137"/>
-      <c r="O26" s="138"/>
-      <c r="P26" s="138"/>
-      <c r="Q26" s="138"/>
-      <c r="R26" s="139"/>
-      <c r="T26" s="137"/>
-      <c r="U26" s="138"/>
-      <c r="V26" s="138"/>
-      <c r="W26" s="138"/>
-      <c r="X26" s="139"/>
+      <c r="B26" s="126"/>
+      <c r="C26" s="127"/>
+      <c r="D26" s="127"/>
+      <c r="E26" s="127"/>
+      <c r="F26" s="128"/>
+      <c r="H26" s="126"/>
+      <c r="I26" s="127"/>
+      <c r="J26" s="127"/>
+      <c r="K26" s="127"/>
+      <c r="L26" s="128"/>
+      <c r="N26" s="126"/>
+      <c r="O26" s="127"/>
+      <c r="P26" s="127"/>
+      <c r="Q26" s="127"/>
+      <c r="R26" s="128"/>
+      <c r="T26" s="126"/>
+      <c r="U26" s="127"/>
+      <c r="V26" s="127"/>
+      <c r="W26" s="127"/>
+      <c r="X26" s="128"/>
     </row>
     <row r="27" spans="2:24" s="58" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="140"/>
-      <c r="C27" s="141"/>
-      <c r="D27" s="142">
+      <c r="B27" s="129"/>
+      <c r="C27" s="130"/>
+      <c r="D27" s="131">
         <f>Src!$A21</f>
         <v>0</v>
       </c>
-      <c r="E27" s="141"/>
-      <c r="F27" s="143"/>
-      <c r="H27" s="140"/>
-      <c r="I27" s="141"/>
-      <c r="J27" s="142">
+      <c r="E27" s="130"/>
+      <c r="F27" s="132"/>
+      <c r="H27" s="129"/>
+      <c r="I27" s="130"/>
+      <c r="J27" s="131">
         <f>Src!A22</f>
         <v>0</v>
       </c>
-      <c r="K27" s="141"/>
-      <c r="L27" s="143"/>
-      <c r="N27" s="140"/>
-      <c r="O27" s="141"/>
-      <c r="P27" s="142">
+      <c r="K27" s="130"/>
+      <c r="L27" s="132"/>
+      <c r="N27" s="129"/>
+      <c r="O27" s="130"/>
+      <c r="P27" s="131">
         <f>Src!A23</f>
         <v>0</v>
       </c>
-      <c r="Q27" s="141"/>
-      <c r="R27" s="143"/>
-      <c r="T27" s="140"/>
-      <c r="U27" s="141"/>
-      <c r="V27" s="142">
+      <c r="Q27" s="130"/>
+      <c r="R27" s="132"/>
+      <c r="T27" s="129"/>
+      <c r="U27" s="130"/>
+      <c r="V27" s="131">
         <f>Src!A24</f>
         <v>0</v>
       </c>
-      <c r="W27" s="141"/>
-      <c r="X27" s="143"/>
+      <c r="W27" s="130"/>
+      <c r="X27" s="132"/>
     </row>
     <row r="28" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="144"/>
-      <c r="C28" s="180">
-        <f>Src!F21</f>
+      <c r="B28" s="133"/>
+      <c r="C28" s="165">
+        <f>Src!E21</f>
         <v>0</v>
       </c>
-      <c r="D28" s="180"/>
-      <c r="E28" s="180"/>
-      <c r="F28" s="146"/>
-      <c r="H28" s="144"/>
-      <c r="I28" s="151"/>
-      <c r="J28" s="145">
-        <f>Src!F22</f>
+      <c r="D28" s="165"/>
+      <c r="E28" s="165"/>
+      <c r="F28" s="134"/>
+      <c r="H28" s="133"/>
+      <c r="I28" s="165">
+        <f>Src!E22</f>
         <v>0</v>
       </c>
-      <c r="K28" s="151"/>
-      <c r="L28" s="146"/>
-      <c r="N28" s="144"/>
-      <c r="O28" s="151"/>
-      <c r="P28" s="145">
-        <f>Src!F23</f>
+      <c r="J28" s="165"/>
+      <c r="K28" s="165"/>
+      <c r="L28" s="134"/>
+      <c r="N28" s="133"/>
+      <c r="O28" s="165">
+        <f>Src!E23</f>
         <v>0</v>
       </c>
-      <c r="Q28" s="151"/>
-      <c r="R28" s="146"/>
-      <c r="T28" s="144"/>
-      <c r="U28" s="151"/>
-      <c r="V28" s="145">
-        <f xml:space="preserve"> Src!F24</f>
+      <c r="P28" s="165"/>
+      <c r="Q28" s="165"/>
+      <c r="R28" s="134"/>
+      <c r="T28" s="133"/>
+      <c r="U28" s="165">
+        <f xml:space="preserve"> Src!E24</f>
         <v>0</v>
       </c>
-      <c r="W28" s="151"/>
-      <c r="X28" s="146"/>
+      <c r="V28" s="165"/>
+      <c r="W28" s="165"/>
+      <c r="X28" s="134"/>
     </row>
     <row r="29" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="144"/>
-      <c r="C29" s="181">
+      <c r="B29" s="133"/>
+      <c r="C29" s="166">
         <f>Src!$C21</f>
         <v>0</v>
       </c>
-      <c r="D29" s="181"/>
-      <c r="E29" s="181"/>
-      <c r="F29" s="147"/>
-      <c r="H29" s="144"/>
-      <c r="I29" s="181">
+      <c r="D29" s="166"/>
+      <c r="E29" s="166"/>
+      <c r="F29" s="135"/>
+      <c r="H29" s="133"/>
+      <c r="I29" s="166">
         <f>Src!$C22</f>
         <v>0</v>
       </c>
-      <c r="J29" s="181"/>
-      <c r="K29" s="181"/>
-      <c r="L29" s="147"/>
-      <c r="N29" s="144"/>
-      <c r="O29" s="181">
+      <c r="J29" s="166"/>
+      <c r="K29" s="166"/>
+      <c r="L29" s="135"/>
+      <c r="N29" s="133"/>
+      <c r="O29" s="166">
         <f>Src!C23</f>
         <v>0</v>
       </c>
-      <c r="P29" s="181"/>
-      <c r="Q29" s="181"/>
-      <c r="R29" s="147"/>
-      <c r="T29" s="144"/>
-      <c r="U29" s="181">
+      <c r="P29" s="166"/>
+      <c r="Q29" s="166"/>
+      <c r="R29" s="135"/>
+      <c r="T29" s="133"/>
+      <c r="U29" s="166">
         <f>Src!C24</f>
         <v>0</v>
       </c>
-      <c r="V29" s="181"/>
-      <c r="W29" s="181"/>
-      <c r="X29" s="147"/>
+      <c r="V29" s="166"/>
+      <c r="W29" s="166"/>
+      <c r="X29" s="135"/>
     </row>
     <row r="30" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="148"/>
-      <c r="C30" s="149"/>
-      <c r="D30" s="149"/>
-      <c r="E30" s="149"/>
-      <c r="F30" s="150"/>
-      <c r="H30" s="148"/>
-      <c r="I30" s="149"/>
-      <c r="J30" s="149"/>
-      <c r="K30" s="149"/>
-      <c r="L30" s="150"/>
-      <c r="N30" s="148"/>
-      <c r="O30" s="149"/>
-      <c r="P30" s="149"/>
-      <c r="Q30" s="149"/>
-      <c r="R30" s="150"/>
-      <c r="T30" s="148"/>
-      <c r="U30" s="149"/>
-      <c r="V30" s="149"/>
-      <c r="W30" s="149"/>
-      <c r="X30" s="150"/>
+      <c r="B30" s="136"/>
+      <c r="C30" s="137"/>
+      <c r="D30" s="137"/>
+      <c r="E30" s="137"/>
+      <c r="F30" s="138"/>
+      <c r="H30" s="136"/>
+      <c r="I30" s="137"/>
+      <c r="J30" s="137"/>
+      <c r="K30" s="137"/>
+      <c r="L30" s="138"/>
+      <c r="N30" s="136"/>
+      <c r="O30" s="137"/>
+      <c r="P30" s="137"/>
+      <c r="Q30" s="137"/>
+      <c r="R30" s="138"/>
+      <c r="T30" s="136"/>
+      <c r="U30" s="137"/>
+      <c r="V30" s="137"/>
+      <c r="W30" s="137"/>
+      <c r="X30" s="138"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="40">
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="C29:E29"/>
     <mergeCell ref="I29:K29"/>
     <mergeCell ref="O29:Q29"/>
     <mergeCell ref="U29:W29"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="O28:Q28"/>
+    <mergeCell ref="U28:W28"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="I23:K23"/>
     <mergeCell ref="O23:Q23"/>
     <mergeCell ref="U23:W23"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="U22:W22"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="I17:K17"/>
     <mergeCell ref="O17:Q17"/>
     <mergeCell ref="U17:W17"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="U16:W16"/>
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="I11:K11"/>
     <mergeCell ref="O11:Q11"/>
     <mergeCell ref="U11:W11"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="U10:W10"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="I5:K5"/>
     <mergeCell ref="O5:Q5"/>
     <mergeCell ref="U5:W5"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="U4:W4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -15053,57 +15272,58 @@
   <sheetPr>
     <tabColor theme="4" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.42578125" customWidth="1"/>
     <col min="3" max="3" width="55.42578125" customWidth="1"/>
-    <col min="5" max="5" width="55.42578125" customWidth="1"/>
-    <col min="6" max="6" width="47.42578125" customWidth="1"/>
-    <col min="8" max="14" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="125"/>
+    <col min="5" max="5" width="47.42578125" customWidth="1"/>
+    <col min="7" max="13" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="58" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="G1" s="58" t="s">
-        <v>19</v>
+      <c r="F1" s="58" t="s">
+        <v>49</v>
       </c>
-      <c r="H1" t="e" vm="2">
+      <c r="G1" t="e" vm="10">
         <v>#VALUE!</v>
       </c>
-      <c r="I1" t="e" vm="3">
+      <c r="H1" t="e" vm="11">
         <v>#VALUE!</v>
       </c>
-      <c r="J1" t="e" vm="4">
+      <c r="I1" t="e" vm="12">
         <v>#VALUE!</v>
       </c>
-      <c r="K1" t="e" vm="5">
+      <c r="J1" t="e" vm="13">
         <v>#VALUE!</v>
       </c>
-      <c r="L1" t="e" vm="6">
+      <c r="K1" t="e" vm="14">
         <v>#VALUE!</v>
       </c>
-      <c r="M1" t="e" vm="7">
+      <c r="L1" t="e" vm="15">
         <v>#VALUE!</v>
       </c>
-      <c r="N1" t="e" vm="8">
+      <c r="M1" t="e" vm="16">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="e" vm="9">
+    <row r="2" spans="1:13" ht="393" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="e" vm="17">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" t="e" vm="10">
+      <c r="C2" t="e" vm="18">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="3" spans="1:14" s="59" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:14" s="61" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" s="59" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D3" s="244"/>
+    </row>
+    <row r="4" spans="1:13" s="61" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="60" t="s">
         <v>2</v>
       </c>
@@ -15113,278 +15333,305 @@
       <c r="C4" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="60" t="s">
+      <c r="D4" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60" t="s">
+      <c r="E4" s="245" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:14" s="61" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" s="61" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="60" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="77" t="s">
-        <v>21</v>
+      <c r="C5" s="72" t="s">
+        <v>20</v>
       </c>
-      <c r="D5" s="90" t="s">
+      <c r="D5" s="245" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="60"/>
-      <c r="F5" s="61" t="e" vm="11">
+      <c r="E5" s="61" t="e" vm="19">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="6" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="77" t="s">
-        <v>20</v>
+    <row r="6" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="72" t="s">
+        <v>19</v>
       </c>
-      <c r="B6" s="77" t="s">
+      <c r="B6" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="77" t="s">
+      <c r="C6" s="72" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="245" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="90" t="s">
+      <c r="E6" s="72" t="e" vm="20">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="72" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="72" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="72" t="s">
         <v>23</v>
       </c>
+      <c r="D7" s="245" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="72" t="e" vm="21">
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="7" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="77" t="s">
-        <v>14</v>
+    <row r="8" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="72" t="s">
+        <v>15</v>
       </c>
-      <c r="B7" s="77" t="s">
+      <c r="B8" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="77" t="s">
+      <c r="C8" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="245" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="72" t="e" vm="22">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="72" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="72" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="72" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="245" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="72" t="e" vm="23">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="72" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="72" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="245" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="72" t="e" vm="24">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="72" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="72" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="90" t="s">
-        <v>9</v>
+      <c r="D11" s="245" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="72" t="e" vm="25">
+        <v>#VALUE!</v>
       </c>
     </row>
-    <row r="8" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="77" t="s">
-        <v>15</v>
+    <row r="12" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="72" t="s">
+        <v>27</v>
       </c>
-      <c r="B8" s="77" t="s">
+      <c r="B12" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="77" t="s">
-        <v>26</v>
+      <c r="C12" s="72" t="s">
+        <v>31</v>
       </c>
-      <c r="D8" s="90" t="s">
-        <v>10</v>
+      <c r="D12" s="245" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="72" t="e" vm="26">
+        <v>#VALUE!</v>
       </c>
     </row>
-    <row r="9" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="77" t="s">
-        <v>17</v>
+    <row r="13" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="72" t="s">
+        <v>28</v>
       </c>
-      <c r="B9" s="77" t="s">
+      <c r="B13" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="77" t="s">
-        <v>30</v>
+      <c r="C13" s="72" t="s">
+        <v>32</v>
       </c>
-      <c r="D9" s="90" t="s">
-        <v>8</v>
+      <c r="D13" s="245" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="72" t="e" vm="27">
+        <v>#VALUE!</v>
       </c>
     </row>
-    <row r="10" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="77" t="s">
-        <v>27</v>
+    <row r="14" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="72" t="s">
+        <v>48</v>
       </c>
-      <c r="B10" s="77" t="s">
-        <v>5</v>
+      <c r="B14" s="72" t="s">
+        <v>13</v>
       </c>
-      <c r="C10" s="77" t="s">
-        <v>31</v>
+      <c r="C14" s="72" t="s">
+        <v>39</v>
       </c>
-      <c r="D10" s="90" t="s">
-        <v>11</v>
+      <c r="D14" s="245" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="77" t="s">
-        <v>16</v>
+    <row r="15" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="72" t="s">
+        <v>33</v>
       </c>
-      <c r="B11" s="77" t="s">
-        <v>5</v>
+      <c r="B15" s="72" t="s">
+        <v>13</v>
       </c>
-      <c r="C11" s="77" t="s">
-        <v>25</v>
+      <c r="C15" s="72" t="s">
+        <v>40</v>
       </c>
-      <c r="D11" s="90" t="s">
-        <v>12</v>
+      <c r="D15" s="245" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="77" t="s">
-        <v>28</v>
+    <row r="16" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="72" t="s">
+        <v>34</v>
       </c>
-      <c r="B12" s="77" t="s">
-        <v>5</v>
+      <c r="B16" s="72" t="s">
+        <v>13</v>
       </c>
-      <c r="C12" s="77" t="s">
-        <v>32</v>
+      <c r="C16" s="72" t="s">
+        <v>41</v>
       </c>
-      <c r="D12" s="90" t="s">
-        <v>8</v>
+      <c r="D16" s="245" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="77" t="s">
-        <v>29</v>
+    <row r="17" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="72" t="s">
+        <v>35</v>
       </c>
-      <c r="B13" s="77" t="s">
-        <v>5</v>
+      <c r="B17" s="72" t="s">
+        <v>13</v>
       </c>
-      <c r="C13" s="77" t="s">
-        <v>33</v>
+      <c r="C17" s="72" t="s">
+        <v>42</v>
       </c>
-      <c r="D13" s="90" t="s">
-        <v>12</v>
+      <c r="D17" s="245" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="77" t="s">
-        <v>34</v>
+    <row r="18" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="72" t="s">
+        <v>36</v>
       </c>
-      <c r="B14" s="77" t="s">
+      <c r="B18" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="77" t="s">
-        <v>41</v>
+      <c r="C18" s="72" t="s">
+        <v>43</v>
       </c>
-      <c r="D14" s="90" t="s">
-        <v>48</v>
+      <c r="D18" s="245" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="77" t="s">
-        <v>35</v>
+    <row r="19" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="72" t="s">
+        <v>37</v>
       </c>
-      <c r="B15" s="77" t="s">
+      <c r="B19" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="77" t="s">
-        <v>42</v>
+      <c r="C19" s="72" t="s">
+        <v>44</v>
       </c>
-      <c r="D15" s="90" t="s">
-        <v>48</v>
+      <c r="D19" s="245" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:14" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="77" t="s">
-        <v>36</v>
+    <row r="20" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="72" t="s">
+        <v>38</v>
       </c>
-      <c r="B16" s="77" t="s">
+      <c r="B20" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="77" t="s">
-        <v>43</v>
+      <c r="C20" s="72" t="s">
+        <v>45</v>
       </c>
-      <c r="D16" s="90" t="s">
-        <v>49</v>
+      <c r="D20" s="245" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="77" t="s">
+    <row r="21" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="77" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="90" t="s">
-        <v>49</v>
-      </c>
+      <c r="D21" s="245"/>
     </row>
-    <row r="18" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="77" t="s">
+    <row r="22" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="90" t="s">
-        <v>48</v>
-      </c>
+      <c r="D22" s="245"/>
     </row>
-    <row r="19" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="77" t="s">
-        <v>39</v>
-      </c>
-      <c r="B19" s="77" t="s">
+    <row r="23" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="77" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="90" t="s">
-        <v>48</v>
-      </c>
+      <c r="D23" s="245"/>
     </row>
-    <row r="20" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="77" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="77" t="s">
+    <row r="24" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="90" t="s">
-        <v>48</v>
-      </c>
+      <c r="D24" s="245"/>
     </row>
-    <row r="21" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="77" t="s">
+    <row r="25" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="90"/>
+      <c r="D25" s="245"/>
     </row>
-    <row r="22" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="77" t="s">
+    <row r="26" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="D22" s="90"/>
+      <c r="D26" s="245"/>
     </row>
-    <row r="23" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="77" t="s">
+    <row r="27" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="72" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="77" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="77" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="77" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" s="77" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="77" t="s">
-        <v>13</v>
-      </c>
+      <c r="D27" s="245"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15418,73 +15665,73 @@
     <row r="3" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
-      <c r="E3" s="204"/>
+      <c r="E3" s="189"/>
       <c r="F3" s="10"/>
       <c r="G3" s="11"/>
       <c r="K3" s="1"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="206"/>
+      <c r="M3" s="191"/>
       <c r="N3" s="2"/>
       <c r="O3" s="3"/>
     </row>
     <row r="4" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="12"/>
-      <c r="D4" s="182"/>
-      <c r="E4" s="205"/>
-      <c r="F4" s="182"/>
+      <c r="D4" s="167"/>
+      <c r="E4" s="190"/>
+      <c r="F4" s="167"/>
       <c r="G4" s="13"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="183"/>
-      <c r="M4" s="207"/>
-      <c r="N4" s="183"/>
+      <c r="L4" s="168"/>
+      <c r="M4" s="192"/>
+      <c r="N4" s="168"/>
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="12"/>
-      <c r="D5" s="182"/>
-      <c r="E5" s="205"/>
-      <c r="F5" s="182"/>
+      <c r="D5" s="167"/>
+      <c r="E5" s="190"/>
+      <c r="F5" s="167"/>
       <c r="G5" s="13"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="183"/>
-      <c r="M5" s="207"/>
-      <c r="N5" s="183"/>
+      <c r="L5" s="168"/>
+      <c r="M5" s="192"/>
+      <c r="N5" s="168"/>
       <c r="O5" s="5"/>
     </row>
     <row r="6" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C6" s="12"/>
-      <c r="D6" s="187"/>
-      <c r="E6" s="187"/>
-      <c r="F6" s="187"/>
+      <c r="D6" s="172"/>
+      <c r="E6" s="172"/>
+      <c r="F6" s="172"/>
       <c r="G6" s="13"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="188"/>
-      <c r="M6" s="188"/>
-      <c r="N6" s="188"/>
+      <c r="L6" s="173"/>
+      <c r="M6" s="173"/>
+      <c r="N6" s="173"/>
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="12"/>
-      <c r="D7" s="186"/>
-      <c r="E7" s="186"/>
-      <c r="F7" s="186"/>
-      <c r="G7" s="66"/>
+      <c r="D7" s="171"/>
+      <c r="E7" s="171"/>
+      <c r="F7" s="171"/>
+      <c r="G7" s="62"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="189"/>
-      <c r="M7" s="189"/>
-      <c r="N7" s="189"/>
-      <c r="O7" s="190"/>
+      <c r="L7" s="174"/>
+      <c r="M7" s="174"/>
+      <c r="N7" s="174"/>
+      <c r="O7" s="175"/>
     </row>
     <row r="8" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="14"/>
-      <c r="D8" s="184"/>
-      <c r="E8" s="184"/>
-      <c r="F8" s="184"/>
+      <c r="D8" s="169"/>
+      <c r="E8" s="169"/>
+      <c r="F8" s="169"/>
       <c r="G8" s="15"/>
       <c r="K8" s="6"/>
-      <c r="L8" s="185"/>
-      <c r="M8" s="185"/>
-      <c r="N8" s="185"/>
+      <c r="L8" s="170"/>
+      <c r="M8" s="170"/>
+      <c r="N8" s="170"/>
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15492,73 +15739,73 @@
     <row r="12" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="16"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="202"/>
+      <c r="E12" s="187"/>
       <c r="F12" s="17"/>
       <c r="G12" s="18"/>
       <c r="K12" s="1"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="199"/>
+      <c r="M12" s="184"/>
       <c r="N12" s="2"/>
       <c r="O12" s="3"/>
     </row>
     <row r="13" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="19"/>
-      <c r="D13" s="194"/>
-      <c r="E13" s="203"/>
-      <c r="F13" s="194"/>
+      <c r="D13" s="179"/>
+      <c r="E13" s="188"/>
+      <c r="F13" s="179"/>
       <c r="G13" s="20"/>
       <c r="K13" s="4"/>
-      <c r="L13" s="183"/>
-      <c r="M13" s="200"/>
-      <c r="N13" s="183"/>
+      <c r="L13" s="168"/>
+      <c r="M13" s="185"/>
+      <c r="N13" s="168"/>
       <c r="O13" s="5"/>
     </row>
     <row r="14" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="19"/>
-      <c r="D14" s="194"/>
-      <c r="E14" s="203"/>
-      <c r="F14" s="194"/>
+      <c r="D14" s="179"/>
+      <c r="E14" s="188"/>
+      <c r="F14" s="179"/>
       <c r="G14" s="20"/>
       <c r="K14" s="4"/>
-      <c r="L14" s="183"/>
-      <c r="M14" s="201"/>
-      <c r="N14" s="183"/>
+      <c r="L14" s="168"/>
+      <c r="M14" s="186"/>
+      <c r="N14" s="168"/>
       <c r="O14" s="5"/>
     </row>
     <row r="15" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C15" s="19"/>
-      <c r="D15" s="198"/>
-      <c r="E15" s="198"/>
-      <c r="F15" s="198"/>
+      <c r="D15" s="183"/>
+      <c r="E15" s="183"/>
+      <c r="F15" s="183"/>
       <c r="G15" s="20"/>
       <c r="K15" s="4"/>
-      <c r="L15" s="195"/>
-      <c r="M15" s="196"/>
-      <c r="N15" s="197"/>
+      <c r="L15" s="180"/>
+      <c r="M15" s="181"/>
+      <c r="N15" s="182"/>
       <c r="O15" s="5"/>
     </row>
     <row r="16" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="19"/>
-      <c r="D16" s="192"/>
-      <c r="E16" s="192"/>
-      <c r="F16" s="192"/>
-      <c r="G16" s="193"/>
+      <c r="D16" s="177"/>
+      <c r="E16" s="177"/>
+      <c r="F16" s="177"/>
+      <c r="G16" s="178"/>
       <c r="K16" s="4"/>
-      <c r="L16" s="189"/>
-      <c r="M16" s="189"/>
-      <c r="N16" s="189"/>
-      <c r="O16" s="190"/>
+      <c r="L16" s="174"/>
+      <c r="M16" s="174"/>
+      <c r="N16" s="174"/>
+      <c r="O16" s="175"/>
     </row>
     <row r="17" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17" s="21"/>
-      <c r="D17" s="191"/>
-      <c r="E17" s="191"/>
-      <c r="F17" s="191"/>
+      <c r="D17" s="176"/>
+      <c r="E17" s="176"/>
+      <c r="F17" s="176"/>
       <c r="G17" s="22"/>
       <c r="K17" s="6"/>
-      <c r="L17" s="185"/>
-      <c r="M17" s="185"/>
-      <c r="N17" s="185"/>
+      <c r="L17" s="170"/>
+      <c r="M17" s="170"/>
+      <c r="N17" s="170"/>
       <c r="O17" s="7"/>
     </row>
     <row r="18" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15566,73 +15813,73 @@
     <row r="21" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="23"/>
       <c r="D21" s="24"/>
-      <c r="E21" s="209"/>
+      <c r="E21" s="194"/>
       <c r="F21" s="24"/>
       <c r="G21" s="25"/>
       <c r="K21" s="1"/>
       <c r="L21" s="2"/>
-      <c r="M21" s="199"/>
+      <c r="M21" s="184"/>
       <c r="N21" s="2"/>
       <c r="O21" s="3"/>
     </row>
     <row r="22" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="26"/>
-      <c r="D22" s="208"/>
-      <c r="E22" s="210"/>
-      <c r="F22" s="208"/>
+      <c r="D22" s="193"/>
+      <c r="E22" s="195"/>
+      <c r="F22" s="193"/>
       <c r="G22" s="27"/>
       <c r="K22" s="4"/>
-      <c r="L22" s="183"/>
-      <c r="M22" s="200"/>
-      <c r="N22" s="183"/>
+      <c r="L22" s="168"/>
+      <c r="M22" s="185"/>
+      <c r="N22" s="168"/>
       <c r="O22" s="5"/>
     </row>
     <row r="23" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="26"/>
-      <c r="D23" s="208"/>
-      <c r="E23" s="210"/>
-      <c r="F23" s="208"/>
+      <c r="D23" s="193"/>
+      <c r="E23" s="195"/>
+      <c r="F23" s="193"/>
       <c r="G23" s="27"/>
       <c r="K23" s="4"/>
-      <c r="L23" s="183"/>
-      <c r="M23" s="201"/>
-      <c r="N23" s="183"/>
+      <c r="L23" s="168"/>
+      <c r="M23" s="186"/>
+      <c r="N23" s="168"/>
       <c r="O23" s="5"/>
     </row>
     <row r="24" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C24" s="26"/>
-      <c r="D24" s="217"/>
-      <c r="E24" s="217"/>
-      <c r="F24" s="217"/>
+      <c r="D24" s="202"/>
+      <c r="E24" s="202"/>
+      <c r="F24" s="202"/>
       <c r="G24" s="27"/>
       <c r="K24" s="4"/>
-      <c r="L24" s="195"/>
-      <c r="M24" s="196"/>
-      <c r="N24" s="197"/>
+      <c r="L24" s="180"/>
+      <c r="M24" s="181"/>
+      <c r="N24" s="182"/>
       <c r="O24" s="5"/>
     </row>
     <row r="25" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C25" s="26"/>
-      <c r="D25" s="215"/>
-      <c r="E25" s="215"/>
-      <c r="F25" s="215"/>
-      <c r="G25" s="216"/>
+      <c r="D25" s="200"/>
+      <c r="E25" s="200"/>
+      <c r="F25" s="200"/>
+      <c r="G25" s="201"/>
       <c r="K25" s="4"/>
-      <c r="L25" s="189"/>
-      <c r="M25" s="189"/>
-      <c r="N25" s="189"/>
-      <c r="O25" s="190"/>
+      <c r="L25" s="174"/>
+      <c r="M25" s="174"/>
+      <c r="N25" s="174"/>
+      <c r="O25" s="175"/>
     </row>
     <row r="26" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C26" s="28"/>
-      <c r="D26" s="214"/>
-      <c r="E26" s="214"/>
-      <c r="F26" s="214"/>
+      <c r="D26" s="199"/>
+      <c r="E26" s="199"/>
+      <c r="F26" s="199"/>
       <c r="G26" s="29"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="185"/>
-      <c r="M26" s="185"/>
-      <c r="N26" s="185"/>
+      <c r="L26" s="170"/>
+      <c r="M26" s="170"/>
+      <c r="N26" s="170"/>
       <c r="O26" s="7"/>
     </row>
     <row r="27" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15640,73 +15887,73 @@
     <row r="30" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="37"/>
       <c r="D30" s="38"/>
-      <c r="E30" s="224"/>
+      <c r="E30" s="209"/>
       <c r="F30" s="38"/>
       <c r="G30" s="39"/>
       <c r="K30" s="1"/>
       <c r="L30" s="2"/>
-      <c r="M30" s="199"/>
+      <c r="M30" s="184"/>
       <c r="N30" s="2"/>
       <c r="O30" s="3"/>
     </row>
     <row r="31" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="40"/>
-      <c r="D31" s="218"/>
-      <c r="E31" s="225"/>
-      <c r="F31" s="218"/>
+      <c r="D31" s="203"/>
+      <c r="E31" s="210"/>
+      <c r="F31" s="203"/>
       <c r="G31" s="41"/>
       <c r="K31" s="4"/>
-      <c r="L31" s="183"/>
-      <c r="M31" s="200"/>
-      <c r="N31" s="183"/>
+      <c r="L31" s="168"/>
+      <c r="M31" s="185"/>
+      <c r="N31" s="168"/>
       <c r="O31" s="5"/>
     </row>
     <row r="32" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="40"/>
-      <c r="D32" s="218"/>
-      <c r="E32" s="225"/>
-      <c r="F32" s="218"/>
+      <c r="D32" s="203"/>
+      <c r="E32" s="210"/>
+      <c r="F32" s="203"/>
       <c r="G32" s="41"/>
       <c r="K32" s="4"/>
-      <c r="L32" s="183"/>
-      <c r="M32" s="201"/>
-      <c r="N32" s="183"/>
+      <c r="L32" s="168"/>
+      <c r="M32" s="186"/>
+      <c r="N32" s="168"/>
       <c r="O32" s="5"/>
     </row>
     <row r="33" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C33" s="40"/>
-      <c r="D33" s="223"/>
-      <c r="E33" s="223"/>
-      <c r="F33" s="223"/>
+      <c r="D33" s="208"/>
+      <c r="E33" s="208"/>
+      <c r="F33" s="208"/>
       <c r="G33" s="41"/>
       <c r="K33" s="4"/>
-      <c r="L33" s="195"/>
-      <c r="M33" s="196"/>
-      <c r="N33" s="197"/>
+      <c r="L33" s="180"/>
+      <c r="M33" s="181"/>
+      <c r="N33" s="182"/>
       <c r="O33" s="5"/>
     </row>
     <row r="34" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="40"/>
-      <c r="D34" s="212"/>
-      <c r="E34" s="212"/>
-      <c r="F34" s="212"/>
-      <c r="G34" s="213"/>
+      <c r="D34" s="197"/>
+      <c r="E34" s="197"/>
+      <c r="F34" s="197"/>
+      <c r="G34" s="198"/>
       <c r="K34" s="4"/>
-      <c r="L34" s="189"/>
-      <c r="M34" s="189"/>
-      <c r="N34" s="189"/>
-      <c r="O34" s="190"/>
+      <c r="L34" s="174"/>
+      <c r="M34" s="174"/>
+      <c r="N34" s="174"/>
+      <c r="O34" s="175"/>
     </row>
     <row r="35" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C35" s="42"/>
-      <c r="D35" s="211"/>
-      <c r="E35" s="211"/>
-      <c r="F35" s="211"/>
+      <c r="D35" s="196"/>
+      <c r="E35" s="196"/>
+      <c r="F35" s="196"/>
       <c r="G35" s="43"/>
       <c r="K35" s="6"/>
-      <c r="L35" s="185"/>
-      <c r="M35" s="185"/>
-      <c r="N35" s="185"/>
+      <c r="L35" s="170"/>
+      <c r="M35" s="170"/>
+      <c r="N35" s="170"/>
       <c r="O35" s="7"/>
     </row>
     <row r="36" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15714,73 +15961,73 @@
     <row r="39" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C39" s="44"/>
       <c r="D39" s="45"/>
-      <c r="E39" s="227"/>
+      <c r="E39" s="212"/>
       <c r="F39" s="45"/>
       <c r="G39" s="46"/>
       <c r="K39" s="1"/>
       <c r="L39" s="2"/>
-      <c r="M39" s="199"/>
+      <c r="M39" s="184"/>
       <c r="N39" s="2"/>
       <c r="O39" s="3"/>
     </row>
     <row r="40" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C40" s="47"/>
-      <c r="D40" s="226"/>
-      <c r="E40" s="228"/>
-      <c r="F40" s="226"/>
+      <c r="D40" s="211"/>
+      <c r="E40" s="213"/>
+      <c r="F40" s="211"/>
       <c r="G40" s="48"/>
       <c r="K40" s="4"/>
-      <c r="L40" s="183"/>
-      <c r="M40" s="200"/>
-      <c r="N40" s="183"/>
+      <c r="L40" s="168"/>
+      <c r="M40" s="185"/>
+      <c r="N40" s="168"/>
       <c r="O40" s="5"/>
     </row>
     <row r="41" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C41" s="47"/>
-      <c r="D41" s="226"/>
-      <c r="E41" s="228"/>
-      <c r="F41" s="226"/>
+      <c r="D41" s="211"/>
+      <c r="E41" s="213"/>
+      <c r="F41" s="211"/>
       <c r="G41" s="48"/>
       <c r="K41" s="4"/>
-      <c r="L41" s="183"/>
-      <c r="M41" s="201"/>
-      <c r="N41" s="183"/>
+      <c r="L41" s="168"/>
+      <c r="M41" s="186"/>
+      <c r="N41" s="168"/>
       <c r="O41" s="5"/>
     </row>
     <row r="42" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C42" s="47"/>
-      <c r="D42" s="222"/>
-      <c r="E42" s="222"/>
-      <c r="F42" s="222"/>
+      <c r="D42" s="207"/>
+      <c r="E42" s="207"/>
+      <c r="F42" s="207"/>
       <c r="G42" s="48"/>
       <c r="K42" s="4"/>
-      <c r="L42" s="195"/>
-      <c r="M42" s="196"/>
-      <c r="N42" s="197"/>
+      <c r="L42" s="180"/>
+      <c r="M42" s="181"/>
+      <c r="N42" s="182"/>
       <c r="O42" s="5"/>
     </row>
     <row r="43" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C43" s="47"/>
-      <c r="D43" s="220"/>
-      <c r="E43" s="220"/>
-      <c r="F43" s="220"/>
-      <c r="G43" s="221"/>
+      <c r="D43" s="205"/>
+      <c r="E43" s="205"/>
+      <c r="F43" s="205"/>
+      <c r="G43" s="206"/>
       <c r="K43" s="4"/>
-      <c r="L43" s="189"/>
-      <c r="M43" s="189"/>
-      <c r="N43" s="189"/>
-      <c r="O43" s="190"/>
+      <c r="L43" s="174"/>
+      <c r="M43" s="174"/>
+      <c r="N43" s="174"/>
+      <c r="O43" s="175"/>
     </row>
     <row r="44" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C44" s="49"/>
-      <c r="D44" s="219"/>
-      <c r="E44" s="219"/>
-      <c r="F44" s="219"/>
+      <c r="D44" s="204"/>
+      <c r="E44" s="204"/>
+      <c r="F44" s="204"/>
       <c r="G44" s="50"/>
       <c r="K44" s="6"/>
-      <c r="L44" s="185"/>
-      <c r="M44" s="185"/>
-      <c r="N44" s="185"/>
+      <c r="L44" s="170"/>
+      <c r="M44" s="170"/>
+      <c r="N44" s="170"/>
       <c r="O44" s="7"/>
     </row>
     <row r="45" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15788,73 +16035,73 @@
     <row r="48" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C48" s="51"/>
       <c r="D48" s="52"/>
-      <c r="E48" s="233"/>
+      <c r="E48" s="218"/>
       <c r="F48" s="52"/>
       <c r="G48" s="53"/>
       <c r="K48" s="1"/>
       <c r="L48" s="2"/>
-      <c r="M48" s="199"/>
+      <c r="M48" s="184"/>
       <c r="N48" s="2"/>
       <c r="O48" s="3"/>
     </row>
     <row r="49" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C49" s="54"/>
-      <c r="D49" s="177"/>
-      <c r="E49" s="234"/>
-      <c r="F49" s="177"/>
+      <c r="D49" s="162"/>
+      <c r="E49" s="219"/>
+      <c r="F49" s="162"/>
       <c r="G49" s="55"/>
       <c r="K49" s="4"/>
-      <c r="L49" s="183"/>
-      <c r="M49" s="200"/>
-      <c r="N49" s="183"/>
+      <c r="L49" s="168"/>
+      <c r="M49" s="185"/>
+      <c r="N49" s="168"/>
       <c r="O49" s="5"/>
     </row>
     <row r="50" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C50" s="54"/>
-      <c r="D50" s="177"/>
-      <c r="E50" s="234"/>
-      <c r="F50" s="177"/>
+      <c r="D50" s="162"/>
+      <c r="E50" s="219"/>
+      <c r="F50" s="162"/>
       <c r="G50" s="55"/>
       <c r="K50" s="4"/>
-      <c r="L50" s="183"/>
-      <c r="M50" s="201"/>
-      <c r="N50" s="183"/>
+      <c r="L50" s="168"/>
+      <c r="M50" s="186"/>
+      <c r="N50" s="168"/>
       <c r="O50" s="5"/>
     </row>
     <row r="51" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C51" s="54"/>
-      <c r="D51" s="232"/>
-      <c r="E51" s="232"/>
-      <c r="F51" s="232"/>
+      <c r="D51" s="217"/>
+      <c r="E51" s="217"/>
+      <c r="F51" s="217"/>
       <c r="G51" s="55"/>
       <c r="K51" s="4"/>
-      <c r="L51" s="195"/>
-      <c r="M51" s="196"/>
-      <c r="N51" s="197"/>
+      <c r="L51" s="180"/>
+      <c r="M51" s="181"/>
+      <c r="N51" s="182"/>
       <c r="O51" s="5"/>
     </row>
     <row r="52" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C52" s="54"/>
-      <c r="D52" s="230"/>
-      <c r="E52" s="230"/>
-      <c r="F52" s="230"/>
-      <c r="G52" s="231"/>
+      <c r="D52" s="215"/>
+      <c r="E52" s="215"/>
+      <c r="F52" s="215"/>
+      <c r="G52" s="216"/>
       <c r="K52" s="4"/>
-      <c r="L52" s="189"/>
-      <c r="M52" s="189"/>
-      <c r="N52" s="189"/>
-      <c r="O52" s="190"/>
+      <c r="L52" s="174"/>
+      <c r="M52" s="174"/>
+      <c r="N52" s="174"/>
+      <c r="O52" s="175"/>
     </row>
     <row r="53" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C53" s="56"/>
-      <c r="D53" s="229"/>
-      <c r="E53" s="229"/>
-      <c r="F53" s="229"/>
+      <c r="D53" s="214"/>
+      <c r="E53" s="214"/>
+      <c r="F53" s="214"/>
       <c r="G53" s="57"/>
       <c r="K53" s="6"/>
-      <c r="L53" s="185"/>
-      <c r="M53" s="185"/>
-      <c r="N53" s="185"/>
+      <c r="L53" s="170"/>
+      <c r="M53" s="170"/>
+      <c r="N53" s="170"/>
       <c r="O53" s="7"/>
     </row>
     <row r="54" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15965,7 +16212,7 @@
     <row r="3" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="30"/>
       <c r="D3" s="31"/>
-      <c r="E3" s="240"/>
+      <c r="E3" s="225"/>
       <c r="F3" s="31"/>
       <c r="G3" s="32"/>
       <c r="K3" s="1"/>
@@ -15976,62 +16223,62 @@
     </row>
     <row r="4" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="33"/>
-      <c r="D4" s="244"/>
-      <c r="E4" s="241"/>
-      <c r="F4" s="244"/>
+      <c r="D4" s="229"/>
+      <c r="E4" s="226"/>
+      <c r="F4" s="229"/>
       <c r="G4" s="34"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="183"/>
+      <c r="L4" s="168"/>
       <c r="M4" s="8"/>
-      <c r="N4" s="183"/>
+      <c r="N4" s="168"/>
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="33"/>
-      <c r="D5" s="244"/>
-      <c r="E5" s="241"/>
-      <c r="F5" s="244"/>
+      <c r="D5" s="229"/>
+      <c r="E5" s="226"/>
+      <c r="F5" s="229"/>
       <c r="G5" s="34"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="183"/>
+      <c r="L5" s="168"/>
       <c r="M5" s="8"/>
-      <c r="N5" s="183"/>
+      <c r="N5" s="168"/>
       <c r="O5" s="5"/>
     </row>
     <row r="6" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C6" s="33"/>
-      <c r="D6" s="245"/>
-      <c r="E6" s="245"/>
-      <c r="F6" s="245"/>
+      <c r="D6" s="230"/>
+      <c r="E6" s="230"/>
+      <c r="F6" s="230"/>
       <c r="G6" s="34"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="235"/>
-      <c r="M6" s="236"/>
-      <c r="N6" s="237"/>
+      <c r="L6" s="220"/>
+      <c r="M6" s="221"/>
+      <c r="N6" s="222"/>
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="33"/>
-      <c r="D7" s="242"/>
-      <c r="E7" s="242"/>
-      <c r="F7" s="242"/>
-      <c r="G7" s="243"/>
+      <c r="D7" s="227"/>
+      <c r="E7" s="227"/>
+      <c r="F7" s="227"/>
+      <c r="G7" s="228"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="238"/>
-      <c r="M7" s="238"/>
-      <c r="N7" s="238"/>
+      <c r="L7" s="223"/>
+      <c r="M7" s="223"/>
+      <c r="N7" s="223"/>
       <c r="O7" s="5"/>
     </row>
     <row r="8" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="35"/>
-      <c r="D8" s="239"/>
-      <c r="E8" s="239"/>
-      <c r="F8" s="239"/>
+      <c r="D8" s="224"/>
+      <c r="E8" s="224"/>
+      <c r="F8" s="224"/>
       <c r="G8" s="36"/>
       <c r="K8" s="6"/>
-      <c r="L8" s="185"/>
-      <c r="M8" s="185"/>
-      <c r="N8" s="185"/>
+      <c r="L8" s="170"/>
+      <c r="M8" s="170"/>
+      <c r="N8" s="170"/>
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Modifier card art WIP
Same as attack cards - added brief temporary art for each modifier card that will be changed as I work on them
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267C5140-6AF5-415C-979F-318696290F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DEDA504-A4CB-4AB2-94FD-39BA62A850A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="27">
+  <futureMetadata name="XLRICHVALUE" count="41">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -233,8 +233,106 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="27"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="28"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="29"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="30"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="31"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="32"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="33"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="34"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="35"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="36"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="37"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="38"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="39"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="40"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="27">
+  <valueMetadata count="41">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -315,6 +413,48 @@
     </bk>
     <bk>
       <rc t="1" v="26"/>
+    </bk>
+    <bk>
+      <rc t="1" v="27"/>
+    </bk>
+    <bk>
+      <rc t="1" v="28"/>
+    </bk>
+    <bk>
+      <rc t="1" v="29"/>
+    </bk>
+    <bk>
+      <rc t="1" v="30"/>
+    </bk>
+    <bk>
+      <rc t="1" v="31"/>
+    </bk>
+    <bk>
+      <rc t="1" v="32"/>
+    </bk>
+    <bk>
+      <rc t="1" v="33"/>
+    </bk>
+    <bk>
+      <rc t="1" v="34"/>
+    </bk>
+    <bk>
+      <rc t="1" v="35"/>
+    </bk>
+    <bk>
+      <rc t="1" v="36"/>
+    </bk>
+    <bk>
+      <rc t="1" v="37"/>
+    </bk>
+    <bk>
+      <rc t="1" v="38"/>
+    </bk>
+    <bk>
+      <rc t="1" v="39"/>
+    </bk>
+    <bk>
+      <rc t="1" v="40"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -477,7 +617,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -559,6 +699,12 @@
     <font>
       <sz val="28"/>
       <color theme="0"/>
+      <name val="Germania One"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="29"/>
+      <color theme="1"/>
       <name val="Germania One"/>
       <family val="2"/>
     </font>
@@ -799,7 +945,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="247">
+  <cellXfs count="248">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1371,6 +1517,9 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1427,7 +1576,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6856"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6880"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1542,7 +1691,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6857"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6881"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1602,7 +1751,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6858"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6882"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1662,7 +1811,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6859"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6883"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1722,7 +1871,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6860"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6884"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1782,7 +1931,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6861"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6885"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1842,7 +1991,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6862"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6886"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1902,7 +2051,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6863"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6887"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1962,7 +2111,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6864"/>
+                  <a14:cameraTool cellRange="Src!$A$2" spid="_x0000_s6888"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2027,7 +2176,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6865"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6889"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2092,7 +2241,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6866"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6890"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2157,7 +2306,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6867"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6891"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2222,7 +2371,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6868"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6892"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2287,7 +2436,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6869"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6893"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2352,7 +2501,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6870"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6894"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2417,7 +2566,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6871"/>
+                  <a14:cameraTool cellRange="Src!$C$2" spid="_x0000_s6895"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2482,7 +2631,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$J$1" spid="_x0000_s6872"/>
+                  <a14:cameraTool cellRange="Src!$J$1" spid="_x0000_s6896"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2547,7 +2696,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$J$1" spid="_x0000_s6873"/>
+                  <a14:cameraTool cellRange="Src!$J$1" spid="_x0000_s6897"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2612,7 +2761,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$K$1" spid="_x0000_s6874"/>
+                  <a14:cameraTool cellRange="Src!$K$1" spid="_x0000_s6898"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2677,7 +2826,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$H$1" spid="_x0000_s6875"/>
+                  <a14:cameraTool cellRange="Src!$H$1" spid="_x0000_s6899"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2742,7 +2891,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$I$1" spid="_x0000_s6876"/>
+                  <a14:cameraTool cellRange="Src!$I$1" spid="_x0000_s6900"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2807,7 +2956,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$L$1" spid="_x0000_s6877"/>
+                  <a14:cameraTool cellRange="Src!$L$1" spid="_x0000_s6901"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2872,7 +3021,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$M$1" spid="_x0000_s6878"/>
+                  <a14:cameraTool cellRange="Src!$M$1" spid="_x0000_s6902"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2937,7 +3086,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="Src!$M$1" spid="_x0000_s6879"/>
+                  <a14:cameraTool cellRange="Src!$M$1" spid="_x0000_s6903"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -14047,7 +14196,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="27">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="41">
   <rv s="0">
     <v>0</v>
     <v>4</v>
@@ -14086,31 +14235,31 @@
   </rv>
   <rv s="0">
     <v>9</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>10</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>11</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>12</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>13</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>14</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>15</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>16</v>
@@ -14118,6 +14267,34 @@
   </rv>
   <rv s="0">
     <v>17</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>18</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>19</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>20</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>21</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>22</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>23</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>24</v>
     <v>5</v>
   </rv>
   <rv s="0">
@@ -14156,6 +14333,34 @@
     <v>8</v>
     <v>5</v>
   </rv>
+  <rv s="0">
+    <v>9</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>10</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>11</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>12</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>13</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>14</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>15</v>
+    <v>5</v>
+  </rv>
 </rvData>
 </file>
 
@@ -14188,6 +14393,13 @@
   <rel r:id="rId16"/>
   <rel r:id="rId17"/>
   <rel r:id="rId18"/>
+  <rel r:id="rId19"/>
+  <rel r:id="rId20"/>
+  <rel r:id="rId21"/>
+  <rel r:id="rId22"/>
+  <rel r:id="rId23"/>
+  <rel r:id="rId24"/>
+  <rel r:id="rId25"/>
 </richValueRels>
 </file>
 
@@ -14843,25 +15055,25 @@
       <c r="E16" s="162"/>
       <c r="F16" s="119"/>
       <c r="H16" s="146"/>
-      <c r="I16" s="246">
+      <c r="I16" s="246" t="e" vm="10">
         <f>Src!E14</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J16" s="246"/>
       <c r="K16" s="246"/>
       <c r="L16" s="147"/>
       <c r="N16" s="146"/>
-      <c r="O16" s="164">
+      <c r="O16" s="164" t="e" vm="11">
         <f>Src!E15</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="P16" s="164"/>
       <c r="Q16" s="164"/>
       <c r="R16" s="147"/>
       <c r="T16" s="146"/>
-      <c r="U16" s="164">
+      <c r="U16" s="164" t="e" vm="12">
         <f xml:space="preserve"> Src!E16</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="V16" s="164"/>
       <c r="W16" s="164"/>
@@ -14973,7 +15185,7 @@
       <c r="R21" s="145"/>
       <c r="T21" s="142"/>
       <c r="U21" s="143"/>
-      <c r="V21" s="154" t="str">
+      <c r="V21" s="247" t="str">
         <f>Src!A20</f>
         <v>HOLY BLADE</v>
       </c>
@@ -14982,33 +15194,33 @@
     </row>
     <row r="22" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="146"/>
-      <c r="C22" s="164">
+      <c r="C22" s="164" t="e" vm="13">
         <f>Src!E17</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="D22" s="164"/>
       <c r="E22" s="164"/>
       <c r="F22" s="147"/>
       <c r="H22" s="146"/>
-      <c r="I22" s="164">
+      <c r="I22" s="164" t="e" vm="14">
         <f>Src!E18</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="J22" s="164"/>
       <c r="K22" s="164"/>
       <c r="L22" s="147"/>
       <c r="N22" s="146"/>
-      <c r="O22" s="164">
+      <c r="O22" s="164" t="e" vm="15">
         <f>Src!E19</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="P22" s="164"/>
       <c r="Q22" s="164"/>
       <c r="R22" s="147"/>
       <c r="T22" s="146"/>
-      <c r="U22" s="164">
+      <c r="U22" s="164" t="e" vm="16">
         <f xml:space="preserve"> Src!E20</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="V22" s="164"/>
       <c r="W22" s="164"/>
@@ -15290,33 +15502,33 @@
       <c r="F1" s="58" t="s">
         <v>49</v>
       </c>
-      <c r="G1" t="e" vm="10">
+      <c r="G1" t="e" vm="17">
         <v>#VALUE!</v>
       </c>
-      <c r="H1" t="e" vm="11">
+      <c r="H1" t="e" vm="18">
         <v>#VALUE!</v>
       </c>
-      <c r="I1" t="e" vm="12">
+      <c r="I1" t="e" vm="19">
         <v>#VALUE!</v>
       </c>
-      <c r="J1" t="e" vm="13">
+      <c r="J1" t="e" vm="20">
         <v>#VALUE!</v>
       </c>
-      <c r="K1" t="e" vm="14">
+      <c r="K1" t="e" vm="21">
         <v>#VALUE!</v>
       </c>
-      <c r="L1" t="e" vm="15">
+      <c r="L1" t="e" vm="22">
         <v>#VALUE!</v>
       </c>
-      <c r="M1" t="e" vm="16">
+      <c r="M1" t="e" vm="23">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="e" vm="17">
+      <c r="A2" t="e" vm="24">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" t="e" vm="18">
+      <c r="C2" t="e" vm="25">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15353,7 +15565,7 @@
       <c r="D5" s="245" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="61" t="e" vm="19">
+      <c r="E5" s="61" t="e" vm="26">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15370,7 +15582,7 @@
       <c r="D6" s="245" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="72" t="e" vm="20">
+      <c r="E6" s="72" t="e" vm="27">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15387,7 +15599,7 @@
       <c r="D7" s="245" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="72" t="e" vm="21">
+      <c r="E7" s="72" t="e" vm="28">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15404,7 +15616,7 @@
       <c r="D8" s="245" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="72" t="e" vm="22">
+      <c r="E8" s="72" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15421,7 +15633,7 @@
       <c r="D9" s="245" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="72" t="e" vm="23">
+      <c r="E9" s="72" t="e" vm="30">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15438,7 +15650,7 @@
       <c r="D10" s="245" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="72" t="e" vm="24">
+      <c r="E10" s="72" t="e" vm="31">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15455,7 +15667,7 @@
       <c r="D11" s="245" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="72" t="e" vm="25">
+      <c r="E11" s="72" t="e" vm="32">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15472,7 +15684,7 @@
       <c r="D12" s="245" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="72" t="e" vm="26">
+      <c r="E12" s="72" t="e" vm="33">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15489,7 +15701,7 @@
       <c r="D13" s="245" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="72" t="e" vm="27">
+      <c r="E13" s="72" t="e" vm="34">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -15506,6 +15718,9 @@
       <c r="D14" s="245" t="s">
         <v>46</v>
       </c>
+      <c r="E14" s="72" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="15" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="72" t="s">
@@ -15519,6 +15734,9 @@
       </c>
       <c r="D15" s="245" t="s">
         <v>46</v>
+      </c>
+      <c r="E15" s="72" t="e" vm="36">
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="1:13" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
@@ -15534,8 +15752,11 @@
       <c r="D16" s="245" t="s">
         <v>47</v>
       </c>
+      <c r="E16" s="72" t="e" vm="37">
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="17" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="72" t="s">
         <v>35</v>
       </c>
@@ -15548,8 +15769,11 @@
       <c r="D17" s="245" t="s">
         <v>47</v>
       </c>
+      <c r="E17" s="72" t="e" vm="38">
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="18" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="72" t="s">
         <v>36</v>
       </c>
@@ -15562,8 +15786,11 @@
       <c r="D18" s="245" t="s">
         <v>46</v>
       </c>
+      <c r="E18" s="72" t="e" vm="39">
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="19" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="72" t="s">
         <v>37</v>
       </c>
@@ -15576,8 +15803,11 @@
       <c r="D19" s="245" t="s">
         <v>46</v>
       </c>
+      <c r="E19" s="72" t="e" vm="40">
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="20" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
         <v>38</v>
       </c>
@@ -15590,44 +15820,47 @@
       <c r="D20" s="245" t="s">
         <v>46</v>
       </c>
+      <c r="E20" s="72" t="e" vm="41">
+        <v>#VALUE!</v>
+      </c>
     </row>
-    <row r="21" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="72" t="s">
         <v>13</v>
       </c>
       <c r="D21" s="245"/>
     </row>
-    <row r="22" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="72" t="s">
         <v>13</v>
       </c>
       <c r="D22" s="245"/>
     </row>
-    <row r="23" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="72" t="s">
         <v>13</v>
       </c>
       <c r="D23" s="245"/>
     </row>
-    <row r="24" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="72" t="s">
         <v>13</v>
       </c>
       <c r="D24" s="245"/>
     </row>
-    <row r="25" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="72" t="s">
         <v>13</v>
       </c>
       <c r="D25" s="245"/>
     </row>
-    <row r="26" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="72" t="s">
         <v>13</v>
       </c>
       <c r="D26" s="245"/>
     </row>
-    <row r="27" spans="1:4" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" s="72" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="72" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Art - Recall and Greed
Added new art for Recall and Greed modifier cards
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB0A483-58EA-410C-897C-A1CEE9EB9D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEE7643-0666-4183-91A8-C247F969FD13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="45">
+  <futureMetadata name="XLRICHVALUE" count="49">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -359,8 +359,36 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="45"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="46"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="47"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="48"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="45">
+  <valueMetadata count="49">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -496,12 +524,24 @@
     <bk>
       <rc t="1" v="44"/>
     </bk>
+    <bk>
+      <rc t="1" v="45"/>
+    </bk>
+    <bk>
+      <rc t="1" v="46"/>
+    </bk>
+    <bk>
+      <rc t="1" v="47"/>
+    </bk>
+    <bk>
+      <rc t="1" v="48"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="55">
   <si>
     <t>FIREBALL</t>
   </si>
@@ -992,7 +1032,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="172">
+  <cellXfs count="178">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1190,9 +1230,6 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1289,9 +1326,6 @@
     <xf numFmtId="0" fontId="5" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1394,7 +1428,31 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1539,7 +1597,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12052"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12151"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1599,7 +1657,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12053"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12152"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1659,7 +1717,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12054"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12153"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1719,7 +1777,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12055"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12154"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1779,7 +1837,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12056"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12155"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1839,7 +1897,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12057"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12156"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1899,7 +1957,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12058"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$A$2" spid="_x0000_s12157"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -1964,7 +2022,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12059"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12158"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2029,7 +2087,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12060"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12159"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2094,7 +2152,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12061"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12160"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2159,7 +2217,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12062"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12161"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2224,7 +2282,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12063"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12162"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2289,7 +2347,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12064"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12163"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2354,7 +2412,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12065"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12164"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2419,7 +2477,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12066"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12165"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2484,7 +2542,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12067"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12166"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2549,7 +2607,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12068"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12167"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2614,7 +2672,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12069"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12168"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2679,7 +2737,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12070"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12169"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2744,7 +2802,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12071"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12170"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2809,7 +2867,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12072"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12171"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2874,7 +2932,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12073"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12172"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2939,7 +2997,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12074"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12173"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3004,7 +3062,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12075"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12174"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3069,7 +3127,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12076"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12175"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3134,7 +3192,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12077"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12176"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3199,7 +3257,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12078"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12177"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3264,7 +3322,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12079"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12178"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3329,7 +3387,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12080"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12179"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3438,7 +3496,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12081"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12180"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3503,7 +3561,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12082"/>
+                  <a14:cameraTool cellRange="'Cards Src'!$C$2" spid="_x0000_s12181"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3568,7 +3626,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12083"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12182"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3633,7 +3691,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12084"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s12183"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -8146,7 +8204,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="45">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="49">
   <rv s="0">
     <v>0</v>
     <v>4</v>
@@ -8213,11 +8271,11 @@
   </rv>
   <rv s="0">
     <v>16</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>17</v>
-    <v>5</v>
+    <v>4</v>
   </rv>
   <rv s="0">
     <v>18</v>
@@ -8225,6 +8283,14 @@
   </rv>
   <rv s="0">
     <v>19</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>20</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>21</v>
     <v>5</v>
   </rv>
   <rv s="0">
@@ -8292,11 +8358,11 @@
     <v>5</v>
   </rv>
   <rv s="0">
-    <v>20</v>
+    <v>16</v>
     <v>5</v>
   </rv>
   <rv s="0">
-    <v>21</v>
+    <v>17</v>
     <v>5</v>
   </rv>
   <rv s="0">
@@ -8325,6 +8391,14 @@
   </rv>
   <rv s="0">
     <v>28</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>29</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>30</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -8370,6 +8444,8 @@
   <rel r:id="rId27"/>
   <rel r:id="rId28"/>
   <rel r:id="rId29"/>
+  <rel r:id="rId30"/>
+  <rel r:id="rId31"/>
 </richValueRels>
 </file>
 
@@ -8723,70 +8799,70 @@
     </row>
     <row r="4" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="49"/>
-      <c r="C4" s="139" t="e" vm="1">
+      <c r="C4" s="137" t="e" vm="1">
         <f>'Cards Src'!E7</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="139"/>
-      <c r="E4" s="139"/>
+      <c r="D4" s="137"/>
+      <c r="E4" s="137"/>
       <c r="F4" s="50"/>
       <c r="H4" s="61"/>
-      <c r="I4" s="144" t="e" vm="2">
+      <c r="I4" s="142" t="e" vm="2">
         <f>'Cards Src'!E8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="144"/>
+      <c r="J4" s="142"/>
+      <c r="K4" s="142"/>
       <c r="L4" s="62"/>
-      <c r="N4" s="125"/>
-      <c r="O4" s="145" t="e" vm="3">
+      <c r="N4" s="124"/>
+      <c r="O4" s="143" t="e" vm="3">
         <f>'Cards Src'!E9</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P4" s="145"/>
-      <c r="Q4" s="145"/>
+      <c r="P4" s="143"/>
+      <c r="Q4" s="143"/>
       <c r="R4" s="72"/>
       <c r="T4" s="15"/>
-      <c r="U4" s="146" t="e" vm="4">
+      <c r="U4" s="144" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V4" s="146"/>
-      <c r="W4" s="146"/>
+      <c r="V4" s="144"/>
+      <c r="W4" s="144"/>
       <c r="X4" s="37"/>
     </row>
     <row r="5" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="49"/>
-      <c r="C5" s="140" t="str">
+      <c r="C5" s="138" t="str">
         <f>'Cards Src'!$C7</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="140"/>
-      <c r="E5" s="140"/>
+      <c r="D5" s="138"/>
+      <c r="E5" s="138"/>
       <c r="F5" s="51"/>
       <c r="H5" s="61"/>
-      <c r="I5" s="141" t="str">
+      <c r="I5" s="139" t="str">
         <f>'Cards Src'!$C8</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="J5" s="141"/>
-      <c r="K5" s="141"/>
+      <c r="J5" s="139"/>
+      <c r="K5" s="139"/>
       <c r="L5" s="63"/>
       <c r="N5" s="11"/>
-      <c r="O5" s="142" t="str">
+      <c r="O5" s="140" t="str">
         <f>'Cards Src'!C9</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="P5" s="142"/>
-      <c r="Q5" s="142"/>
+      <c r="P5" s="140"/>
+      <c r="Q5" s="140"/>
       <c r="R5" s="73"/>
       <c r="T5" s="15"/>
-      <c r="U5" s="143" t="str">
+      <c r="U5" s="141" t="str">
         <f>'Cards Src'!C10</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="V5" s="143"/>
-      <c r="W5" s="143"/>
+      <c r="V5" s="141"/>
+      <c r="W5" s="141"/>
       <c r="X5" s="38"/>
     </row>
     <row r="6" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8817,7 +8893,7 @@
       <c r="C8" s="18"/>
       <c r="D8" s="18"/>
       <c r="E8" s="18"/>
-      <c r="F8" s="126"/>
+      <c r="F8" s="125"/>
       <c r="H8" s="21"/>
       <c r="I8" s="22"/>
       <c r="J8" s="22"/>
@@ -8832,17 +8908,17 @@
       <c r="U8" s="18"/>
       <c r="V8" s="18"/>
       <c r="W8" s="18"/>
-      <c r="X8" s="126"/>
+      <c r="X8" s="125"/>
     </row>
     <row r="9" spans="2:24" s="29" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="127"/>
-      <c r="C9" s="128"/>
-      <c r="D9" s="129" t="str">
+      <c r="B9" s="126"/>
+      <c r="C9" s="127"/>
+      <c r="D9" s="128" t="str">
         <f>'Cards Src'!$A11</f>
         <v>LIGHTNING BOLT</v>
       </c>
-      <c r="E9" s="128"/>
-      <c r="F9" s="130"/>
+      <c r="E9" s="127"/>
+      <c r="F9" s="129"/>
       <c r="H9" s="77"/>
       <c r="I9" s="78"/>
       <c r="J9" s="94" t="str">
@@ -8859,89 +8935,89 @@
       </c>
       <c r="Q9" s="86"/>
       <c r="R9" s="88"/>
-      <c r="T9" s="127"/>
-      <c r="U9" s="128"/>
-      <c r="V9" s="129" t="str">
+      <c r="T9" s="126"/>
+      <c r="U9" s="127"/>
+      <c r="V9" s="128" t="str">
         <f>'Cards Src'!A14</f>
         <v>CHAIN LIGHTNING</v>
       </c>
-      <c r="W9" s="128"/>
-      <c r="X9" s="130"/>
+      <c r="W9" s="127"/>
+      <c r="X9" s="129"/>
     </row>
     <row r="10" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="19"/>
-      <c r="C10" s="147" t="e" vm="5">
+      <c r="C10" s="145" t="e" vm="5">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D10" s="147"/>
-      <c r="E10" s="147"/>
-      <c r="F10" s="135"/>
+      <c r="D10" s="145"/>
+      <c r="E10" s="145"/>
+      <c r="F10" s="134"/>
       <c r="H10" s="23"/>
-      <c r="I10" s="151" t="e" vm="6">
+      <c r="I10" s="149" t="e" vm="6">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J10" s="151"/>
-      <c r="K10" s="151"/>
+      <c r="J10" s="149"/>
+      <c r="K10" s="149"/>
       <c r="L10" s="80"/>
       <c r="N10" s="27"/>
-      <c r="O10" s="152" t="e" vm="7">
+      <c r="O10" s="150" t="e" vm="7">
         <f>'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P10" s="152"/>
-      <c r="Q10" s="152"/>
+      <c r="P10" s="150"/>
+      <c r="Q10" s="150"/>
       <c r="R10" s="89"/>
       <c r="T10" s="19"/>
-      <c r="U10" s="147" t="e" vm="8">
+      <c r="U10" s="145" t="e" vm="8">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V10" s="147"/>
-      <c r="W10" s="147"/>
-      <c r="X10" s="131"/>
+      <c r="V10" s="145"/>
+      <c r="W10" s="145"/>
+      <c r="X10" s="130"/>
     </row>
     <row r="11" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="19"/>
-      <c r="C11" s="148" t="str">
+      <c r="C11" s="146" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Casts a bolt of lightning</v>
       </c>
-      <c r="D11" s="148"/>
-      <c r="E11" s="148"/>
-      <c r="F11" s="132"/>
+      <c r="D11" s="146"/>
+      <c r="E11" s="146"/>
+      <c r="F11" s="131"/>
       <c r="H11" s="23"/>
-      <c r="I11" s="149" t="str">
+      <c r="I11" s="147" t="str">
         <f>'Cards Src'!$C12</f>
         <v>Vacuums in nearby enemies</v>
       </c>
-      <c r="J11" s="149"/>
-      <c r="K11" s="149"/>
+      <c r="J11" s="147"/>
+      <c r="K11" s="147"/>
       <c r="L11" s="81"/>
       <c r="N11" s="27"/>
-      <c r="O11" s="150" t="str">
+      <c r="O11" s="148" t="str">
         <f>'Cards Src'!C13</f>
         <v>Flies to the nearest enemy in vision</v>
       </c>
-      <c r="P11" s="150"/>
-      <c r="Q11" s="150"/>
+      <c r="P11" s="148"/>
+      <c r="Q11" s="148"/>
       <c r="R11" s="90"/>
       <c r="T11" s="19"/>
-      <c r="U11" s="148" t="str">
+      <c r="U11" s="146" t="str">
         <f>'Cards Src'!C14</f>
         <v>Casts a tracking bolt of lightning that can chain to close enemies</v>
       </c>
-      <c r="V11" s="148"/>
-      <c r="W11" s="148"/>
-      <c r="X11" s="132"/>
+      <c r="V11" s="146"/>
+      <c r="W11" s="146"/>
+      <c r="X11" s="131"/>
     </row>
     <row r="12" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="20"/>
-      <c r="C12" s="133"/>
-      <c r="D12" s="133"/>
-      <c r="E12" s="133"/>
-      <c r="F12" s="134"/>
+      <c r="C12" s="132"/>
+      <c r="D12" s="132"/>
+      <c r="E12" s="132"/>
+      <c r="F12" s="133"/>
       <c r="H12" s="24"/>
       <c r="I12" s="82"/>
       <c r="J12" s="82"/>
@@ -8953,10 +9029,10 @@
       <c r="Q12" s="91"/>
       <c r="R12" s="92"/>
       <c r="T12" s="20"/>
-      <c r="U12" s="133"/>
-      <c r="V12" s="133"/>
-      <c r="W12" s="133"/>
-      <c r="X12" s="134"/>
+      <c r="U12" s="132"/>
+      <c r="V12" s="132"/>
+      <c r="W12" s="132"/>
+      <c r="X12" s="133"/>
     </row>
     <row r="13" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8965,21 +9041,21 @@
       <c r="D14" s="26"/>
       <c r="E14" s="26"/>
       <c r="F14" s="84"/>
-      <c r="H14" s="109"/>
-      <c r="I14" s="110"/>
-      <c r="J14" s="110"/>
-      <c r="K14" s="110"/>
-      <c r="L14" s="111"/>
-      <c r="N14" s="109"/>
-      <c r="O14" s="110"/>
-      <c r="P14" s="110"/>
-      <c r="Q14" s="110"/>
-      <c r="R14" s="111"/>
-      <c r="T14" s="109"/>
-      <c r="U14" s="110"/>
-      <c r="V14" s="110"/>
-      <c r="W14" s="110"/>
-      <c r="X14" s="111"/>
+      <c r="H14" s="108"/>
+      <c r="I14" s="109"/>
+      <c r="J14" s="109"/>
+      <c r="K14" s="109"/>
+      <c r="L14" s="110"/>
+      <c r="N14" s="108"/>
+      <c r="O14" s="109"/>
+      <c r="P14" s="109"/>
+      <c r="Q14" s="109"/>
+      <c r="R14" s="110"/>
+      <c r="T14" s="108"/>
+      <c r="U14" s="109"/>
+      <c r="V14" s="109"/>
+      <c r="W14" s="109"/>
+      <c r="X14" s="110"/>
     </row>
     <row r="15" spans="2:24" s="29" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="85"/>
@@ -8990,98 +9066,98 @@
       </c>
       <c r="E15" s="86"/>
       <c r="F15" s="88"/>
-      <c r="H15" s="112"/>
-      <c r="I15" s="113"/>
-      <c r="J15" s="114" t="str">
+      <c r="H15" s="111"/>
+      <c r="I15" s="112"/>
+      <c r="J15" s="113" t="str">
         <f>'Cards Src'!A16</f>
         <v>HASTE</v>
       </c>
-      <c r="K15" s="113"/>
-      <c r="L15" s="115"/>
-      <c r="N15" s="112"/>
-      <c r="O15" s="113"/>
-      <c r="P15" s="114" t="str">
+      <c r="K15" s="112"/>
+      <c r="L15" s="114"/>
+      <c r="N15" s="111"/>
+      <c r="O15" s="112"/>
+      <c r="P15" s="113" t="str">
         <f>'Cards Src'!A17</f>
         <v>HINDER</v>
       </c>
-      <c r="Q15" s="113"/>
-      <c r="R15" s="115"/>
-      <c r="T15" s="112"/>
-      <c r="U15" s="113"/>
-      <c r="V15" s="123" t="str">
+      <c r="Q15" s="112"/>
+      <c r="R15" s="114"/>
+      <c r="T15" s="111"/>
+      <c r="U15" s="112"/>
+      <c r="V15" s="122" t="str">
         <f>'Cards Src'!A18</f>
         <v>MULLIGAN</v>
       </c>
-      <c r="W15" s="113"/>
-      <c r="X15" s="115"/>
+      <c r="W15" s="112"/>
+      <c r="X15" s="114"/>
     </row>
     <row r="16" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="27"/>
-      <c r="C16" s="152" t="e" vm="9">
+      <c r="C16" s="150" t="e" vm="9">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D16" s="152"/>
-      <c r="E16" s="152"/>
+      <c r="D16" s="150"/>
+      <c r="E16" s="150"/>
       <c r="F16" s="89"/>
-      <c r="H16" s="116"/>
-      <c r="I16" s="155" t="e" vm="10">
+      <c r="H16" s="115"/>
+      <c r="I16" s="153" t="e" vm="10">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J16" s="155"/>
-      <c r="K16" s="155"/>
-      <c r="L16" s="117"/>
-      <c r="N16" s="116"/>
-      <c r="O16" s="156" t="e" vm="11">
+      <c r="J16" s="153"/>
+      <c r="K16" s="153"/>
+      <c r="L16" s="116"/>
+      <c r="N16" s="115"/>
+      <c r="O16" s="154" t="e" vm="11">
         <f>'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P16" s="156"/>
-      <c r="Q16" s="156"/>
-      <c r="R16" s="117"/>
-      <c r="T16" s="116"/>
-      <c r="U16" s="156" t="e" vm="12">
+      <c r="P16" s="154"/>
+      <c r="Q16" s="154"/>
+      <c r="R16" s="116"/>
+      <c r="T16" s="115"/>
+      <c r="U16" s="154" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V16" s="156"/>
-      <c r="W16" s="156"/>
-      <c r="X16" s="117"/>
+      <c r="V16" s="154"/>
+      <c r="W16" s="154"/>
+      <c r="X16" s="116"/>
     </row>
     <row r="17" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="27"/>
-      <c r="C17" s="153" t="str">
+      <c r="C17" s="151" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D17" s="153"/>
-      <c r="E17" s="153"/>
+      <c r="D17" s="151"/>
+      <c r="E17" s="151"/>
       <c r="F17" s="90"/>
-      <c r="H17" s="116"/>
-      <c r="I17" s="154" t="str">
+      <c r="H17" s="115"/>
+      <c r="I17" s="152" t="str">
         <f>'Cards Src'!$C16</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="J17" s="154"/>
-      <c r="K17" s="154"/>
-      <c r="L17" s="119"/>
-      <c r="N17" s="116"/>
-      <c r="O17" s="154" t="str">
+      <c r="J17" s="152"/>
+      <c r="K17" s="152"/>
+      <c r="L17" s="118"/>
+      <c r="N17" s="115"/>
+      <c r="O17" s="152" t="str">
         <f>'Cards Src'!C17</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="P17" s="154"/>
-      <c r="Q17" s="154"/>
-      <c r="R17" s="119"/>
-      <c r="T17" s="116"/>
-      <c r="U17" s="154" t="str">
+      <c r="P17" s="152"/>
+      <c r="Q17" s="152"/>
+      <c r="R17" s="118"/>
+      <c r="T17" s="115"/>
+      <c r="U17" s="152" t="str">
         <f>'Cards Src'!C18</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="V17" s="154"/>
-      <c r="W17" s="154"/>
-      <c r="X17" s="119"/>
+      <c r="V17" s="152"/>
+      <c r="W17" s="152"/>
+      <c r="X17" s="118"/>
     </row>
     <row r="18" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="28"/>
@@ -9089,315 +9165,315 @@
       <c r="D18" s="91"/>
       <c r="E18" s="91"/>
       <c r="F18" s="92"/>
-      <c r="H18" s="120"/>
-      <c r="I18" s="121"/>
-      <c r="J18" s="121"/>
-      <c r="K18" s="121"/>
-      <c r="L18" s="122"/>
-      <c r="N18" s="120"/>
-      <c r="O18" s="121"/>
-      <c r="P18" s="121"/>
-      <c r="Q18" s="121"/>
-      <c r="R18" s="122"/>
-      <c r="T18" s="120"/>
-      <c r="U18" s="121"/>
-      <c r="V18" s="121"/>
-      <c r="W18" s="121"/>
-      <c r="X18" s="122"/>
+      <c r="H18" s="119"/>
+      <c r="I18" s="120"/>
+      <c r="J18" s="120"/>
+      <c r="K18" s="120"/>
+      <c r="L18" s="121"/>
+      <c r="N18" s="119"/>
+      <c r="O18" s="120"/>
+      <c r="P18" s="120"/>
+      <c r="Q18" s="120"/>
+      <c r="R18" s="121"/>
+      <c r="T18" s="119"/>
+      <c r="U18" s="120"/>
+      <c r="V18" s="120"/>
+      <c r="W18" s="120"/>
+      <c r="X18" s="121"/>
     </row>
     <row r="19" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="20" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="109"/>
-      <c r="C20" s="110"/>
-      <c r="D20" s="110"/>
-      <c r="E20" s="110"/>
-      <c r="F20" s="111"/>
-      <c r="H20" s="109"/>
-      <c r="I20" s="110"/>
-      <c r="J20" s="110"/>
-      <c r="K20" s="110"/>
-      <c r="L20" s="111"/>
-      <c r="N20" s="109"/>
-      <c r="O20" s="110"/>
-      <c r="P20" s="110"/>
-      <c r="Q20" s="110"/>
-      <c r="R20" s="111"/>
-      <c r="T20" s="109"/>
-      <c r="U20" s="110"/>
-      <c r="V20" s="110"/>
-      <c r="W20" s="110"/>
-      <c r="X20" s="111"/>
+      <c r="B20" s="108"/>
+      <c r="C20" s="109"/>
+      <c r="D20" s="109"/>
+      <c r="E20" s="109"/>
+      <c r="F20" s="110"/>
+      <c r="H20" s="108"/>
+      <c r="I20" s="109"/>
+      <c r="J20" s="109"/>
+      <c r="K20" s="109"/>
+      <c r="L20" s="110"/>
+      <c r="N20" s="108"/>
+      <c r="O20" s="109"/>
+      <c r="P20" s="109"/>
+      <c r="Q20" s="109"/>
+      <c r="R20" s="110"/>
+      <c r="T20" s="108"/>
+      <c r="U20" s="109"/>
+      <c r="V20" s="109"/>
+      <c r="W20" s="109"/>
+      <c r="X20" s="110"/>
     </row>
     <row r="21" spans="2:24" s="29" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="112"/>
-      <c r="C21" s="113"/>
-      <c r="D21" s="118" t="str">
+      <c r="B21" s="111"/>
+      <c r="C21" s="112"/>
+      <c r="D21" s="117" t="str">
         <f>'Cards Src'!$A19</f>
         <v>BUT WAIT, THERE'S MORE</v>
       </c>
-      <c r="E21" s="113"/>
-      <c r="F21" s="115"/>
-      <c r="H21" s="112"/>
-      <c r="I21" s="113"/>
-      <c r="J21" s="124" t="str">
+      <c r="E21" s="112"/>
+      <c r="F21" s="114"/>
+      <c r="H21" s="111"/>
+      <c r="I21" s="112"/>
+      <c r="J21" s="123" t="str">
         <f>'Cards Src'!A20</f>
         <v>MANA SHIELD</v>
       </c>
-      <c r="K21" s="113"/>
-      <c r="L21" s="115"/>
-      <c r="N21" s="112"/>
-      <c r="O21" s="113"/>
-      <c r="P21" s="124" t="str">
+      <c r="K21" s="112"/>
+      <c r="L21" s="114"/>
+      <c r="N21" s="111"/>
+      <c r="O21" s="112"/>
+      <c r="P21" s="123" t="str">
         <f>'Cards Src'!A21</f>
         <v>RUNAWAY BULL</v>
       </c>
-      <c r="Q21" s="113"/>
-      <c r="R21" s="115"/>
-      <c r="T21" s="112"/>
-      <c r="U21" s="113"/>
-      <c r="V21" s="138" t="str">
+      <c r="Q21" s="112"/>
+      <c r="R21" s="114"/>
+      <c r="T21" s="111"/>
+      <c r="U21" s="112"/>
+      <c r="V21" s="136" t="str">
         <f>'Cards Src'!A22</f>
         <v>HOLY BLADE</v>
       </c>
-      <c r="W21" s="113"/>
-      <c r="X21" s="115"/>
+      <c r="W21" s="112"/>
+      <c r="X21" s="114"/>
     </row>
     <row r="22" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="116"/>
-      <c r="C22" s="156" t="e" vm="13">
+      <c r="B22" s="115"/>
+      <c r="C22" s="154" t="e" vm="13">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D22" s="156"/>
-      <c r="E22" s="156"/>
-      <c r="F22" s="117"/>
-      <c r="H22" s="116"/>
-      <c r="I22" s="156" t="e" vm="14">
+      <c r="D22" s="154"/>
+      <c r="E22" s="154"/>
+      <c r="F22" s="116"/>
+      <c r="H22" s="115"/>
+      <c r="I22" s="154" t="e" vm="14">
         <f>'Cards Src'!E20</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J22" s="156"/>
-      <c r="K22" s="156"/>
-      <c r="L22" s="117"/>
-      <c r="N22" s="116"/>
-      <c r="O22" s="156" t="e" vm="15">
+      <c r="J22" s="154"/>
+      <c r="K22" s="154"/>
+      <c r="L22" s="116"/>
+      <c r="N22" s="115"/>
+      <c r="O22" s="154" t="e" vm="15">
         <f>'Cards Src'!E21</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P22" s="156"/>
-      <c r="Q22" s="156"/>
-      <c r="R22" s="117"/>
-      <c r="T22" s="116"/>
-      <c r="U22" s="156" t="e" vm="16">
+      <c r="P22" s="154"/>
+      <c r="Q22" s="154"/>
+      <c r="R22" s="116"/>
+      <c r="T22" s="115"/>
+      <c r="U22" s="154" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E22</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V22" s="156"/>
-      <c r="W22" s="156"/>
-      <c r="X22" s="117"/>
+      <c r="V22" s="154"/>
+      <c r="W22" s="154"/>
+      <c r="X22" s="116"/>
     </row>
     <row r="23" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="116"/>
-      <c r="C23" s="154" t="str">
+      <c r="B23" s="115"/>
+      <c r="C23" s="152" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D23" s="154"/>
-      <c r="E23" s="154"/>
-      <c r="F23" s="119"/>
-      <c r="H23" s="116"/>
-      <c r="I23" s="154" t="str">
+      <c r="D23" s="152"/>
+      <c r="E23" s="152"/>
+      <c r="F23" s="118"/>
+      <c r="H23" s="115"/>
+      <c r="I23" s="152" t="str">
         <f>'Cards Src'!$C20</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="J23" s="154"/>
-      <c r="K23" s="154"/>
-      <c r="L23" s="119"/>
-      <c r="N23" s="116"/>
-      <c r="O23" s="157" t="str">
+      <c r="J23" s="152"/>
+      <c r="K23" s="152"/>
+      <c r="L23" s="118"/>
+      <c r="N23" s="115"/>
+      <c r="O23" s="155" t="str">
         <f>'Cards Src'!C21</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="P23" s="157"/>
-      <c r="Q23" s="157"/>
-      <c r="R23" s="119"/>
-      <c r="T23" s="116"/>
-      <c r="U23" s="154" t="str">
+      <c r="P23" s="155"/>
+      <c r="Q23" s="155"/>
+      <c r="R23" s="118"/>
+      <c r="T23" s="115"/>
+      <c r="U23" s="152" t="str">
         <f>'Cards Src'!C22</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="V23" s="154"/>
-      <c r="W23" s="154"/>
-      <c r="X23" s="119"/>
+      <c r="V23" s="152"/>
+      <c r="W23" s="152"/>
+      <c r="X23" s="118"/>
     </row>
     <row r="24" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="120"/>
-      <c r="C24" s="121"/>
-      <c r="D24" s="121"/>
-      <c r="E24" s="121"/>
-      <c r="F24" s="122"/>
-      <c r="H24" s="120"/>
-      <c r="I24" s="121"/>
-      <c r="J24" s="121"/>
-      <c r="K24" s="121"/>
-      <c r="L24" s="122"/>
-      <c r="N24" s="120"/>
-      <c r="O24" s="121"/>
-      <c r="P24" s="121"/>
-      <c r="Q24" s="121"/>
-      <c r="R24" s="122"/>
-      <c r="T24" s="120"/>
-      <c r="U24" s="121"/>
-      <c r="V24" s="121"/>
-      <c r="W24" s="121"/>
-      <c r="X24" s="122"/>
+      <c r="B24" s="119"/>
+      <c r="C24" s="120"/>
+      <c r="D24" s="120"/>
+      <c r="E24" s="120"/>
+      <c r="F24" s="121"/>
+      <c r="H24" s="119"/>
+      <c r="I24" s="120"/>
+      <c r="J24" s="120"/>
+      <c r="K24" s="120"/>
+      <c r="L24" s="121"/>
+      <c r="N24" s="119"/>
+      <c r="O24" s="120"/>
+      <c r="P24" s="120"/>
+      <c r="Q24" s="120"/>
+      <c r="R24" s="121"/>
+      <c r="T24" s="119"/>
+      <c r="U24" s="120"/>
+      <c r="V24" s="120"/>
+      <c r="W24" s="120"/>
+      <c r="X24" s="121"/>
     </row>
     <row r="25" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="109"/>
-      <c r="C26" s="110"/>
-      <c r="D26" s="110"/>
-      <c r="E26" s="110"/>
-      <c r="F26" s="111"/>
-      <c r="H26" s="109"/>
-      <c r="I26" s="110"/>
-      <c r="J26" s="110"/>
-      <c r="K26" s="110"/>
-      <c r="L26" s="111"/>
-      <c r="N26" s="96"/>
-      <c r="O26" s="97"/>
-      <c r="P26" s="97"/>
-      <c r="Q26" s="97"/>
-      <c r="R26" s="98"/>
-      <c r="T26" s="96"/>
-      <c r="U26" s="97"/>
-      <c r="V26" s="97"/>
-      <c r="W26" s="97"/>
-      <c r="X26" s="98"/>
+      <c r="B26" s="108"/>
+      <c r="C26" s="109"/>
+      <c r="D26" s="109"/>
+      <c r="E26" s="109"/>
+      <c r="F26" s="110"/>
+      <c r="H26" s="108"/>
+      <c r="I26" s="109"/>
+      <c r="J26" s="109"/>
+      <c r="K26" s="109"/>
+      <c r="L26" s="110"/>
+      <c r="N26" s="95"/>
+      <c r="O26" s="96"/>
+      <c r="P26" s="96"/>
+      <c r="Q26" s="96"/>
+      <c r="R26" s="97"/>
+      <c r="T26" s="95"/>
+      <c r="U26" s="96"/>
+      <c r="V26" s="96"/>
+      <c r="W26" s="96"/>
+      <c r="X26" s="97"/>
     </row>
     <row r="27" spans="2:24" s="29" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="112"/>
-      <c r="C27" s="113"/>
-      <c r="D27" s="114" t="str">
+      <c r="B27" s="111"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="113" t="str">
         <f>'Cards Src'!$A23</f>
         <v>RECALL</v>
       </c>
-      <c r="E27" s="113"/>
-      <c r="F27" s="115"/>
-      <c r="H27" s="112"/>
-      <c r="I27" s="113"/>
-      <c r="J27" s="114" t="str">
+      <c r="E27" s="112"/>
+      <c r="F27" s="114"/>
+      <c r="H27" s="111"/>
+      <c r="I27" s="112"/>
+      <c r="J27" s="113" t="str">
         <f>'Cards Src'!A24</f>
         <v>GREED</v>
       </c>
-      <c r="K27" s="113"/>
-      <c r="L27" s="115"/>
-      <c r="N27" s="99"/>
-      <c r="O27" s="100"/>
-      <c r="P27" s="101">
+      <c r="K27" s="112"/>
+      <c r="L27" s="114"/>
+      <c r="N27" s="98"/>
+      <c r="O27" s="99"/>
+      <c r="P27" s="100">
         <f>'Cards Src'!A25</f>
         <v>0</v>
       </c>
-      <c r="Q27" s="100"/>
-      <c r="R27" s="102"/>
-      <c r="T27" s="99"/>
-      <c r="U27" s="100"/>
-      <c r="V27" s="101">
+      <c r="Q27" s="99"/>
+      <c r="R27" s="101"/>
+      <c r="T27" s="98"/>
+      <c r="U27" s="99"/>
+      <c r="V27" s="100">
         <f>'Cards Src'!A26</f>
         <v>0</v>
       </c>
-      <c r="W27" s="100"/>
-      <c r="X27" s="102"/>
+      <c r="W27" s="99"/>
+      <c r="X27" s="101"/>
     </row>
     <row r="28" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="116"/>
-      <c r="C28" s="156">
+      <c r="B28" s="115"/>
+      <c r="C28" s="154" t="e" vm="17">
         <f>'Cards Src'!E23</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="156"/>
-      <c r="E28" s="156"/>
-      <c r="F28" s="117"/>
-      <c r="H28" s="116"/>
-      <c r="I28" s="156">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D28" s="154"/>
+      <c r="E28" s="154"/>
+      <c r="F28" s="116"/>
+      <c r="H28" s="115"/>
+      <c r="I28" s="154" t="e" vm="18">
         <f>'Cards Src'!E24</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="156"/>
-      <c r="K28" s="156"/>
-      <c r="L28" s="117"/>
-      <c r="N28" s="103"/>
-      <c r="O28" s="159">
+        <v>#VALUE!</v>
+      </c>
+      <c r="J28" s="154"/>
+      <c r="K28" s="154"/>
+      <c r="L28" s="116"/>
+      <c r="N28" s="102"/>
+      <c r="O28" s="157">
         <f>'Cards Src'!E25</f>
         <v>0</v>
       </c>
-      <c r="P28" s="159"/>
-      <c r="Q28" s="159"/>
-      <c r="R28" s="104"/>
-      <c r="T28" s="103"/>
-      <c r="U28" s="159">
+      <c r="P28" s="157"/>
+      <c r="Q28" s="157"/>
+      <c r="R28" s="103"/>
+      <c r="T28" s="102"/>
+      <c r="U28" s="157">
         <f xml:space="preserve"> 'Cards Src'!E26</f>
         <v>0</v>
       </c>
-      <c r="V28" s="159"/>
-      <c r="W28" s="159"/>
-      <c r="X28" s="104"/>
+      <c r="V28" s="157"/>
+      <c r="W28" s="157"/>
+      <c r="X28" s="103"/>
     </row>
     <row r="29" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="116"/>
-      <c r="C29" s="154" t="str">
+      <c r="B29" s="115"/>
+      <c r="C29" s="152" t="str">
         <f>'Cards Src'!$C23</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D29" s="154"/>
-      <c r="E29" s="154"/>
-      <c r="F29" s="119"/>
-      <c r="H29" s="116"/>
-      <c r="I29" s="154" t="str">
+      <c r="D29" s="152"/>
+      <c r="E29" s="152"/>
+      <c r="F29" s="118"/>
+      <c r="H29" s="115"/>
+      <c r="I29" s="152" t="str">
         <f>'Cards Src'!$C24</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="J29" s="154"/>
-      <c r="K29" s="154"/>
-      <c r="L29" s="119"/>
-      <c r="N29" s="103"/>
-      <c r="O29" s="158">
+      <c r="J29" s="152"/>
+      <c r="K29" s="152"/>
+      <c r="L29" s="118"/>
+      <c r="N29" s="102"/>
+      <c r="O29" s="156">
         <f>'Cards Src'!C25</f>
         <v>0</v>
       </c>
-      <c r="P29" s="158"/>
-      <c r="Q29" s="158"/>
-      <c r="R29" s="105"/>
-      <c r="T29" s="103"/>
-      <c r="U29" s="158">
+      <c r="P29" s="156"/>
+      <c r="Q29" s="156"/>
+      <c r="R29" s="104"/>
+      <c r="T29" s="102"/>
+      <c r="U29" s="156">
         <f>'Cards Src'!C26</f>
         <v>0</v>
       </c>
-      <c r="V29" s="158"/>
-      <c r="W29" s="158"/>
-      <c r="X29" s="105"/>
+      <c r="V29" s="156"/>
+      <c r="W29" s="156"/>
+      <c r="X29" s="104"/>
     </row>
     <row r="30" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="120"/>
-      <c r="C30" s="121"/>
-      <c r="D30" s="121"/>
-      <c r="E30" s="121"/>
-      <c r="F30" s="122"/>
-      <c r="H30" s="120"/>
-      <c r="I30" s="121"/>
-      <c r="J30" s="121"/>
-      <c r="K30" s="121"/>
-      <c r="L30" s="122"/>
-      <c r="N30" s="106"/>
-      <c r="O30" s="107"/>
-      <c r="P30" s="107"/>
-      <c r="Q30" s="107"/>
-      <c r="R30" s="108"/>
-      <c r="T30" s="106"/>
-      <c r="U30" s="107"/>
-      <c r="V30" s="107"/>
-      <c r="W30" s="107"/>
-      <c r="X30" s="108"/>
+      <c r="B30" s="119"/>
+      <c r="C30" s="120"/>
+      <c r="D30" s="120"/>
+      <c r="E30" s="120"/>
+      <c r="F30" s="121"/>
+      <c r="H30" s="119"/>
+      <c r="I30" s="120"/>
+      <c r="J30" s="120"/>
+      <c r="K30" s="120"/>
+      <c r="L30" s="121"/>
+      <c r="N30" s="105"/>
+      <c r="O30" s="106"/>
+      <c r="P30" s="106"/>
+      <c r="Q30" s="106"/>
+      <c r="R30" s="107"/>
+      <c r="T30" s="105"/>
+      <c r="U30" s="106"/>
+      <c r="V30" s="106"/>
+      <c r="W30" s="106"/>
+      <c r="X30" s="107"/>
     </row>
   </sheetData>
   <mergeCells count="40">
@@ -9458,37 +9534,39 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.42578125" customWidth="1"/>
-    <col min="3" max="3" width="55.42578125" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="95"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="55.42578125" style="173" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="169" customWidth="1"/>
     <col min="5" max="5" width="47.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="81" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="29"/>
+      <c r="C1" s="172"/>
       <c r="F1" s="29"/>
     </row>
     <row r="2" spans="1:6" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="e" vm="17">
+      <c r="A2" t="e" vm="19">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" t="e" vm="18">
+      <c r="C2" s="173" t="e" vm="20">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:6" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="171" t="e" vm="19">
+      <c r="A4" s="170" t="e" vm="21">
         <v>#VALUE!</v>
       </c>
-      <c r="C4" s="171" t="e" vm="20">
+      <c r="C4" s="174" t="e" vm="22">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="30" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D5" s="136"/>
+      <c r="C5" s="175"/>
+      <c r="D5" s="171"/>
     </row>
     <row r="6" spans="1:6" s="32" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
@@ -9497,13 +9575,13 @@
       <c r="B6" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="176" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="137" t="s">
+      <c r="E6" s="135" t="s">
         <v>17</v>
       </c>
     </row>
@@ -9514,13 +9592,13 @@
       <c r="B7" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="177" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="137" t="s">
+      <c r="D7" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="32" t="e" vm="21">
+      <c r="E7" s="32" t="e" vm="23">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9531,13 +9609,13 @@
       <c r="B8" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="177" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="137" t="s">
+      <c r="D8" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="42" t="e" vm="22">
+      <c r="E8" s="42" t="e" vm="24">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9548,13 +9626,13 @@
       <c r="B9" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="C9" s="177" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="137" t="s">
+      <c r="D9" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="42" t="e" vm="23">
+      <c r="E9" s="42" t="e" vm="25">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9565,13 +9643,13 @@
       <c r="B10" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="42" t="s">
+      <c r="C10" s="177" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="137" t="s">
+      <c r="D10" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="42" t="e" vm="24">
+      <c r="E10" s="42" t="e" vm="26">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9582,13 +9660,13 @@
       <c r="B11" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="177" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="137" t="s">
+      <c r="D11" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="42" t="e" vm="25">
+      <c r="E11" s="42" t="e" vm="27">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9599,13 +9677,13 @@
       <c r="B12" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="C12" s="177" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="137" t="s">
+      <c r="D12" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="42" t="e" vm="26">
+      <c r="E12" s="42" t="e" vm="28">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9616,13 +9694,13 @@
       <c r="B13" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="177" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="137" t="s">
+      <c r="D13" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="42" t="e" vm="27">
+      <c r="E13" s="42" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9633,13 +9711,13 @@
       <c r="B14" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="42" t="s">
+      <c r="C14" s="177" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="137" t="s">
+      <c r="D14" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="E14" s="42" t="e" vm="28">
+      <c r="E14" s="42" t="e" vm="30">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9650,13 +9728,13 @@
       <c r="B15" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="177" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="137" t="s">
+      <c r="D15" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="42" t="e" vm="29">
+      <c r="E15" s="42" t="e" vm="31">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9667,13 +9745,13 @@
       <c r="B16" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="42" t="s">
+      <c r="C16" s="177" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="137" t="s">
+      <c r="D16" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="42" t="e" vm="30">
+      <c r="E16" s="42" t="e" vm="32">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9684,13 +9762,13 @@
       <c r="B17" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="42" t="s">
+      <c r="C17" s="177" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="137" t="s">
+      <c r="D17" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="42" t="e" vm="31">
+      <c r="E17" s="42" t="e" vm="33">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9701,13 +9779,13 @@
       <c r="B18" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="42" t="s">
+      <c r="C18" s="177" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="137" t="s">
+      <c r="D18" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="42" t="e" vm="32">
+      <c r="E18" s="42" t="e" vm="34">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9718,13 +9796,13 @@
       <c r="B19" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="42" t="s">
+      <c r="C19" s="177" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="137" t="s">
+      <c r="D19" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="42" t="e" vm="33">
+      <c r="E19" s="42" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9735,13 +9813,13 @@
       <c r="B20" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="42" t="s">
+      <c r="C20" s="177" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="137" t="s">
+      <c r="D20" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="42" t="e" vm="34">
+      <c r="E20" s="42" t="e" vm="36">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9752,13 +9830,13 @@
       <c r="B21" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="42" t="s">
+      <c r="C21" s="177" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="137" t="s">
+      <c r="D21" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="42" t="e" vm="35">
+      <c r="E21" s="42" t="e" vm="37">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9769,13 +9847,13 @@
       <c r="B22" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="42" t="s">
+      <c r="C22" s="177" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="137" t="s">
+      <c r="D22" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="42" t="e" vm="36">
+      <c r="E22" s="42" t="e" vm="38">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9786,11 +9864,14 @@
       <c r="B23" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C23" s="42" t="s">
+      <c r="C23" s="177" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="137" t="s">
+      <c r="D23" s="42" t="s">
         <v>46</v>
+      </c>
+      <c r="E23" s="42" t="e" vm="39">
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="42" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
@@ -9800,42 +9881,30 @@
       <c r="B24" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="42" t="s">
+      <c r="C24" s="177" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="137" t="s">
+      <c r="D24" s="42" t="s">
         <v>46</v>
+      </c>
+      <c r="E24" s="42" t="e" vm="40">
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="42" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="137"/>
+      <c r="C25" s="177"/>
     </row>
     <row r="26" spans="1:5" s="42" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="137"/>
+      <c r="C26" s="177"/>
     </row>
     <row r="27" spans="1:5" s="42" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="137"/>
+      <c r="C27" s="177"/>
     </row>
     <row r="28" spans="1:5" s="42" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" s="137"/>
+      <c r="C28" s="177"/>
     </row>
     <row r="29" spans="1:5" s="42" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="137"/>
+      <c r="C29" s="177"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9857,31 +9926,31 @@
       <c r="A2" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="B2" t="e" vm="37">
+      <c r="B2" t="e" vm="41">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" t="e" vm="38">
+      <c r="C2" t="e" vm="42">
         <v>#VALUE!</v>
       </c>
-      <c r="D2" t="e" vm="39">
+      <c r="D2" t="e" vm="43">
         <v>#VALUE!</v>
       </c>
-      <c r="E2" t="e" vm="40">
+      <c r="E2" t="e" vm="44">
         <v>#VALUE!</v>
       </c>
-      <c r="F2" t="e" vm="41">
+      <c r="F2" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
-      <c r="G2" t="e" vm="42">
+      <c r="G2" t="e" vm="46">
         <v>#VALUE!</v>
       </c>
-      <c r="H2" t="e" vm="43">
+      <c r="H2" t="e" vm="47">
         <v>#VALUE!</v>
       </c>
-      <c r="I2" t="e" vm="44">
+      <c r="I2" t="e" vm="48">
         <v>#VALUE!</v>
       </c>
-      <c r="J2" t="e" vm="45">
+      <c r="J2" t="e" vm="49">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -9922,7 +9991,7 @@
     <row r="3" spans="3:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="165"/>
+      <c r="E3" s="163"/>
       <c r="F3" s="2"/>
       <c r="G3" s="3"/>
       <c r="K3" s="1"/>
@@ -9933,62 +10002,62 @@
     </row>
     <row r="4" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="4"/>
-      <c r="D4" s="160"/>
-      <c r="E4" s="166"/>
-      <c r="F4" s="160"/>
+      <c r="D4" s="158"/>
+      <c r="E4" s="164"/>
+      <c r="F4" s="158"/>
       <c r="G4" s="5"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="160"/>
+      <c r="L4" s="158"/>
       <c r="M4" s="8"/>
-      <c r="N4" s="160"/>
+      <c r="N4" s="158"/>
       <c r="O4" s="5"/>
     </row>
     <row r="5" spans="3:15" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="4"/>
-      <c r="D5" s="160"/>
-      <c r="E5" s="166"/>
-      <c r="F5" s="160"/>
+      <c r="D5" s="158"/>
+      <c r="E5" s="164"/>
+      <c r="F5" s="158"/>
       <c r="G5" s="5"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="160"/>
+      <c r="L5" s="158"/>
       <c r="M5" s="8"/>
-      <c r="N5" s="160"/>
+      <c r="N5" s="158"/>
       <c r="O5" s="5"/>
     </row>
     <row r="6" spans="3:15" ht="288" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C6" s="4"/>
-      <c r="D6" s="162"/>
-      <c r="E6" s="162"/>
-      <c r="F6" s="162"/>
+      <c r="D6" s="160"/>
+      <c r="E6" s="160"/>
+      <c r="F6" s="160"/>
       <c r="G6" s="5"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="167"/>
-      <c r="M6" s="168"/>
-      <c r="N6" s="169"/>
+      <c r="L6" s="165"/>
+      <c r="M6" s="166"/>
+      <c r="N6" s="167"/>
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="3:15" ht="169.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="4"/>
-      <c r="D7" s="163"/>
-      <c r="E7" s="163"/>
-      <c r="F7" s="163"/>
-      <c r="G7" s="164"/>
+      <c r="D7" s="161"/>
+      <c r="E7" s="161"/>
+      <c r="F7" s="161"/>
+      <c r="G7" s="162"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="170"/>
-      <c r="M7" s="170"/>
-      <c r="N7" s="170"/>
+      <c r="L7" s="168"/>
+      <c r="M7" s="168"/>
+      <c r="N7" s="168"/>
       <c r="O7" s="5"/>
     </row>
     <row r="8" spans="3:15" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="6"/>
-      <c r="D8" s="161"/>
-      <c r="E8" s="161"/>
-      <c r="F8" s="161"/>
+      <c r="D8" s="159"/>
+      <c r="E8" s="159"/>
+      <c r="F8" s="159"/>
       <c r="G8" s="7"/>
       <c r="K8" s="6"/>
-      <c r="L8" s="161"/>
-      <c r="M8" s="161"/>
-      <c r="N8" s="161"/>
+      <c r="L8" s="159"/>
+      <c r="M8" s="159"/>
+      <c r="N8" s="159"/>
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="3:15" ht="10.15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Art - Frost Nova + border re-tool
Added card art for Frost Nova; changed card sourcing so art comes with inner border attached, and then full card border is separate
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1C881A-6E42-4009-9871-D25753DAAC56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA735DA-EE75-42FD-9D85-576C46CCECC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="15" r:id="rId1"/>
@@ -1188,7 +1188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1478,6 +1478,69 @@
     <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1501,73 +1564,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1604,6 +1600,982 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="56" name="Picture 55">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6643A80E-1E86-43F0-A209-C1D50216F722}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="609600" y="16287750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="57" name="Picture 56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6E4D18E-8A8E-450E-9786-783FDD5E9176}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4914900" y="16287750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="58" name="Picture 57">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37A6EFF8-4851-4285-81EF-A040AC6311C1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9220200" y="16287750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="59" name="Picture 58">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1184FE64-8B56-433D-BBF5-2BB9046EEC7B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13525500" y="16287750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="60" name="Picture 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1E8C2D1-BE90-4701-A257-39737621BDF1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="609600" y="21650325"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="61" name="Picture 60">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94E4EFA5-2E34-4FC3-8A05-36E8EAB45292}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4914900" y="21650325"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="54" name="Picture 53">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA45D086-D230-4AA1-9245-BE67E5F173D0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13525500" y="10925175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="53" name="Picture 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3EF0721-4DDE-4F40-987C-1C816DC4241E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9220200" y="10925175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="52" name="Picture 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7DAF7DC-C28D-B648-A1F5-9051912EDC0A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4914900" y="10925175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="47" name="Picture 46">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49043CFD-EA61-4065-882F-869A50F62868}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="609600" y="10925175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="46" name="Picture 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0BCCACA-3FFB-42EA-85C5-1F7808814533}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13525500" y="5562600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="45" name="Picture 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5541008-5B1A-4E98-9BF9-323D3A316D73}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9220200" y="5562600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="44" name="Picture 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3CA5460E-7BB0-46BB-A7D2-173FA277090E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4914900" y="5562600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="43" name="Picture 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E43082E8-05A2-42EC-96D7-B4898EC02DC5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="609600" y="5562600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="42" name="Picture 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E44C4CD6-3A14-456D-8EA3-7EB195BCAAF3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13525500" y="200025"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="40" name="Picture 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12768679-C79D-4B7B-8101-1BA455F1D492}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9220200" y="200025"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
@@ -1611,37 +2583,54 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>9525</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="41" name="Picture 40">
+        <xdr:cNvPr id="37" name="Picture 36">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{40A2F210-53DF-4CA9-8A4F-A28D51BA16D9}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC10B69C-B64B-489A-B4BC-2C910640F2C0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
           <a:off x="4914900" y="200025"/>
-          <a:ext cx="3695700" cy="4991100"/>
+          <a:ext cx="3705225" cy="5000625"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1655,916 +2644,58 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>9525</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="71" name="Picture 70">
+        <xdr:cNvPr id="31" name="Picture 30">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE3B254A-05A6-48FC-B070-5BFC034133FD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DED3668-45A2-22A6-F40E-B93BA0C28FB8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
           <a:off x="609600" y="200025"/>
-          <a:ext cx="3695700" cy="4991100"/>
+          <a:ext cx="3705225" cy="5000625"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
-        <xdr:from>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>1</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:ext cx="3705225" cy="5000625"/>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="18" name="Picture 17">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55B11F5E-763A-404B-B231-BB497A0C6281}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16577"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="200025"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:oneCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
-        <xdr:from>
-          <xdr:col>19</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>1</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:ext cx="3705225" cy="5000625"/>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="19" name="Picture 18">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3316334-D9FF-41B1-89B8-D994EF00B359}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16578"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="13525500" y="200025"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:oneCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
-        <xdr:from>
-          <xdr:col>19</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:ext cx="3705225" cy="5000625"/>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="20" name="Picture 19">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BFE5DA9D-2717-4BAA-AACB-A77E3AF34F35}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16579"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="13525500" y="5562600"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:oneCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
-        <xdr:from>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:ext cx="3705225" cy="5000625"/>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="21" name="Picture 20">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4EF40632-C9BA-40AC-93A9-93ED92891B60}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16580"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="5562600"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:oneCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
-        <xdr:from>
-          <xdr:col>7</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:ext cx="3705225" cy="5000625"/>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="22" name="Picture 21">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35BBB72F-5133-4BDD-B5F7-4F69820251BE}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16581"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="5562600"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:oneCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:ext cx="3705225" cy="5000625"/>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="23" name="Picture 22">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{76D65C39-E8FB-4AB3-815E-7F6DDA656958}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16582"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="5562600"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:oneCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:oneCellAnchor>
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:ext cx="3705225" cy="5000625"/>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="24" name="Picture 23">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6FB6548D-FFE1-40A8-8546-811979858E52}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16583"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="10925175"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:oneCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>7</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>12</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>18</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="3" name="Picture 2">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBBF2DB2-FBBD-E209-1034-87EB6702CE75}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16584"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="10925175"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>18</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>18</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="4" name="Picture 3">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F71B6122-5D31-4279-8B77-2525453DE722}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16585"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="10925175"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>19</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>24</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>18</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="5" name="Picture 4">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F4A0A05-EAEB-43E7-926C-D1ED54F0F978}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16586"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="13525500" y="10925175"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>6</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>24</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="6" name="Picture 5">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48E4F5A0-DF6D-48FD-BB66-DAC83E81E077}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16587"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="16287750"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>7</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>12</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>24</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="7" name="Picture 6">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26158A2E-0158-4E51-8F64-6A048A099696}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16588"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="16287750"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>18</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>24</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="8" name="Picture 7">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06B5C7DE-6CFA-4958-94FC-DC4C415E193B}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16589"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="16287750"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>19</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>24</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>24</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="9" name="Picture 8">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79D01B02-5DCA-4108-8783-A59C268AEE8B}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16590"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="13525500" y="16287750"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
@@ -2593,13 +2724,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16591"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16683"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -2658,13 +2789,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16592"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16684"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -2723,13 +2854,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16593"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16685"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -2788,13 +2919,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16594"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16686"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -2853,13 +2984,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16595"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16687"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -2918,13 +3049,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16596"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16688"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -2983,13 +3114,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16597"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16689"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3048,13 +3179,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16598"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16690"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3113,13 +3244,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16599"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16691"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3178,13 +3309,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16600"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16692"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3243,13 +3374,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16601"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16693"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3308,13 +3439,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16602"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16694"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3373,13 +3504,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16603"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16695"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3438,13 +3569,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16604"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16696"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3503,13 +3634,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16605"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16697"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3567,7 +3698,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3584,136 +3715,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>25</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>6</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>30</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="16" name="Picture 15">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{424869C4-9B51-4F72-BD92-76BDFE2D4B79}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16606"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="21650325"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>7</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>25</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>12</xdr:col>
-          <xdr:colOff>9525</xdr:colOff>
-          <xdr:row>30</xdr:row>
-          <xdr:rowOff>19050</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="27" name="Picture 26">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{957F9E96-7DD7-48A2-94DF-BEBAB69F7817}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16607"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="21650325"/>
-              <a:ext cx="3705225" cy="5000625"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
@@ -3742,13 +3743,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16608"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16698"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3807,13 +3808,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16609"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16699"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -4583,70 +4584,70 @@
     </row>
     <row r="4" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
-      <c r="C4" s="129" t="e" vm="1">
+      <c r="C4" s="150" t="e" vm="1">
         <f>'Cards Src'!E2</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="129"/>
-      <c r="E4" s="129"/>
+      <c r="D4" s="150"/>
+      <c r="E4" s="150"/>
       <c r="F4" s="42"/>
       <c r="H4" s="53"/>
-      <c r="I4" s="134" t="e" vm="2">
+      <c r="I4" s="155" t="e" vm="2">
         <f>'Cards Src'!E3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J4" s="134"/>
-      <c r="K4" s="134"/>
+      <c r="J4" s="155"/>
+      <c r="K4" s="155"/>
       <c r="L4" s="54"/>
       <c r="N4" s="116"/>
-      <c r="O4" s="135" t="e" vm="3">
+      <c r="O4" s="156" t="e" vm="3">
         <f>'Cards Src'!E4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P4" s="135"/>
-      <c r="Q4" s="135"/>
+      <c r="P4" s="156"/>
+      <c r="Q4" s="156"/>
       <c r="R4" s="64"/>
       <c r="T4" s="7"/>
-      <c r="U4" s="136" t="e" vm="4">
+      <c r="U4" s="157" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V4" s="136"/>
-      <c r="W4" s="136"/>
+      <c r="V4" s="157"/>
+      <c r="W4" s="157"/>
       <c r="X4" s="29"/>
     </row>
     <row r="5" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
-      <c r="C5" s="130" t="str">
+      <c r="C5" s="151" t="str">
         <f>'Cards Src'!$C2</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="130"/>
-      <c r="E5" s="130"/>
+      <c r="D5" s="151"/>
+      <c r="E5" s="151"/>
       <c r="F5" s="43"/>
       <c r="H5" s="53"/>
-      <c r="I5" s="131" t="str">
+      <c r="I5" s="152" t="str">
         <f>'Cards Src'!$C3</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="J5" s="131"/>
-      <c r="K5" s="131"/>
+      <c r="J5" s="152"/>
+      <c r="K5" s="152"/>
       <c r="L5" s="55"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="132" t="str">
+      <c r="O5" s="153" t="str">
         <f>'Cards Src'!C4</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="P5" s="132"/>
-      <c r="Q5" s="132"/>
+      <c r="P5" s="153"/>
+      <c r="Q5" s="153"/>
       <c r="R5" s="65"/>
       <c r="T5" s="7"/>
-      <c r="U5" s="133" t="str">
+      <c r="U5" s="154" t="str">
         <f>'Cards Src'!C5</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="V5" s="133"/>
-      <c r="W5" s="133"/>
+      <c r="V5" s="154"/>
+      <c r="W5" s="154"/>
       <c r="X5" s="30"/>
     </row>
     <row r="6" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4730,20 +4731,20 @@
     </row>
     <row r="10" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="11"/>
-      <c r="C10" s="137" t="e" vm="5">
+      <c r="C10" s="145" t="e" vm="5">
         <f>'Cards Src'!E6</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D10" s="137"/>
-      <c r="E10" s="137"/>
+      <c r="D10" s="145"/>
+      <c r="E10" s="145"/>
       <c r="F10" s="126"/>
       <c r="H10" s="15"/>
-      <c r="I10" s="141" t="e" vm="6">
+      <c r="I10" s="149" t="e" vm="6">
         <f>'Cards Src'!E7</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J10" s="141"/>
-      <c r="K10" s="141"/>
+      <c r="J10" s="149"/>
+      <c r="K10" s="149"/>
       <c r="L10" s="72"/>
       <c r="N10" s="19"/>
       <c r="O10" s="142" t="e" vm="7">
@@ -4754,46 +4755,46 @@
       <c r="Q10" s="142"/>
       <c r="R10" s="81"/>
       <c r="T10" s="11"/>
-      <c r="U10" s="137" t="e" vm="8">
+      <c r="U10" s="145" t="e" vm="8">
         <f>'Cards Src'!E9</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V10" s="137"/>
-      <c r="W10" s="137"/>
+      <c r="V10" s="145"/>
+      <c r="W10" s="145"/>
       <c r="X10" s="122"/>
     </row>
     <row r="11" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="11"/>
-      <c r="C11" s="138" t="str">
+      <c r="C11" s="146" t="str">
         <f>'Cards Src'!$C6</f>
         <v>Casts a bolt of lightning</v>
       </c>
-      <c r="D11" s="138"/>
-      <c r="E11" s="138"/>
+      <c r="D11" s="146"/>
+      <c r="E11" s="146"/>
       <c r="F11" s="123"/>
       <c r="H11" s="15"/>
-      <c r="I11" s="139" t="str">
+      <c r="I11" s="147" t="str">
         <f>'Cards Src'!$C7</f>
         <v>Vacuums in nearby enemies</v>
       </c>
-      <c r="J11" s="139"/>
-      <c r="K11" s="139"/>
+      <c r="J11" s="147"/>
+      <c r="K11" s="147"/>
       <c r="L11" s="73"/>
       <c r="N11" s="19"/>
-      <c r="O11" s="140" t="str">
+      <c r="O11" s="148" t="str">
         <f>'Cards Src'!C8</f>
         <v>Flies to the nearest enemy in vision</v>
       </c>
-      <c r="P11" s="140"/>
-      <c r="Q11" s="140"/>
+      <c r="P11" s="148"/>
+      <c r="Q11" s="148"/>
       <c r="R11" s="82"/>
       <c r="T11" s="11"/>
-      <c r="U11" s="138" t="str">
+      <c r="U11" s="146" t="str">
         <f>'Cards Src'!C9</f>
         <v>Casts a tracking bolt of lightning that can chain to close enemies</v>
       </c>
-      <c r="V11" s="138"/>
-      <c r="W11" s="138"/>
+      <c r="V11" s="146"/>
+      <c r="W11" s="146"/>
       <c r="X11" s="123"/>
     </row>
     <row r="12" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4885,28 +4886,28 @@
       <c r="E16" s="142"/>
       <c r="F16" s="81"/>
       <c r="H16" s="107"/>
-      <c r="I16" s="145" t="e" vm="10">
+      <c r="I16" s="144" t="e" vm="10">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J16" s="145"/>
-      <c r="K16" s="145"/>
+      <c r="J16" s="144"/>
+      <c r="K16" s="144"/>
       <c r="L16" s="108"/>
       <c r="N16" s="107"/>
-      <c r="O16" s="146" t="e" vm="11">
+      <c r="O16" s="137" t="e" vm="11">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P16" s="146"/>
-      <c r="Q16" s="146"/>
+      <c r="P16" s="137"/>
+      <c r="Q16" s="137"/>
       <c r="R16" s="108"/>
       <c r="T16" s="107"/>
-      <c r="U16" s="146" t="e" vm="12">
+      <c r="U16" s="137" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V16" s="146"/>
-      <c r="W16" s="146"/>
+      <c r="V16" s="137"/>
+      <c r="W16" s="137"/>
       <c r="X16" s="108"/>
     </row>
     <row r="17" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
@@ -4919,28 +4920,28 @@
       <c r="E17" s="143"/>
       <c r="F17" s="82"/>
       <c r="H17" s="107"/>
-      <c r="I17" s="144" t="str">
+      <c r="I17" s="138" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="J17" s="144"/>
-      <c r="K17" s="144"/>
+      <c r="J17" s="138"/>
+      <c r="K17" s="138"/>
       <c r="L17" s="110"/>
       <c r="N17" s="107"/>
-      <c r="O17" s="144" t="str">
+      <c r="O17" s="138" t="str">
         <f>'Cards Src'!C12</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="P17" s="144"/>
-      <c r="Q17" s="144"/>
+      <c r="P17" s="138"/>
+      <c r="Q17" s="138"/>
       <c r="R17" s="110"/>
       <c r="T17" s="107"/>
-      <c r="U17" s="144" t="str">
+      <c r="U17" s="138" t="str">
         <f>'Cards Src'!C13</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="V17" s="144"/>
-      <c r="W17" s="144"/>
+      <c r="V17" s="138"/>
+      <c r="W17" s="138"/>
       <c r="X17" s="110"/>
     </row>
     <row r="18" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5024,70 +5025,70 @@
     </row>
     <row r="22" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="107"/>
-      <c r="C22" s="146" t="e" vm="13">
+      <c r="C22" s="137" t="e" vm="13">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D22" s="146"/>
-      <c r="E22" s="146"/>
+      <c r="D22" s="137"/>
+      <c r="E22" s="137"/>
       <c r="F22" s="108"/>
       <c r="H22" s="107"/>
-      <c r="I22" s="146" t="e" vm="14">
+      <c r="I22" s="137" t="e" vm="14">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J22" s="146"/>
-      <c r="K22" s="146"/>
+      <c r="J22" s="137"/>
+      <c r="K22" s="137"/>
       <c r="L22" s="108"/>
       <c r="N22" s="107"/>
-      <c r="O22" s="146" t="e" vm="15">
+      <c r="O22" s="137" t="e" vm="15">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P22" s="146"/>
-      <c r="Q22" s="146"/>
+      <c r="P22" s="137"/>
+      <c r="Q22" s="137"/>
       <c r="R22" s="108"/>
       <c r="T22" s="107"/>
-      <c r="U22" s="146" t="e" vm="16">
+      <c r="U22" s="137" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V22" s="146"/>
-      <c r="W22" s="146"/>
+      <c r="V22" s="137"/>
+      <c r="W22" s="137"/>
       <c r="X22" s="108"/>
     </row>
     <row r="23" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="107"/>
-      <c r="C23" s="144" t="str">
+      <c r="C23" s="138" t="str">
         <f>'Cards Src'!$C14</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D23" s="144"/>
-      <c r="E23" s="144"/>
+      <c r="D23" s="138"/>
+      <c r="E23" s="138"/>
       <c r="F23" s="110"/>
       <c r="H23" s="107"/>
-      <c r="I23" s="144" t="str">
+      <c r="I23" s="138" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="J23" s="144"/>
-      <c r="K23" s="144"/>
+      <c r="J23" s="138"/>
+      <c r="K23" s="138"/>
       <c r="L23" s="110"/>
       <c r="N23" s="107"/>
-      <c r="O23" s="147" t="str">
+      <c r="O23" s="141" t="str">
         <f>'Cards Src'!C16</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="P23" s="147"/>
-      <c r="Q23" s="147"/>
+      <c r="P23" s="141"/>
+      <c r="Q23" s="141"/>
       <c r="R23" s="110"/>
       <c r="T23" s="107"/>
-      <c r="U23" s="144" t="str">
+      <c r="U23" s="138" t="str">
         <f>'Cards Src'!C17</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="V23" s="144"/>
-      <c r="W23" s="144"/>
+      <c r="V23" s="138"/>
+      <c r="W23" s="138"/>
       <c r="X23" s="110"/>
     </row>
     <row r="24" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5171,70 +5172,70 @@
     </row>
     <row r="28" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="107"/>
-      <c r="C28" s="146" t="e" vm="17">
+      <c r="C28" s="137" t="e" vm="17">
         <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D28" s="146"/>
-      <c r="E28" s="146"/>
+      <c r="D28" s="137"/>
+      <c r="E28" s="137"/>
       <c r="F28" s="108"/>
       <c r="H28" s="107"/>
-      <c r="I28" s="146" t="e" vm="18">
+      <c r="I28" s="137" t="e" vm="18">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J28" s="146"/>
-      <c r="K28" s="146"/>
+      <c r="J28" s="137"/>
+      <c r="K28" s="137"/>
       <c r="L28" s="108"/>
       <c r="N28" s="94"/>
-      <c r="O28" s="149">
+      <c r="O28" s="140">
         <f>'Cards Src'!E20</f>
         <v>0</v>
       </c>
-      <c r="P28" s="149"/>
-      <c r="Q28" s="149"/>
+      <c r="P28" s="140"/>
+      <c r="Q28" s="140"/>
       <c r="R28" s="95"/>
       <c r="T28" s="94"/>
-      <c r="U28" s="149">
+      <c r="U28" s="140">
         <f xml:space="preserve"> 'Cards Src'!E21</f>
         <v>0</v>
       </c>
-      <c r="V28" s="149"/>
-      <c r="W28" s="149"/>
+      <c r="V28" s="140"/>
+      <c r="W28" s="140"/>
       <c r="X28" s="95"/>
     </row>
     <row r="29" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="107"/>
-      <c r="C29" s="144" t="str">
+      <c r="C29" s="138" t="str">
         <f>'Cards Src'!$C18</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D29" s="144"/>
-      <c r="E29" s="144"/>
+      <c r="D29" s="138"/>
+      <c r="E29" s="138"/>
       <c r="F29" s="110"/>
       <c r="H29" s="107"/>
-      <c r="I29" s="144" t="str">
+      <c r="I29" s="138" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="J29" s="144"/>
-      <c r="K29" s="144"/>
+      <c r="J29" s="138"/>
+      <c r="K29" s="138"/>
       <c r="L29" s="110"/>
       <c r="N29" s="94"/>
-      <c r="O29" s="148">
+      <c r="O29" s="139">
         <f>'Cards Src'!C20</f>
         <v>0</v>
       </c>
-      <c r="P29" s="148"/>
-      <c r="Q29" s="148"/>
+      <c r="P29" s="139"/>
+      <c r="Q29" s="139"/>
       <c r="R29" s="96"/>
       <c r="T29" s="94"/>
-      <c r="U29" s="148">
+      <c r="U29" s="139">
         <f>'Cards Src'!C21</f>
         <v>0</v>
       </c>
-      <c r="V29" s="148"/>
-      <c r="W29" s="148"/>
+      <c r="V29" s="139"/>
+      <c r="W29" s="139"/>
       <c r="X29" s="96"/>
     </row>
     <row r="30" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5261,6 +5262,38 @@
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="U5:W5"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="U4:W4"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="U10:W10"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="O17:Q17"/>
+    <mergeCell ref="U17:W17"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="U16:W16"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="O23:Q23"/>
+    <mergeCell ref="U23:W23"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="U22:W22"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="C29:E29"/>
     <mergeCell ref="I29:K29"/>
@@ -5269,38 +5302,6 @@
     <mergeCell ref="I28:K28"/>
     <mergeCell ref="O28:Q28"/>
     <mergeCell ref="U28:W28"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="U23:W23"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="U22:W22"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="U17:W17"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="U16:W16"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="O11:Q11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="U10:W10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="U5:W5"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="U4:W4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5319,8 +5320,8 @@
   <cols>
     <col min="1" max="1" width="55.42578125" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="55.42578125" style="153" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="150" customWidth="1"/>
+    <col min="3" max="3" width="55.42578125" style="131" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="129" customWidth="1"/>
     <col min="5" max="5" width="47.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5331,7 +5332,7 @@
       <c r="B1" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="156" t="s">
+      <c r="C1" s="133" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="34" t="s">
@@ -5348,7 +5349,7 @@
       <c r="B2" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="157" t="s">
+      <c r="C2" s="134" t="s">
         <v>20</v>
       </c>
       <c r="D2" s="34" t="s">
@@ -5365,7 +5366,7 @@
       <c r="B3" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="157" t="s">
+      <c r="C3" s="134" t="s">
         <v>21</v>
       </c>
       <c r="D3" s="34" t="s">
@@ -5382,7 +5383,7 @@
       <c r="B4" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="157" t="s">
+      <c r="C4" s="134" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="34" t="s">
@@ -5399,7 +5400,7 @@
       <c r="B5" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="157" t="s">
+      <c r="C5" s="134" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="34" t="s">
@@ -5416,7 +5417,7 @@
       <c r="B6" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="157" t="s">
+      <c r="C6" s="134" t="s">
         <v>29</v>
       </c>
       <c r="D6" s="34" t="s">
@@ -5433,7 +5434,7 @@
       <c r="B7" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="157" t="s">
+      <c r="C7" s="134" t="s">
         <v>30</v>
       </c>
       <c r="D7" s="34" t="s">
@@ -5450,7 +5451,7 @@
       <c r="B8" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="157" t="s">
+      <c r="C8" s="134" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="34" t="s">
@@ -5467,7 +5468,7 @@
       <c r="B9" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="157" t="s">
+      <c r="C9" s="134" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="34" t="s">
@@ -5484,7 +5485,7 @@
       <c r="B10" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="157" t="s">
+      <c r="C10" s="134" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="34" t="s">
@@ -5501,7 +5502,7 @@
       <c r="B11" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="157" t="s">
+      <c r="C11" s="134" t="s">
         <v>39</v>
       </c>
       <c r="D11" s="34" t="s">
@@ -5518,7 +5519,7 @@
       <c r="B12" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="157" t="s">
+      <c r="C12" s="134" t="s">
         <v>40</v>
       </c>
       <c r="D12" s="34" t="s">
@@ -5535,7 +5536,7 @@
       <c r="B13" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="157" t="s">
+      <c r="C13" s="134" t="s">
         <v>41</v>
       </c>
       <c r="D13" s="34" t="s">
@@ -5552,7 +5553,7 @@
       <c r="B14" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="157" t="s">
+      <c r="C14" s="134" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="34" t="s">
@@ -5569,7 +5570,7 @@
       <c r="B15" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="157" t="s">
+      <c r="C15" s="134" t="s">
         <v>43</v>
       </c>
       <c r="D15" s="34" t="s">
@@ -5586,7 +5587,7 @@
       <c r="B16" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="157" t="s">
+      <c r="C16" s="134" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="34" t="s">
@@ -5603,7 +5604,7 @@
       <c r="B17" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="157" t="s">
+      <c r="C17" s="134" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="34" t="s">
@@ -5620,7 +5621,7 @@
       <c r="B18" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="157" t="s">
+      <c r="C18" s="134" t="s">
         <v>51</v>
       </c>
       <c r="D18" s="34" t="s">
@@ -5637,7 +5638,7 @@
       <c r="B19" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="157" t="s">
+      <c r="C19" s="134" t="s">
         <v>52</v>
       </c>
       <c r="D19" s="34" t="s">
@@ -5648,19 +5649,19 @@
       </c>
     </row>
     <row r="20" spans="1:5" s="34" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="157"/>
+      <c r="C20" s="134"/>
     </row>
     <row r="21" spans="1:5" s="34" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="157"/>
+      <c r="C21" s="134"/>
     </row>
     <row r="22" spans="1:5" s="34" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="157"/>
+      <c r="C22" s="134"/>
     </row>
     <row r="23" spans="1:5" s="34" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="157"/>
+      <c r="C23" s="134"/>
     </row>
     <row r="24" spans="1:5" s="34" customFormat="1" ht="186" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="157"/>
+      <c r="C24" s="134"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5771,32 +5772,32 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="155" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="B6" s="158" t="s">
+    <row r="6" spans="1:10" s="132" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="135" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="159" t="s">
+      <c r="C6" s="136" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="159" t="s">
+      <c r="D6" s="136" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="159" t="s">
+      <c r="E6" s="136" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="159" t="s">
+      <c r="F6" s="136" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="159" t="s">
+      <c r="G6" s="136" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="159" t="s">
+      <c r="H6" s="136" t="s">
         <v>16</v>
       </c>
-      <c r="I6" s="159" t="s">
+      <c r="I6" s="136" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="159" t="s">
+      <c r="J6" s="136" t="s">
         <v>28</v>
       </c>
     </row>
@@ -5832,32 +5833,32 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="155" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="B9" s="159" t="s">
+    <row r="9" spans="1:10" s="132" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="136" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="159" t="s">
+      <c r="C9" s="136" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="159" t="s">
+      <c r="D9" s="136" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="159" t="s">
+      <c r="E9" s="136" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="159" t="s">
+      <c r="F9" s="136" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="159" t="s">
+      <c r="G9" s="136" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="159" t="s">
+      <c r="H9" s="136" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="159" t="s">
+      <c r="I9" s="136" t="s">
         <v>49</v>
       </c>
-      <c r="J9" s="159" t="s">
+      <c r="J9" s="136" t="s">
         <v>50</v>
       </c>
     </row>
@@ -5876,21 +5877,21 @@
   <cols>
     <col min="1" max="1" width="55.42578125" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="55.42578125" style="153" customWidth="1"/>
+    <col min="3" max="3" width="55.42578125" style="131" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="152"/>
+      <c r="C1" s="130"/>
       <c r="D1" s="21"/>
     </row>
     <row r="2" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="e" vm="64">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="153" t="e" vm="65">
+      <c r="C2" s="131" t="e" vm="65">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -5898,14 +5899,14 @@
       <c r="A3" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="152"/>
+      <c r="C3" s="130"/>
       <c r="D3" s="21"/>
     </row>
     <row r="4" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="e" vm="66">
         <v>#VALUE!</v>
       </c>
-      <c r="C4" s="153" t="e" vm="67">
+      <c r="C4" s="131" t="e" vm="67">
         <v>#VALUE!</v>
       </c>
     </row>
@@ -5913,14 +5914,14 @@
       <c r="A5" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="152"/>
+      <c r="C5" s="130"/>
       <c r="D5" s="21"/>
     </row>
     <row r="6" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="151" t="e" vm="68">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C6" s="154" t="e" vm="69">
+      <c r="A6" t="e" vm="68">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C6" s="131" t="e" vm="69">
         <v>#VALUE!</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Art - Astral Dagger
Added Astral Dagger attack card art
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E009630-33D3-48EC-B42E-2C28DA2C7D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEAC17BA-D342-4EF2-9BFE-C75B0AEECD0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1502,67 +1502,67 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2724,7 +2724,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16735"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16752"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2789,7 +2789,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16736"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16753"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2854,7 +2854,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16737"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16754"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2919,7 +2919,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16738"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16755"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2984,7 +2984,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16739"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16756"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3049,7 +3049,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16740"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16757"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3114,7 +3114,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16741"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16758"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3179,7 +3179,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16742"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16759"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3244,7 +3244,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16743"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16760"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3309,7 +3309,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16744"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16761"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3374,7 +3374,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16745"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16762"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3439,7 +3439,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16746"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16763"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3504,7 +3504,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16747"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16764"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3569,7 +3569,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16748"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16765"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3634,7 +3634,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16749"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16766"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3743,7 +3743,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16750"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16767"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3808,7 +3808,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16751"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16768"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -4584,70 +4584,70 @@
     </row>
     <row r="4" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
-      <c r="C4" s="150" t="e" vm="1">
+      <c r="C4" s="137" t="e" vm="1">
         <f>'Cards Src'!E2</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="150"/>
-      <c r="E4" s="150"/>
+      <c r="D4" s="137"/>
+      <c r="E4" s="137"/>
       <c r="F4" s="42"/>
       <c r="H4" s="53"/>
-      <c r="I4" s="155" t="e" vm="2">
+      <c r="I4" s="142" t="e" vm="2">
         <f>'Cards Src'!E3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J4" s="155"/>
-      <c r="K4" s="155"/>
+      <c r="J4" s="142"/>
+      <c r="K4" s="142"/>
       <c r="L4" s="54"/>
       <c r="N4" s="116"/>
-      <c r="O4" s="156" t="e" vm="3">
+      <c r="O4" s="143" t="e" vm="3">
         <f>'Cards Src'!E4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P4" s="156"/>
-      <c r="Q4" s="156"/>
+      <c r="P4" s="143"/>
+      <c r="Q4" s="143"/>
       <c r="R4" s="64"/>
       <c r="T4" s="7"/>
-      <c r="U4" s="157" t="e" vm="4">
+      <c r="U4" s="144" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V4" s="157"/>
-      <c r="W4" s="157"/>
+      <c r="V4" s="144"/>
+      <c r="W4" s="144"/>
       <c r="X4" s="29"/>
     </row>
     <row r="5" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
-      <c r="C5" s="151" t="str">
+      <c r="C5" s="138" t="str">
         <f>'Cards Src'!$C2</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="151"/>
-      <c r="E5" s="151"/>
+      <c r="D5" s="138"/>
+      <c r="E5" s="138"/>
       <c r="F5" s="43"/>
       <c r="H5" s="53"/>
-      <c r="I5" s="152" t="str">
+      <c r="I5" s="139" t="str">
         <f>'Cards Src'!$C3</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="J5" s="152"/>
-      <c r="K5" s="152"/>
+      <c r="J5" s="139"/>
+      <c r="K5" s="139"/>
       <c r="L5" s="55"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="153" t="str">
+      <c r="O5" s="140" t="str">
         <f>'Cards Src'!C4</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="P5" s="153"/>
-      <c r="Q5" s="153"/>
+      <c r="P5" s="140"/>
+      <c r="Q5" s="140"/>
       <c r="R5" s="65"/>
       <c r="T5" s="7"/>
-      <c r="U5" s="154" t="str">
+      <c r="U5" s="141" t="str">
         <f>'Cards Src'!C5</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="V5" s="154"/>
-      <c r="W5" s="154"/>
+      <c r="V5" s="141"/>
+      <c r="W5" s="141"/>
       <c r="X5" s="30"/>
     </row>
     <row r="6" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4747,12 +4747,12 @@
       <c r="K10" s="149"/>
       <c r="L10" s="72"/>
       <c r="N10" s="19"/>
-      <c r="O10" s="142" t="e" vm="7">
+      <c r="O10" s="150" t="e" vm="7">
         <f>'Cards Src'!E8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P10" s="142"/>
-      <c r="Q10" s="142"/>
+      <c r="P10" s="150"/>
+      <c r="Q10" s="150"/>
       <c r="R10" s="81"/>
       <c r="T10" s="11"/>
       <c r="U10" s="145" t="e" vm="8">
@@ -4878,70 +4878,70 @@
     </row>
     <row r="16" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="19"/>
-      <c r="C16" s="142" t="e" vm="9">
+      <c r="C16" s="150" t="e" vm="9">
         <f>'Cards Src'!E10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D16" s="142"/>
-      <c r="E16" s="142"/>
+      <c r="D16" s="150"/>
+      <c r="E16" s="150"/>
       <c r="F16" s="81"/>
       <c r="H16" s="107"/>
-      <c r="I16" s="144" t="e" vm="10">
+      <c r="I16" s="153" t="e" vm="10">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J16" s="144"/>
-      <c r="K16" s="144"/>
+      <c r="J16" s="153"/>
+      <c r="K16" s="153"/>
       <c r="L16" s="108"/>
       <c r="N16" s="107"/>
-      <c r="O16" s="137" t="e" vm="11">
+      <c r="O16" s="154" t="e" vm="11">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P16" s="137"/>
-      <c r="Q16" s="137"/>
+      <c r="P16" s="154"/>
+      <c r="Q16" s="154"/>
       <c r="R16" s="108"/>
       <c r="T16" s="107"/>
-      <c r="U16" s="137" t="e" vm="12">
+      <c r="U16" s="154" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V16" s="137"/>
-      <c r="W16" s="137"/>
+      <c r="V16" s="154"/>
+      <c r="W16" s="154"/>
       <c r="X16" s="108"/>
     </row>
     <row r="17" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="19"/>
-      <c r="C17" s="143" t="str">
+      <c r="C17" s="151" t="str">
         <f>'Cards Src'!$C10</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D17" s="143"/>
-      <c r="E17" s="143"/>
+      <c r="D17" s="151"/>
+      <c r="E17" s="151"/>
       <c r="F17" s="82"/>
       <c r="H17" s="107"/>
-      <c r="I17" s="138" t="str">
+      <c r="I17" s="152" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="J17" s="138"/>
-      <c r="K17" s="138"/>
+      <c r="J17" s="152"/>
+      <c r="K17" s="152"/>
       <c r="L17" s="110"/>
       <c r="N17" s="107"/>
-      <c r="O17" s="138" t="str">
+      <c r="O17" s="152" t="str">
         <f>'Cards Src'!C12</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="P17" s="138"/>
-      <c r="Q17" s="138"/>
+      <c r="P17" s="152"/>
+      <c r="Q17" s="152"/>
       <c r="R17" s="110"/>
       <c r="T17" s="107"/>
-      <c r="U17" s="138" t="str">
+      <c r="U17" s="152" t="str">
         <f>'Cards Src'!C13</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="V17" s="138"/>
-      <c r="W17" s="138"/>
+      <c r="V17" s="152"/>
+      <c r="W17" s="152"/>
       <c r="X17" s="110"/>
     </row>
     <row r="18" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5025,70 +5025,70 @@
     </row>
     <row r="22" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="107"/>
-      <c r="C22" s="137" t="e" vm="13">
+      <c r="C22" s="154" t="e" vm="13">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D22" s="137"/>
-      <c r="E22" s="137"/>
+      <c r="D22" s="154"/>
+      <c r="E22" s="154"/>
       <c r="F22" s="108"/>
       <c r="H22" s="107"/>
-      <c r="I22" s="137" t="e" vm="14">
+      <c r="I22" s="154" t="e" vm="14">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J22" s="137"/>
-      <c r="K22" s="137"/>
+      <c r="J22" s="154"/>
+      <c r="K22" s="154"/>
       <c r="L22" s="108"/>
       <c r="N22" s="107"/>
-      <c r="O22" s="137" t="e" vm="15">
+      <c r="O22" s="154" t="e" vm="15">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P22" s="137"/>
-      <c r="Q22" s="137"/>
+      <c r="P22" s="154"/>
+      <c r="Q22" s="154"/>
       <c r="R22" s="108"/>
       <c r="T22" s="107"/>
-      <c r="U22" s="137" t="e" vm="16">
+      <c r="U22" s="154" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V22" s="137"/>
-      <c r="W22" s="137"/>
+      <c r="V22" s="154"/>
+      <c r="W22" s="154"/>
       <c r="X22" s="108"/>
     </row>
     <row r="23" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="107"/>
-      <c r="C23" s="138" t="str">
+      <c r="C23" s="152" t="str">
         <f>'Cards Src'!$C14</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D23" s="138"/>
-      <c r="E23" s="138"/>
+      <c r="D23" s="152"/>
+      <c r="E23" s="152"/>
       <c r="F23" s="110"/>
       <c r="H23" s="107"/>
-      <c r="I23" s="138" t="str">
+      <c r="I23" s="152" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="J23" s="138"/>
-      <c r="K23" s="138"/>
+      <c r="J23" s="152"/>
+      <c r="K23" s="152"/>
       <c r="L23" s="110"/>
       <c r="N23" s="107"/>
-      <c r="O23" s="141" t="str">
+      <c r="O23" s="155" t="str">
         <f>'Cards Src'!C16</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="P23" s="141"/>
-      <c r="Q23" s="141"/>
+      <c r="P23" s="155"/>
+      <c r="Q23" s="155"/>
       <c r="R23" s="110"/>
       <c r="T23" s="107"/>
-      <c r="U23" s="138" t="str">
+      <c r="U23" s="152" t="str">
         <f>'Cards Src'!C17</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="V23" s="138"/>
-      <c r="W23" s="138"/>
+      <c r="V23" s="152"/>
+      <c r="W23" s="152"/>
       <c r="X23" s="110"/>
     </row>
     <row r="24" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5172,70 +5172,70 @@
     </row>
     <row r="28" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="107"/>
-      <c r="C28" s="137" t="e" vm="17">
+      <c r="C28" s="154" t="e" vm="17">
         <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D28" s="137"/>
-      <c r="E28" s="137"/>
+      <c r="D28" s="154"/>
+      <c r="E28" s="154"/>
       <c r="F28" s="108"/>
       <c r="H28" s="107"/>
-      <c r="I28" s="137" t="e" vm="18">
+      <c r="I28" s="154" t="e" vm="18">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J28" s="137"/>
-      <c r="K28" s="137"/>
+      <c r="J28" s="154"/>
+      <c r="K28" s="154"/>
       <c r="L28" s="108"/>
       <c r="N28" s="94"/>
-      <c r="O28" s="140">
+      <c r="O28" s="157">
         <f>'Cards Src'!E20</f>
         <v>0</v>
       </c>
-      <c r="P28" s="140"/>
-      <c r="Q28" s="140"/>
+      <c r="P28" s="157"/>
+      <c r="Q28" s="157"/>
       <c r="R28" s="95"/>
       <c r="T28" s="94"/>
-      <c r="U28" s="140">
+      <c r="U28" s="157">
         <f xml:space="preserve"> 'Cards Src'!E21</f>
         <v>0</v>
       </c>
-      <c r="V28" s="140"/>
-      <c r="W28" s="140"/>
+      <c r="V28" s="157"/>
+      <c r="W28" s="157"/>
       <c r="X28" s="95"/>
     </row>
     <row r="29" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="107"/>
-      <c r="C29" s="138" t="str">
+      <c r="C29" s="152" t="str">
         <f>'Cards Src'!$C18</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D29" s="138"/>
-      <c r="E29" s="138"/>
+      <c r="D29" s="152"/>
+      <c r="E29" s="152"/>
       <c r="F29" s="110"/>
       <c r="H29" s="107"/>
-      <c r="I29" s="138" t="str">
+      <c r="I29" s="152" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="J29" s="138"/>
-      <c r="K29" s="138"/>
+      <c r="J29" s="152"/>
+      <c r="K29" s="152"/>
       <c r="L29" s="110"/>
       <c r="N29" s="94"/>
-      <c r="O29" s="139">
+      <c r="O29" s="156">
         <f>'Cards Src'!C20</f>
         <v>0</v>
       </c>
-      <c r="P29" s="139"/>
-      <c r="Q29" s="139"/>
+      <c r="P29" s="156"/>
+      <c r="Q29" s="156"/>
       <c r="R29" s="96"/>
       <c r="T29" s="94"/>
-      <c r="U29" s="139">
+      <c r="U29" s="156">
         <f>'Cards Src'!C21</f>
         <v>0</v>
       </c>
-      <c r="V29" s="139"/>
-      <c r="W29" s="139"/>
+      <c r="V29" s="156"/>
+      <c r="W29" s="156"/>
       <c r="X29" s="96"/>
     </row>
     <row r="30" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5262,6 +5262,38 @@
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="U29:W29"/>
+    <mergeCell ref="I28:K28"/>
+    <mergeCell ref="O28:Q28"/>
+    <mergeCell ref="U28:W28"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="O23:Q23"/>
+    <mergeCell ref="U23:W23"/>
+    <mergeCell ref="I22:K22"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="U22:W22"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="O17:Q17"/>
+    <mergeCell ref="U17:W17"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="U16:W16"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="O11:Q11"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="O10:Q10"/>
+    <mergeCell ref="U10:W10"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="I5:K5"/>
@@ -5270,38 +5302,6 @@
     <mergeCell ref="I4:K4"/>
     <mergeCell ref="O4:Q4"/>
     <mergeCell ref="U4:W4"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="O11:Q11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="U10:W10"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="U17:W17"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="U16:W16"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="U23:W23"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="U22:W22"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="U29:W29"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="U28:W28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Art - Haste + Hinder
Added art for Haste and Hinder modifier cards
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEAC17BA-D342-4EF2-9BFE-C75B0AEECD0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8336CE25-34B3-42AF-9151-F9AC82A7BDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2724,7 +2724,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16752"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16769"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2789,7 +2789,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16753"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16770"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2854,7 +2854,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16754"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16771"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2919,7 +2919,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16755"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16772"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2984,7 +2984,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16756"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16773"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3049,7 +3049,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16757"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16774"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3114,7 +3114,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16758"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16775"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3179,7 +3179,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16759"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16776"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3244,7 +3244,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16760"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16777"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3309,7 +3309,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16761"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16778"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3374,7 +3374,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16762"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16779"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3439,7 +3439,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16763"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16780"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3504,7 +3504,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16764"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16781"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3569,7 +3569,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16765"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16782"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3634,7 +3634,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16766"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16783"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3743,7 +3743,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16767"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16784"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3808,7 +3808,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16768"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16785"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>

</xml_diff>

<commit_message>
Art - Holy Blade
Add art for Holy Blade modifier card
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8336CE25-34B3-42AF-9151-F9AC82A7BDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E4B0C39-D0B1-4911-AD2D-BB6CE0B58C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2724,7 +2724,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16769"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16820"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2789,7 +2789,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16770"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16821"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2854,7 +2854,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16771"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16822"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2919,7 +2919,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16772"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16823"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2984,7 +2984,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16773"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16824"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3049,7 +3049,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16774"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16825"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3114,7 +3114,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16775"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16826"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3179,7 +3179,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16776"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16827"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3244,7 +3244,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16777"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16828"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3309,7 +3309,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16778"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16829"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3374,7 +3374,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16779"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16830"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3439,7 +3439,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16780"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16831"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3504,7 +3504,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16781"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16832"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3569,7 +3569,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16782"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16833"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3634,7 +3634,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16783"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16834"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3743,7 +3743,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16784"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16835"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3808,7 +3808,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16785"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16836"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>

</xml_diff>

<commit_message>
Icons - new cards
Added icons for all the new art added to cards: Astral Dagger, Haste, Hinder, Holy Blade
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E4B0C39-D0B1-4911-AD2D-BB6CE0B58C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D23EE9-BA75-4444-8933-57CFB2A18285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2724,7 +2724,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16820"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16854"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2789,7 +2789,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16821"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16855"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2854,7 +2854,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16822"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16856"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2919,7 +2919,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16823"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16857"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2984,7 +2984,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16824"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16858"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3049,7 +3049,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16825"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16859"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3114,7 +3114,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16826"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16860"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3179,7 +3179,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16827"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16861"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3244,7 +3244,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16828"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16862"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3309,7 +3309,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16829"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16863"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3374,7 +3374,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16830"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16864"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3439,7 +3439,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16831"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16865"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3504,7 +3504,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16832"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16866"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3569,7 +3569,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16833"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16867"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3634,7 +3634,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16834"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16868"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3743,7 +3743,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16835"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16869"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3808,7 +3808,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16836"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16870"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>

</xml_diff>

<commit_message>
Art - Lightning Bolt + updates
Added art for Lightning Bolt attack card; updated art for Astral Dagger, Haste, Hinder
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D23EE9-BA75-4444-8933-57CFB2A18285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA294477-9A38-45C4-B254-2F4D3BD666CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="69">
+  <futureMetadata name="XLRICHVALUE" count="70">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -527,8 +527,15 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="69"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="69">
+  <valueMetadata count="70">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -735,13 +742,16 @@
     </bk>
     <bk>
       <rc t="1" v="68"/>
+    </bk>
+    <bk>
+      <rc t="1" v="69"/>
     </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="59">
   <si>
     <t>FIREBALL</t>
   </si>
@@ -915,6 +925,9 @@
   </si>
   <si>
     <t>Mod Cards</t>
+  </si>
+  <si>
+    <t>Shadow</t>
   </si>
 </sst>
 </file>
@@ -1502,14 +1515,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1517,43 +1551,22 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2724,7 +2737,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16854"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17260"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2789,7 +2802,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16855"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17261"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2837,9 +2850,9 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
+          <xdr:colOff>39000</xdr:colOff>
           <xdr:row>2</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
+          <xdr:rowOff>867675</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
           <xdr:nvPicPr>
@@ -2854,7 +2867,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16856"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17262"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2869,72 +2882,7 @@
           <xdr:spPr bwMode="auto">
             <a:xfrm>
               <a:off x="4914900" y="200025"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>1</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>15</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="12" name="Picture 11">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C994F9A-5B33-67AA-9C9C-D9DC82FDA6AD}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16857"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="200025"/>
-              <a:ext cx="1038225" cy="1038225"/>
+              <a:ext cx="1029600" cy="1029600"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -2984,13 +2932,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16858"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17263"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3049,13 +2997,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16859"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17264"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3114,13 +3062,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16860"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17265"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3179,13 +3127,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16861"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17266"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3244,13 +3192,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16862"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17267"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3309,13 +3257,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16863"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17268"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3374,13 +3322,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16864"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17269"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3439,13 +3387,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16865"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17270"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3504,13 +3452,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16866"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17271"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3569,13 +3517,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16867"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17272"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3634,13 +3582,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16868"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17273"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3698,7 +3646,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3743,13 +3691,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16869"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17274"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3808,13 +3756,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s16870"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17275"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3845,6 +3793,496 @@
     </mc:Choice>
     <mc:Fallback/>
   </mc:AlternateContent>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>876300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="48" name="Picture 47">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F5E0CB1F-02DA-C872-A939-68E2534E8E22}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9220200" y="200025"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A47A4D9-D75D-4D66-96C3-449B2874EB89}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9220200" y="200025"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A134AF24-B6D7-4AB8-8EF4-B5842E828C94}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13525500" y="200025"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47C718FD-AAC6-481E-85D4-59F075E8B6E6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4924425" y="5562600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0C9055C-53C5-4603-A264-B13B380B06C5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="619125" y="10925175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{36E5BE00-8060-08B8-1A46-54B06B9CFE18}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4914900" y="16287750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{342F9020-4A63-480A-9CF7-EBAC246CABE1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9210675" y="16278225"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>371475</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="Rectangle 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A516ECD-B904-7AC4-F9EC-16B12B828337}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9210675" y="21640800"/>
+          <a:ext cx="8010525" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-CA" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3889,7 +4327,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="69">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="70">
   <rv s="0">
     <v>0</v>
     <v>4</v>
@@ -4164,6 +4602,10 @@
   </rv>
   <rv s="0">
     <v>50</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>51</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -4231,6 +4673,7 @@
   <rel r:id="rId49"/>
   <rel r:id="rId50"/>
   <rel r:id="rId51"/>
+  <rel r:id="rId52"/>
 </richValueRels>
 </file>
 
@@ -4584,70 +5027,70 @@
     </row>
     <row r="4" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
-      <c r="C4" s="137" t="e" vm="1">
+      <c r="C4" s="143" t="e" vm="1">
         <f>'Cards Src'!E2</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="137"/>
-      <c r="E4" s="137"/>
+      <c r="D4" s="143"/>
+      <c r="E4" s="143"/>
       <c r="F4" s="42"/>
       <c r="H4" s="53"/>
-      <c r="I4" s="142" t="e" vm="2">
+      <c r="I4" s="144" t="e" vm="2">
         <f>'Cards Src'!E3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J4" s="142"/>
-      <c r="K4" s="142"/>
+      <c r="J4" s="144"/>
+      <c r="K4" s="144"/>
       <c r="L4" s="54"/>
       <c r="N4" s="116"/>
-      <c r="O4" s="143" t="e" vm="3">
+      <c r="O4" s="149" t="e" vm="3">
         <f>'Cards Src'!E4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P4" s="143"/>
-      <c r="Q4" s="143"/>
+      <c r="P4" s="149"/>
+      <c r="Q4" s="149"/>
       <c r="R4" s="64"/>
       <c r="T4" s="7"/>
-      <c r="U4" s="144" t="e" vm="4">
+      <c r="U4" s="150" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V4" s="144"/>
-      <c r="W4" s="144"/>
+      <c r="V4" s="150"/>
+      <c r="W4" s="150"/>
       <c r="X4" s="29"/>
     </row>
     <row r="5" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
-      <c r="C5" s="138" t="str">
+      <c r="C5" s="137" t="str">
         <f>'Cards Src'!$C2</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="138"/>
-      <c r="E5" s="138"/>
+      <c r="D5" s="137"/>
+      <c r="E5" s="137"/>
       <c r="F5" s="43"/>
       <c r="H5" s="53"/>
-      <c r="I5" s="139" t="str">
+      <c r="I5" s="138" t="str">
         <f>'Cards Src'!$C3</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="J5" s="139"/>
-      <c r="K5" s="139"/>
+      <c r="J5" s="138"/>
+      <c r="K5" s="138"/>
       <c r="L5" s="55"/>
       <c r="N5" s="3"/>
-      <c r="O5" s="140" t="str">
+      <c r="O5" s="147" t="str">
         <f>'Cards Src'!C4</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="P5" s="140"/>
-      <c r="Q5" s="140"/>
+      <c r="P5" s="147"/>
+      <c r="Q5" s="147"/>
       <c r="R5" s="65"/>
       <c r="T5" s="7"/>
-      <c r="U5" s="141" t="str">
+      <c r="U5" s="148" t="str">
         <f>'Cards Src'!C5</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="V5" s="141"/>
-      <c r="W5" s="141"/>
+      <c r="V5" s="148"/>
+      <c r="W5" s="148"/>
       <c r="X5" s="30"/>
     </row>
     <row r="6" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4731,70 +5174,70 @@
     </row>
     <row r="10" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="11"/>
-      <c r="C10" s="145" t="e" vm="5">
+      <c r="C10" s="146" t="e" vm="5">
         <f>'Cards Src'!E6</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D10" s="145"/>
-      <c r="E10" s="145"/>
+      <c r="D10" s="146"/>
+      <c r="E10" s="146"/>
       <c r="F10" s="126"/>
       <c r="H10" s="15"/>
-      <c r="I10" s="149" t="e" vm="6">
+      <c r="I10" s="152" t="e" vm="6">
         <f>'Cards Src'!E7</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J10" s="149"/>
-      <c r="K10" s="149"/>
+      <c r="J10" s="152"/>
+      <c r="K10" s="152"/>
       <c r="L10" s="72"/>
       <c r="N10" s="19"/>
-      <c r="O10" s="150" t="e" vm="7">
+      <c r="O10" s="145" t="e" vm="7">
         <f>'Cards Src'!E8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P10" s="150"/>
-      <c r="Q10" s="150"/>
+      <c r="P10" s="145"/>
+      <c r="Q10" s="145"/>
       <c r="R10" s="81"/>
       <c r="T10" s="11"/>
-      <c r="U10" s="145" t="e" vm="8">
+      <c r="U10" s="146" t="e" vm="8">
         <f>'Cards Src'!E9</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V10" s="145"/>
-      <c r="W10" s="145"/>
+      <c r="V10" s="146"/>
+      <c r="W10" s="146"/>
       <c r="X10" s="122"/>
     </row>
     <row r="11" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="11"/>
-      <c r="C11" s="146" t="str">
+      <c r="C11" s="140" t="str">
         <f>'Cards Src'!$C6</f>
         <v>Casts a bolt of lightning</v>
       </c>
-      <c r="D11" s="146"/>
-      <c r="E11" s="146"/>
+      <c r="D11" s="140"/>
+      <c r="E11" s="140"/>
       <c r="F11" s="123"/>
       <c r="H11" s="15"/>
-      <c r="I11" s="147" t="str">
+      <c r="I11" s="151" t="str">
         <f>'Cards Src'!$C7</f>
         <v>Vacuums in nearby enemies</v>
       </c>
-      <c r="J11" s="147"/>
-      <c r="K11" s="147"/>
+      <c r="J11" s="151"/>
+      <c r="K11" s="151"/>
       <c r="L11" s="73"/>
       <c r="N11" s="19"/>
-      <c r="O11" s="148" t="str">
+      <c r="O11" s="139" t="str">
         <f>'Cards Src'!C8</f>
         <v>Flies to the nearest enemy in vision</v>
       </c>
-      <c r="P11" s="148"/>
-      <c r="Q11" s="148"/>
+      <c r="P11" s="139"/>
+      <c r="Q11" s="139"/>
       <c r="R11" s="82"/>
       <c r="T11" s="11"/>
-      <c r="U11" s="146" t="str">
+      <c r="U11" s="140" t="str">
         <f>'Cards Src'!C9</f>
         <v>Casts a tracking bolt of lightning that can chain to close enemies</v>
       </c>
-      <c r="V11" s="146"/>
-      <c r="W11" s="146"/>
+      <c r="V11" s="140"/>
+      <c r="W11" s="140"/>
       <c r="X11" s="123"/>
     </row>
     <row r="12" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4878,70 +5321,70 @@
     </row>
     <row r="16" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="19"/>
-      <c r="C16" s="150" t="e" vm="9">
+      <c r="C16" s="145" t="e" vm="9">
         <f>'Cards Src'!E10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D16" s="150"/>
-      <c r="E16" s="150"/>
+      <c r="D16" s="145"/>
+      <c r="E16" s="145"/>
       <c r="F16" s="81"/>
       <c r="H16" s="107"/>
-      <c r="I16" s="153" t="e" vm="10">
+      <c r="I16" s="154" t="e" vm="10">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J16" s="153"/>
-      <c r="K16" s="153"/>
+      <c r="J16" s="154"/>
+      <c r="K16" s="154"/>
       <c r="L16" s="108"/>
       <c r="N16" s="107"/>
-      <c r="O16" s="154" t="e" vm="11">
+      <c r="O16" s="141" t="e" vm="11">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P16" s="154"/>
-      <c r="Q16" s="154"/>
+      <c r="P16" s="141"/>
+      <c r="Q16" s="141"/>
       <c r="R16" s="108"/>
       <c r="T16" s="107"/>
-      <c r="U16" s="154" t="e" vm="12">
+      <c r="U16" s="141" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V16" s="154"/>
-      <c r="W16" s="154"/>
+      <c r="V16" s="141"/>
+      <c r="W16" s="141"/>
       <c r="X16" s="108"/>
     </row>
     <row r="17" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="19"/>
-      <c r="C17" s="151" t="str">
+      <c r="C17" s="153" t="str">
         <f>'Cards Src'!$C10</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D17" s="151"/>
-      <c r="E17" s="151"/>
+      <c r="D17" s="153"/>
+      <c r="E17" s="153"/>
       <c r="F17" s="82"/>
       <c r="H17" s="107"/>
-      <c r="I17" s="152" t="str">
+      <c r="I17" s="142" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="J17" s="152"/>
-      <c r="K17" s="152"/>
+      <c r="J17" s="142"/>
+      <c r="K17" s="142"/>
       <c r="L17" s="110"/>
       <c r="N17" s="107"/>
-      <c r="O17" s="152" t="str">
+      <c r="O17" s="142" t="str">
         <f>'Cards Src'!C12</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="P17" s="152"/>
-      <c r="Q17" s="152"/>
+      <c r="P17" s="142"/>
+      <c r="Q17" s="142"/>
       <c r="R17" s="110"/>
       <c r="T17" s="107"/>
-      <c r="U17" s="152" t="str">
+      <c r="U17" s="142" t="str">
         <f>'Cards Src'!C13</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="V17" s="152"/>
-      <c r="W17" s="152"/>
+      <c r="V17" s="142"/>
+      <c r="W17" s="142"/>
       <c r="X17" s="110"/>
     </row>
     <row r="18" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5025,54 +5468,54 @@
     </row>
     <row r="22" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="107"/>
-      <c r="C22" s="154" t="e" vm="13">
+      <c r="C22" s="141" t="e" vm="13">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D22" s="154"/>
-      <c r="E22" s="154"/>
+      <c r="D22" s="141"/>
+      <c r="E22" s="141"/>
       <c r="F22" s="108"/>
       <c r="H22" s="107"/>
-      <c r="I22" s="154" t="e" vm="14">
+      <c r="I22" s="141" t="e" vm="14">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J22" s="154"/>
-      <c r="K22" s="154"/>
+      <c r="J22" s="141"/>
+      <c r="K22" s="141"/>
       <c r="L22" s="108"/>
       <c r="N22" s="107"/>
-      <c r="O22" s="154" t="e" vm="15">
+      <c r="O22" s="141" t="e" vm="15">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P22" s="154"/>
-      <c r="Q22" s="154"/>
+      <c r="P22" s="141"/>
+      <c r="Q22" s="141"/>
       <c r="R22" s="108"/>
       <c r="T22" s="107"/>
-      <c r="U22" s="154" t="e" vm="16">
+      <c r="U22" s="141" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V22" s="154"/>
-      <c r="W22" s="154"/>
+      <c r="V22" s="141"/>
+      <c r="W22" s="141"/>
       <c r="X22" s="108"/>
     </row>
     <row r="23" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="107"/>
-      <c r="C23" s="152" t="str">
+      <c r="C23" s="142" t="str">
         <f>'Cards Src'!$C14</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D23" s="152"/>
-      <c r="E23" s="152"/>
+      <c r="D23" s="142"/>
+      <c r="E23" s="142"/>
       <c r="F23" s="110"/>
       <c r="H23" s="107"/>
-      <c r="I23" s="152" t="str">
+      <c r="I23" s="142" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="J23" s="152"/>
-      <c r="K23" s="152"/>
+      <c r="J23" s="142"/>
+      <c r="K23" s="142"/>
       <c r="L23" s="110"/>
       <c r="N23" s="107"/>
       <c r="O23" s="155" t="str">
@@ -5083,12 +5526,12 @@
       <c r="Q23" s="155"/>
       <c r="R23" s="110"/>
       <c r="T23" s="107"/>
-      <c r="U23" s="152" t="str">
+      <c r="U23" s="142" t="str">
         <f>'Cards Src'!C17</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="V23" s="152"/>
-      <c r="W23" s="152"/>
+      <c r="V23" s="142"/>
+      <c r="W23" s="142"/>
       <c r="X23" s="110"/>
     </row>
     <row r="24" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5172,20 +5615,20 @@
     </row>
     <row r="28" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="107"/>
-      <c r="C28" s="154" t="e" vm="17">
+      <c r="C28" s="141" t="e" vm="17">
         <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D28" s="154"/>
-      <c r="E28" s="154"/>
+      <c r="D28" s="141"/>
+      <c r="E28" s="141"/>
       <c r="F28" s="108"/>
       <c r="H28" s="107"/>
-      <c r="I28" s="154" t="e" vm="18">
+      <c r="I28" s="141" t="e" vm="18">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J28" s="154"/>
-      <c r="K28" s="154"/>
+      <c r="J28" s="141"/>
+      <c r="K28" s="141"/>
       <c r="L28" s="108"/>
       <c r="N28" s="94"/>
       <c r="O28" s="157">
@@ -5206,20 +5649,20 @@
     </row>
     <row r="29" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="107"/>
-      <c r="C29" s="152" t="str">
+      <c r="C29" s="142" t="str">
         <f>'Cards Src'!$C18</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D29" s="152"/>
-      <c r="E29" s="152"/>
+      <c r="D29" s="142"/>
+      <c r="E29" s="142"/>
       <c r="F29" s="110"/>
       <c r="H29" s="107"/>
-      <c r="I29" s="152" t="str">
+      <c r="I29" s="142" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="J29" s="152"/>
-      <c r="K29" s="152"/>
+      <c r="J29" s="142"/>
+      <c r="K29" s="142"/>
       <c r="L29" s="110"/>
       <c r="N29" s="94"/>
       <c r="O29" s="156">
@@ -5872,7 +6315,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.42578125" customWidth="1"/>
@@ -5925,6 +6368,18 @@
         <v>#VALUE!</v>
       </c>
     </row>
+    <row r="7" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="130"/>
+      <c r="D7" s="21"/>
+    </row>
+    <row r="8" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="e" vm="70">
+        <v>#VALUE!</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Icons - Lightning Bolt + updates
Added Lightning Bolt icon and updated same icons as before
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA294477-9A38-45C4-B254-2F4D3BD666CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C776112E-87DA-4608-88D8-1C02E353FA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2737,7 +2737,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17260"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17337"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2802,7 +2802,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17261"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17338"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2867,7 +2867,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17262"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17339"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2932,7 +2932,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17263"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17340"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2997,7 +2997,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17264"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17341"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3062,7 +3062,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17265"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17342"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3127,7 +3127,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17266"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17343"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3192,7 +3192,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17267"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17344"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3257,7 +3257,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17268"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17345"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3322,7 +3322,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17269"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17346"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3387,7 +3387,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17270"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17347"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3452,7 +3452,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17271"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17348"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3517,7 +3517,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17272"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17349"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3582,7 +3582,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17273"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17350"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3691,7 +3691,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17274"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17351"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3756,7 +3756,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17275"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17352"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -4281,6 +4281,738 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>481013</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>885825</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>604838</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Picture 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8831CAF-765A-376B-CBC4-016EA1EE93D7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="10058400" y="22293263"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1114425</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>481013</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>604838</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06988B88-EB59-AB4A-D5B7-BDC424D1F0BA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11325225" y="22293263"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>481013</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>604838</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Picture 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FF812E4-B6D6-CECC-5B4A-73868D65CA98}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12592050" y="22293263"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>481013</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>604838</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Picture 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB7D0B06-DE13-1417-6EF2-6A6EF94310A1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13858875" y="22293263"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>481013</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1647825</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>604838</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Picture 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A5315F95-4D46-66EE-C323-64D3F2E3321B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="15125700" y="22293263"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1143000</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>828676</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>1866901</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Picture 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DD0C64F-AAA2-6E40-37DC-E20C00999C48}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11353800" y="23555326"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>669925</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>828676</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>107950</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>1866901</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="49" name="Picture 48">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3962F17-29F7-6F8E-C3A8-2D817E6F1ED5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12595225" y="23555326"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>527050</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>2157414</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1565275</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>852489</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="50" name="Picture 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C78D2958-1504-39E6-0311-D5797A816C59}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="10737850" y="24884064"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>95603</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>2157414</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>143228</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>852489</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="51" name="Picture 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8705D76C-A8C6-42B5-FFF9-4BDF5A67539D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12020903" y="24884064"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>44450</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>828676</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>358775</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>1866901</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="55" name="Picture 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21652EF6-F28C-E8CD-6828-D68EA02E418F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13836650" y="23555326"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>388056</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>2157414</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>549981</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>852489</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="62" name="Picture 61">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{327DF20A-8EF9-89BE-E67E-B5B4D1744CFA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="13303956" y="24884064"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>70909</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>2157414</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>1109134</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>852489</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="63" name="Picture 62">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27A495BE-20CF-A560-F49E-CF01492E2C8C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="14587009" y="24884064"/>
+          <a:ext cx="1038225" cy="1038225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>

<commit_message>
Art - Mana Shield
Art for Mana Shield modifier card
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C776112E-87DA-4608-88D8-1C02E353FA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA34AD08-B85F-4F96-AB2E-4E65F65B978D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="70">
+  <futureMetadata name="XLRICHVALUE" count="76">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -534,8 +534,50 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="70"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="71"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="72"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="73"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="74"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="75"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="70">
+  <valueMetadata count="76">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -745,6 +787,24 @@
     </bk>
     <bk>
       <rc t="1" v="69"/>
+    </bk>
+    <bk>
+      <rc t="1" v="70"/>
+    </bk>
+    <bk>
+      <rc t="1" v="71"/>
+    </bk>
+    <bk>
+      <rc t="1" v="72"/>
+    </bk>
+    <bk>
+      <rc t="1" v="73"/>
+    </bk>
+    <bk>
+      <rc t="1" v="74"/>
+    </bk>
+    <bk>
+      <rc t="1" v="75"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -1003,7 +1063,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1085,6 +1145,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD6DCE4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1201,7 +1267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1515,67 +1581,71 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1615,13 +1685,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1674,15 +1744,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1735,15 +1805,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1796,15 +1866,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>19</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1859,13 +1929,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1918,15 +1988,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1979,15 +2049,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>19</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2040,15 +2110,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2101,15 +2171,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2164,13 +2234,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2223,15 +2293,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>19</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2284,15 +2354,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2345,15 +2415,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2408,13 +2478,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2467,13 +2537,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>19</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
@@ -2528,13 +2598,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
@@ -2589,13 +2659,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
@@ -2715,13 +2785,13 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
+          <xdr:row>6</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>8</xdr:row>
+          <xdr:row>7</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -2737,7 +2807,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17337"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26099"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2778,15 +2848,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>19</xdr:col>
+          <xdr:col>16</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
+          <xdr:row>6</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>21</xdr:col>
+          <xdr:col>18</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>8</xdr:row>
+          <xdr:row>7</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -2802,7 +2872,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17338"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26100"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2843,13 +2913,13 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>7</xdr:col>
+          <xdr:col>6</xdr:col>
           <xdr:colOff>0</xdr:colOff>
           <xdr:row>1</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>9</xdr:col>
+          <xdr:col>8</xdr:col>
           <xdr:colOff>39000</xdr:colOff>
           <xdr:row>2</xdr:row>
           <xdr:rowOff>867675</xdr:rowOff>
@@ -2867,7 +2937,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17339"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26101"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2908,13 +2978,13 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>19</xdr:col>
+          <xdr:col>16</xdr:col>
           <xdr:colOff>0</xdr:colOff>
           <xdr:row>1</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>21</xdr:col>
+          <xdr:col>18</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
           <xdr:row>2</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
@@ -2932,7 +3002,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17340"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26102"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2973,15 +3043,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>7</xdr:col>
+          <xdr:col>6</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
+          <xdr:row>6</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>9</xdr:col>
+          <xdr:col>8</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>8</xdr:row>
+          <xdr:row>7</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -2997,7 +3067,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17341"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26103"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3038,15 +3108,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>13</xdr:col>
+          <xdr:col>11</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>7</xdr:row>
+          <xdr:row>6</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>15</xdr:col>
+          <xdr:col>13</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>8</xdr:row>
+          <xdr:row>7</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3062,7 +3132,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17342"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26104"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3105,13 +3175,13 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
+          <xdr:row>11</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>14</xdr:row>
+          <xdr:row>12</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3127,7 +3197,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17343"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26105"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3168,15 +3238,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>7</xdr:col>
+          <xdr:col>6</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
+          <xdr:row>11</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>9</xdr:col>
+          <xdr:col>8</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>14</xdr:row>
+          <xdr:row>12</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3192,7 +3262,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17344"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26106"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3233,15 +3303,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>13</xdr:col>
+          <xdr:col>11</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
+          <xdr:row>11</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>15</xdr:col>
+          <xdr:col>13</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>14</xdr:row>
+          <xdr:row>12</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3257,7 +3327,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17345"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26107"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3298,15 +3368,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>13</xdr:col>
+          <xdr:col>11</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
+          <xdr:row>16</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>15</xdr:col>
+          <xdr:col>13</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>20</xdr:row>
+          <xdr:row>17</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3322,7 +3392,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17346"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26108"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3363,15 +3433,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>7</xdr:col>
+          <xdr:col>6</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
+          <xdr:row>16</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>9</xdr:col>
+          <xdr:col>8</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>20</xdr:row>
+          <xdr:row>17</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3387,7 +3457,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17347"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26109"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3428,15 +3498,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>19</xdr:col>
+          <xdr:col>16</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
+          <xdr:row>16</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>21</xdr:col>
+          <xdr:col>18</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>20</xdr:row>
+          <xdr:row>17</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3452,7 +3522,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17348"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26110"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3493,15 +3563,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>19</xdr:col>
+          <xdr:col>16</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>13</xdr:row>
+          <xdr:row>11</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>21</xdr:col>
+          <xdr:col>18</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>14</xdr:row>
+          <xdr:row>12</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3517,7 +3587,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17349"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26111"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3560,13 +3630,13 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>19</xdr:row>
+          <xdr:row>16</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>20</xdr:row>
+          <xdr:row>17</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3582,7 +3652,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17350"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26112"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3669,13 +3739,13 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>25</xdr:row>
+          <xdr:row>21</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>26</xdr:row>
+          <xdr:row>22</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3691,7 +3761,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17351"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26113"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3732,15 +3802,15 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>7</xdr:col>
+          <xdr:col>6</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>25</xdr:row>
+          <xdr:row>21</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>9</xdr:col>
+          <xdr:col>8</xdr:col>
           <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>26</xdr:row>
+          <xdr:row>22</xdr:row>
           <xdr:rowOff>876300</xdr:rowOff>
         </xdr:to>
         <xdr:pic>
@@ -3756,7 +3826,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s17352"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26114"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3795,13 +3865,13 @@
   </mc:AlternateContent>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>876300</xdr:rowOff>
@@ -3856,23 +3926,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 7">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A47A4D9-D75D-4D66-96C3-449B2874EB89}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D012A3C-9297-C268-573B-B28B633BBB5A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3895,7 +3965,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="9220200" y="200025"/>
+          <a:off x="7391400" y="19926300"/>
           <a:ext cx="3705225" cy="5000625"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3917,206 +3987,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>19</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Picture 8">
+        <xdr:cNvPr id="5" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A134AF24-B6D7-4AB8-8EF4-B5842E828C94}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13525500" y="200025"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 11">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47C718FD-AAC6-481E-85D4-59F075E8B6E6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4924425" y="5562600"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="Picture 15">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0C9055C-53C5-4603-A264-B13B380B06C5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="619125" y="10925175"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Picture 16">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{36E5BE00-8060-08B8-1A46-54B06B9CFE18}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE9ED85E-3DA5-B5A1-932D-D8944C0DEEC1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4139,864 +4026,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4914900" y="16287750"/>
+          <a:off x="11087100" y="19926300"/>
           <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>371475</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Picture 17">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{342F9020-4A63-480A-9CF7-EBAC246CABE1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9210675" y="16278225"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>371475</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="Rectangle 20">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A516ECD-B904-7AC4-F9EC-16B12B828337}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9210675" y="21640800"/>
-          <a:ext cx="8010525" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1"/>
-        </a:solidFill>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-CA" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>481013</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>885825</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>604838</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="22" name="Picture 21">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8831CAF-765A-376B-CBC4-016EA1EE93D7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="10058400" y="22293263"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>1114425</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>481013</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>438150</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>604838</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="Picture 22">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06988B88-EB59-AB4A-D5B7-BDC424D1F0BA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11325225" y="22293263"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>666750</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>481013</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>604838</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="27" name="Picture 26">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FF812E4-B6D6-CECC-5B4A-73868D65CA98}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="12592050" y="22293263"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>481013</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>604838</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="32" name="Picture 31">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB7D0B06-DE13-1417-6EF2-6A6EF94310A1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13858875" y="22293263"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>609600</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>481013</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>1647825</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>604838</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="36" name="Picture 35">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A5315F95-4D46-66EE-C323-64D3F2E3321B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="15125700" y="22293263"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>1143000</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>828676</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>466725</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>1866901</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="41" name="Picture 40">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DD0C64F-AAA2-6E40-37DC-E20C00999C48}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11353800" y="23555326"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>669925</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>828676</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>107950</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>1866901</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="49" name="Picture 48">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3962F17-29F7-6F8E-C3A8-2D817E6F1ED5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="12595225" y="23555326"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>527050</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>2157414</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>1565275</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>852489</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="50" name="Picture 49">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C78D2958-1504-39E6-0311-D5797A816C59}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="10737850" y="24884064"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>95603</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>2157414</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>143228</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>852489</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="51" name="Picture 50">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8705D76C-A8C6-42B5-FFF9-4BDF5A67539D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="12020903" y="24884064"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>44450</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>828676</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>358775</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>1866901</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="55" name="Picture 54">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21652EF6-F28C-E8CD-6828-D68EA02E418F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13836650" y="23555326"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>388056</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>2157414</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>549981</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>852489</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="62" name="Picture 61">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{327DF20A-8EF9-89BE-E67E-B5B4D1744CFA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13303956" y="24884064"/>
-          <a:ext cx="1038225" cy="1038225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>70909</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>2157414</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>1109134</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>852489</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="63" name="Picture 62">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27A495BE-20CF-A560-F49E-CF01492E2C8C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="14587009" y="24884064"/>
-          <a:ext cx="1038225" cy="1038225"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5059,7 +4090,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="70">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="76">
   <rv s="0">
     <v>0</v>
     <v>4</v>
@@ -5338,6 +4369,30 @@
   </rv>
   <rv s="0">
     <v>51</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>52</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>53</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>54</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>55</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>56</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>57</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -5406,6 +4461,12 @@
   <rel r:id="rId50"/>
   <rel r:id="rId51"/>
   <rel r:id="rId52"/>
+  <rel r:id="rId53"/>
+  <rel r:id="rId54"/>
+  <rel r:id="rId55"/>
+  <rel r:id="rId56"/>
+  <rel r:id="rId57"/>
+  <rel r:id="rId58"/>
 </richValueRels>
 </file>
 
@@ -5675,55 +4736,55 @@
   <sheetPr>
     <tabColor theme="7"/>
   </sheetPr>
-  <dimension ref="B1:X30"/>
+  <dimension ref="A1:V27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="2.7109375" style="137" customWidth="1"/>
     <col min="2" max="2" width="4" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" customWidth="1"/>
     <col min="4" max="4" width="25.7109375" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" customWidth="1"/>
-    <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="8" max="8" width="4" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="25.7109375" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" customWidth="1"/>
-    <col min="12" max="12" width="4" customWidth="1"/>
-    <col min="14" max="14" width="4" customWidth="1"/>
+    <col min="6" max="7" width="4" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" customWidth="1"/>
+    <col min="11" max="12" width="4" customWidth="1"/>
+    <col min="13" max="13" width="10.85546875" customWidth="1"/>
+    <col min="14" max="14" width="25.7109375" customWidth="1"/>
     <col min="15" max="15" width="10.85546875" customWidth="1"/>
-    <col min="16" max="16" width="25.7109375" customWidth="1"/>
-    <col min="17" max="17" width="10.85546875" customWidth="1"/>
-    <col min="18" max="18" width="4" customWidth="1"/>
-    <col min="20" max="20" width="4" customWidth="1"/>
-    <col min="21" max="21" width="10.85546875" customWidth="1"/>
-    <col min="22" max="22" width="25.7109375" customWidth="1"/>
-    <col min="23" max="23" width="10.85546875" customWidth="1"/>
-    <col min="24" max="24" width="4" customWidth="1"/>
+    <col min="16" max="17" width="4" customWidth="1"/>
+    <col min="18" max="18" width="10.85546875" customWidth="1"/>
+    <col min="19" max="19" width="25.7109375" customWidth="1"/>
+    <col min="20" max="20" width="10.85546875" customWidth="1"/>
+    <col min="21" max="21" width="4" customWidth="1"/>
+    <col min="22" max="22" width="2.7109375" style="137" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="137" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="35"/>
       <c r="C2" s="36"/>
       <c r="D2" s="36"/>
       <c r="E2" s="36"/>
       <c r="F2" s="37"/>
-      <c r="H2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="48"/>
       <c r="I2" s="48"/>
       <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="49"/>
-      <c r="N2" s="1"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
       <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="59"/>
-      <c r="T2" s="5"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
-      <c r="X2" s="25"/>
+      <c r="P2" s="59"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="25"/>
     </row>
-    <row r="3" spans="2:24" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="138"/>
       <c r="B3" s="38"/>
       <c r="C3" s="39"/>
       <c r="D3" s="39" t="str">
@@ -5732,751 +4793,757 @@
       </c>
       <c r="E3" s="39"/>
       <c r="F3" s="40"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="85" t="str">
+      <c r="G3" s="50"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="85" t="str">
         <f>'Cards Src'!A3</f>
         <v>FROST NOVA</v>
       </c>
-      <c r="K3" s="51"/>
-      <c r="L3" s="52"/>
-      <c r="N3" s="60"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="62" t="str">
+      <c r="J3" s="51"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="62" t="str">
         <f>'Cards Src'!A4</f>
         <v>TIDAL WAVE</v>
       </c>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="63"/>
-      <c r="T3" s="26"/>
-      <c r="U3" s="27"/>
-      <c r="V3" s="33" t="str">
+      <c r="O3" s="61"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="27"/>
+      <c r="S3" s="33" t="str">
         <f>'Cards Src'!A5</f>
         <v>BRAMBLE SNARE</v>
       </c>
-      <c r="W3" s="27"/>
-      <c r="X3" s="28"/>
+      <c r="T3" s="27"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="138"/>
     </row>
-    <row r="4" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
-      <c r="C4" s="143" t="e" vm="1">
+      <c r="C4" s="152" t="e" vm="1">
         <f>'Cards Src'!E2</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="143"/>
-      <c r="E4" s="143"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
       <c r="F4" s="42"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="144" t="e" vm="2">
+      <c r="G4" s="53"/>
+      <c r="H4" s="157" t="e" vm="2">
         <f>'Cards Src'!E3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J4" s="144"/>
-      <c r="K4" s="144"/>
-      <c r="L4" s="54"/>
-      <c r="N4" s="116"/>
-      <c r="O4" s="149" t="e" vm="3">
+      <c r="I4" s="157"/>
+      <c r="J4" s="157"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="116"/>
+      <c r="M4" s="158" t="e" vm="3">
         <f>'Cards Src'!E4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P4" s="149"/>
-      <c r="Q4" s="149"/>
-      <c r="R4" s="64"/>
-      <c r="T4" s="7"/>
-      <c r="U4" s="150" t="e" vm="4">
+      <c r="N4" s="158"/>
+      <c r="O4" s="158"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="159" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V4" s="150"/>
-      <c r="W4" s="150"/>
-      <c r="X4" s="29"/>
+      <c r="S4" s="159"/>
+      <c r="T4" s="159"/>
+      <c r="U4" s="29"/>
     </row>
-    <row r="5" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
-      <c r="C5" s="137" t="str">
+      <c r="C5" s="153" t="str">
         <f>'Cards Src'!$C2</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
+      <c r="D5" s="153"/>
+      <c r="E5" s="153"/>
       <c r="F5" s="43"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="138" t="str">
+      <c r="G5" s="53"/>
+      <c r="H5" s="154" t="str">
         <f>'Cards Src'!$C3</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="J5" s="138"/>
-      <c r="K5" s="138"/>
-      <c r="L5" s="55"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="147" t="str">
+      <c r="I5" s="154"/>
+      <c r="J5" s="154"/>
+      <c r="K5" s="55"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="155" t="str">
         <f>'Cards Src'!C4</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="P5" s="147"/>
-      <c r="Q5" s="147"/>
-      <c r="R5" s="65"/>
-      <c r="T5" s="7"/>
-      <c r="U5" s="148" t="str">
+      <c r="N5" s="155"/>
+      <c r="O5" s="155"/>
+      <c r="P5" s="65"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="156" t="str">
         <f>'Cards Src'!C5</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="V5" s="148"/>
-      <c r="W5" s="148"/>
-      <c r="X5" s="30"/>
+      <c r="S5" s="156"/>
+      <c r="T5" s="156"/>
+      <c r="U5" s="30"/>
     </row>
-    <row r="6" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="44"/>
       <c r="C6" s="45"/>
       <c r="D6" s="45"/>
       <c r="E6" s="45"/>
       <c r="F6" s="46"/>
-      <c r="H6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="57"/>
       <c r="I6" s="57"/>
       <c r="J6" s="57"/>
-      <c r="K6" s="57"/>
-      <c r="L6" s="58"/>
-      <c r="N6" s="4"/>
+      <c r="K6" s="58"/>
+      <c r="L6" s="4"/>
+      <c r="M6" s="66"/>
+      <c r="N6" s="66"/>
       <c r="O6" s="66"/>
-      <c r="P6" s="66"/>
-      <c r="Q6" s="66"/>
-      <c r="R6" s="67"/>
-      <c r="T6" s="8"/>
-      <c r="U6" s="31"/>
-      <c r="V6" s="31"/>
-      <c r="W6" s="31"/>
-      <c r="X6" s="32"/>
+      <c r="P6" s="67"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="31"/>
+      <c r="S6" s="31"/>
+      <c r="T6" s="31"/>
+      <c r="U6" s="32"/>
     </row>
-    <row r="7" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="117"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="68"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="18"/>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="76"/>
-      <c r="T8" s="9"/>
-      <c r="U8" s="10"/>
-      <c r="V8" s="10"/>
-      <c r="W8" s="10"/>
-      <c r="X8" s="117"/>
+    <row r="7" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="117"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="68"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="76"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="117"/>
     </row>
-    <row r="9" spans="2:24" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="118"/>
-      <c r="C9" s="119"/>
-      <c r="D9" s="120" t="str">
+    <row r="8" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="138"/>
+      <c r="B8" s="118"/>
+      <c r="C8" s="119"/>
+      <c r="D8" s="120" t="str">
         <f>'Cards Src'!$A6</f>
         <v>LIGHTNING BOLT</v>
       </c>
-      <c r="E9" s="119"/>
-      <c r="F9" s="121"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="70"/>
-      <c r="J9" s="86" t="str">
+      <c r="E8" s="119"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="69"/>
+      <c r="H8" s="70"/>
+      <c r="I8" s="86" t="str">
         <f>'Cards Src'!A7</f>
         <v>BLACK HOLE</v>
       </c>
-      <c r="K9" s="70"/>
-      <c r="L9" s="71"/>
-      <c r="N9" s="77"/>
-      <c r="O9" s="78"/>
-      <c r="P9" s="79" t="str">
+      <c r="J8" s="70"/>
+      <c r="K8" s="71"/>
+      <c r="L8" s="77"/>
+      <c r="M8" s="78"/>
+      <c r="N8" s="79" t="str">
         <f>'Cards Src'!A8</f>
         <v>ASTRAL DAGGER</v>
       </c>
-      <c r="Q9" s="78"/>
-      <c r="R9" s="80"/>
-      <c r="T9" s="118"/>
-      <c r="U9" s="119"/>
-      <c r="V9" s="120" t="str">
+      <c r="O8" s="78"/>
+      <c r="P8" s="80"/>
+      <c r="Q8" s="118"/>
+      <c r="R8" s="119"/>
+      <c r="S8" s="120" t="str">
         <f>'Cards Src'!A9</f>
         <v>CHAIN LIGHTNING</v>
       </c>
-      <c r="W9" s="119"/>
-      <c r="X9" s="121"/>
+      <c r="T8" s="119"/>
+      <c r="U8" s="121"/>
+      <c r="V8" s="138"/>
     </row>
-    <row r="10" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="11"/>
+      <c r="C9" s="147" t="e" vm="5">
+        <f>'Cards Src'!E6</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D9" s="147"/>
+      <c r="E9" s="147"/>
+      <c r="F9" s="126"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="151" t="e" vm="6">
+        <f>'Cards Src'!E7</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I9" s="151"/>
+      <c r="J9" s="151"/>
+      <c r="K9" s="72"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="144" t="e" vm="7">
+        <f>'Cards Src'!E8</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="N9" s="144"/>
+      <c r="O9" s="144"/>
+      <c r="P9" s="81"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="147" t="e" vm="8">
+        <f>'Cards Src'!E9</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="S9" s="147"/>
+      <c r="T9" s="147"/>
+      <c r="U9" s="122"/>
+    </row>
+    <row r="10" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="11"/>
-      <c r="C10" s="146" t="e" vm="5">
-        <f>'Cards Src'!E6</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D10" s="146"/>
-      <c r="E10" s="146"/>
-      <c r="F10" s="126"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="152" t="e" vm="6">
-        <f>'Cards Src'!E7</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J10" s="152"/>
-      <c r="K10" s="152"/>
-      <c r="L10" s="72"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="145" t="e" vm="7">
-        <f>'Cards Src'!E8</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="P10" s="145"/>
-      <c r="Q10" s="145"/>
-      <c r="R10" s="81"/>
-      <c r="T10" s="11"/>
-      <c r="U10" s="146" t="e" vm="8">
-        <f>'Cards Src'!E9</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="V10" s="146"/>
-      <c r="W10" s="146"/>
-      <c r="X10" s="122"/>
-    </row>
-    <row r="11" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="11"/>
-      <c r="C11" s="140" t="str">
+      <c r="C10" s="148" t="str">
         <f>'Cards Src'!$C6</f>
         <v>Casts a bolt of lightning</v>
       </c>
-      <c r="D11" s="140"/>
-      <c r="E11" s="140"/>
-      <c r="F11" s="123"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="151" t="str">
+      <c r="D10" s="148"/>
+      <c r="E10" s="148"/>
+      <c r="F10" s="123"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="149" t="str">
         <f>'Cards Src'!$C7</f>
         <v>Vacuums in nearby enemies</v>
       </c>
-      <c r="J11" s="151"/>
-      <c r="K11" s="151"/>
-      <c r="L11" s="73"/>
-      <c r="N11" s="19"/>
-      <c r="O11" s="139" t="str">
+      <c r="I10" s="149"/>
+      <c r="J10" s="149"/>
+      <c r="K10" s="73"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="150" t="str">
         <f>'Cards Src'!C8</f>
         <v>Flies to the nearest enemy in vision</v>
       </c>
-      <c r="P11" s="139"/>
-      <c r="Q11" s="139"/>
-      <c r="R11" s="82"/>
-      <c r="T11" s="11"/>
-      <c r="U11" s="140" t="str">
+      <c r="N10" s="150"/>
+      <c r="O10" s="150"/>
+      <c r="P10" s="82"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="148" t="str">
         <f>'Cards Src'!C9</f>
         <v>Casts a tracking bolt of lightning that can chain to close enemies</v>
       </c>
-      <c r="V11" s="140"/>
-      <c r="W11" s="140"/>
-      <c r="X11" s="123"/>
+      <c r="S10" s="148"/>
+      <c r="T10" s="148"/>
+      <c r="U10" s="123"/>
     </row>
-    <row r="12" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="12"/>
-      <c r="C12" s="124"/>
-      <c r="D12" s="124"/>
-      <c r="E12" s="124"/>
-      <c r="F12" s="125"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="74"/>
-      <c r="J12" s="74"/>
-      <c r="K12" s="74"/>
-      <c r="L12" s="75"/>
-      <c r="N12" s="20"/>
-      <c r="O12" s="83"/>
-      <c r="P12" s="83"/>
-      <c r="Q12" s="83"/>
-      <c r="R12" s="84"/>
-      <c r="T12" s="12"/>
-      <c r="U12" s="124"/>
-      <c r="V12" s="124"/>
-      <c r="W12" s="124"/>
-      <c r="X12" s="125"/>
+    <row r="11" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="12"/>
+      <c r="C11" s="124"/>
+      <c r="D11" s="124"/>
+      <c r="E11" s="124"/>
+      <c r="F11" s="125"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="74"/>
+      <c r="I11" s="74"/>
+      <c r="J11" s="74"/>
+      <c r="K11" s="75"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="83"/>
+      <c r="N11" s="83"/>
+      <c r="O11" s="83"/>
+      <c r="P11" s="84"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="124"/>
+      <c r="S11" s="124"/>
+      <c r="T11" s="124"/>
+      <c r="U11" s="125"/>
     </row>
-    <row r="13" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="17"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="76"/>
-      <c r="H14" s="100"/>
-      <c r="I14" s="101"/>
-      <c r="J14" s="101"/>
-      <c r="K14" s="101"/>
-      <c r="L14" s="102"/>
-      <c r="N14" s="100"/>
-      <c r="O14" s="101"/>
-      <c r="P14" s="101"/>
-      <c r="Q14" s="101"/>
-      <c r="R14" s="102"/>
-      <c r="T14" s="100"/>
-      <c r="U14" s="101"/>
-      <c r="V14" s="101"/>
-      <c r="W14" s="101"/>
-      <c r="X14" s="102"/>
+    <row r="12" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="17"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="76"/>
+      <c r="G12" s="100"/>
+      <c r="H12" s="101"/>
+      <c r="I12" s="101"/>
+      <c r="J12" s="101"/>
+      <c r="K12" s="102"/>
+      <c r="L12" s="100"/>
+      <c r="M12" s="101"/>
+      <c r="N12" s="101"/>
+      <c r="O12" s="101"/>
+      <c r="P12" s="102"/>
+      <c r="Q12" s="100"/>
+      <c r="R12" s="101"/>
+      <c r="S12" s="101"/>
+      <c r="T12" s="101"/>
+      <c r="U12" s="102"/>
     </row>
-    <row r="15" spans="2:24" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="77"/>
-      <c r="C15" s="78"/>
-      <c r="D15" s="79" t="str">
+    <row r="13" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="138"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="78"/>
+      <c r="D13" s="79" t="str">
         <f>'Cards Src'!$A10</f>
         <v>DIVINE JUDGEMENT</v>
       </c>
-      <c r="E15" s="78"/>
-      <c r="F15" s="80"/>
-      <c r="H15" s="103"/>
-      <c r="I15" s="104"/>
-      <c r="J15" s="105" t="str">
+      <c r="E13" s="78"/>
+      <c r="F13" s="80"/>
+      <c r="G13" s="103"/>
+      <c r="H13" s="104"/>
+      <c r="I13" s="105" t="str">
         <f>'Cards Src'!A11</f>
         <v>HASTE</v>
       </c>
-      <c r="K15" s="104"/>
-      <c r="L15" s="106"/>
-      <c r="N15" s="103"/>
-      <c r="O15" s="104"/>
-      <c r="P15" s="105" t="str">
+      <c r="J13" s="104"/>
+      <c r="K13" s="106"/>
+      <c r="L13" s="103"/>
+      <c r="M13" s="104"/>
+      <c r="N13" s="105" t="str">
         <f>'Cards Src'!A12</f>
         <v>HINDER</v>
       </c>
-      <c r="Q15" s="104"/>
-      <c r="R15" s="106"/>
-      <c r="T15" s="103"/>
-      <c r="U15" s="104"/>
-      <c r="V15" s="114" t="str">
+      <c r="O13" s="104"/>
+      <c r="P13" s="106"/>
+      <c r="Q13" s="103"/>
+      <c r="R13" s="104"/>
+      <c r="S13" s="114" t="str">
         <f>'Cards Src'!A13</f>
         <v>MULLIGAN</v>
       </c>
-      <c r="W15" s="104"/>
-      <c r="X15" s="106"/>
+      <c r="T13" s="104"/>
+      <c r="U13" s="106"/>
+      <c r="V13" s="138"/>
     </row>
-    <row r="16" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="19"/>
-      <c r="C16" s="145" t="e" vm="9">
+    <row r="14" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="19"/>
+      <c r="C14" s="144" t="e" vm="9">
         <f>'Cards Src'!E10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D16" s="145"/>
-      <c r="E16" s="145"/>
-      <c r="F16" s="81"/>
-      <c r="H16" s="107"/>
-      <c r="I16" s="154" t="e" vm="10">
+      <c r="D14" s="144"/>
+      <c r="E14" s="144"/>
+      <c r="F14" s="81"/>
+      <c r="G14" s="107"/>
+      <c r="H14" s="146" t="e" vm="10">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J16" s="154"/>
-      <c r="K16" s="154"/>
-      <c r="L16" s="108"/>
-      <c r="N16" s="107"/>
-      <c r="O16" s="141" t="e" vm="11">
+      <c r="I14" s="146"/>
+      <c r="J14" s="146"/>
+      <c r="K14" s="108"/>
+      <c r="L14" s="107"/>
+      <c r="M14" s="139" t="e" vm="11">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P16" s="141"/>
-      <c r="Q16" s="141"/>
-      <c r="R16" s="108"/>
-      <c r="T16" s="107"/>
-      <c r="U16" s="141" t="e" vm="12">
+      <c r="N14" s="139"/>
+      <c r="O14" s="139"/>
+      <c r="P14" s="108"/>
+      <c r="Q14" s="107"/>
+      <c r="R14" s="139" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V16" s="141"/>
-      <c r="W16" s="141"/>
-      <c r="X16" s="108"/>
+      <c r="S14" s="139"/>
+      <c r="T14" s="139"/>
+      <c r="U14" s="108"/>
     </row>
-    <row r="17" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="19"/>
-      <c r="C17" s="153" t="str">
+    <row r="15" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="19"/>
+      <c r="C15" s="145" t="str">
         <f>'Cards Src'!$C10</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D17" s="153"/>
-      <c r="E17" s="153"/>
-      <c r="F17" s="82"/>
-      <c r="H17" s="107"/>
-      <c r="I17" s="142" t="str">
+      <c r="D15" s="145"/>
+      <c r="E15" s="145"/>
+      <c r="F15" s="82"/>
+      <c r="G15" s="107"/>
+      <c r="H15" s="140" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="J17" s="142"/>
-      <c r="K17" s="142"/>
-      <c r="L17" s="110"/>
-      <c r="N17" s="107"/>
-      <c r="O17" s="142" t="str">
+      <c r="I15" s="140"/>
+      <c r="J15" s="140"/>
+      <c r="K15" s="110"/>
+      <c r="L15" s="107"/>
+      <c r="M15" s="140" t="str">
         <f>'Cards Src'!C12</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="P17" s="142"/>
-      <c r="Q17" s="142"/>
-      <c r="R17" s="110"/>
-      <c r="T17" s="107"/>
-      <c r="U17" s="142" t="str">
+      <c r="N15" s="140"/>
+      <c r="O15" s="140"/>
+      <c r="P15" s="110"/>
+      <c r="Q15" s="107"/>
+      <c r="R15" s="140" t="str">
         <f>'Cards Src'!C13</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="V17" s="142"/>
-      <c r="W17" s="142"/>
-      <c r="X17" s="110"/>
+      <c r="S15" s="140"/>
+      <c r="T15" s="140"/>
+      <c r="U15" s="110"/>
     </row>
-    <row r="18" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="20"/>
-      <c r="C18" s="83"/>
-      <c r="D18" s="83"/>
-      <c r="E18" s="83"/>
-      <c r="F18" s="84"/>
-      <c r="H18" s="111"/>
-      <c r="I18" s="112"/>
-      <c r="J18" s="112"/>
-      <c r="K18" s="112"/>
-      <c r="L18" s="113"/>
-      <c r="N18" s="111"/>
-      <c r="O18" s="112"/>
-      <c r="P18" s="112"/>
-      <c r="Q18" s="112"/>
-      <c r="R18" s="113"/>
-      <c r="T18" s="111"/>
-      <c r="U18" s="112"/>
-      <c r="V18" s="112"/>
-      <c r="W18" s="112"/>
-      <c r="X18" s="113"/>
+    <row r="16" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="20"/>
+      <c r="C16" s="83"/>
+      <c r="D16" s="83"/>
+      <c r="E16" s="83"/>
+      <c r="F16" s="84"/>
+      <c r="G16" s="111"/>
+      <c r="H16" s="112"/>
+      <c r="I16" s="112"/>
+      <c r="J16" s="112"/>
+      <c r="K16" s="113"/>
+      <c r="L16" s="111"/>
+      <c r="M16" s="112"/>
+      <c r="N16" s="112"/>
+      <c r="O16" s="112"/>
+      <c r="P16" s="113"/>
+      <c r="Q16" s="111"/>
+      <c r="R16" s="112"/>
+      <c r="S16" s="112"/>
+      <c r="T16" s="112"/>
+      <c r="U16" s="113"/>
     </row>
-    <row r="19" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="100"/>
-      <c r="C20" s="101"/>
-      <c r="D20" s="101"/>
-      <c r="E20" s="101"/>
-      <c r="F20" s="102"/>
-      <c r="H20" s="100"/>
-      <c r="I20" s="101"/>
-      <c r="J20" s="101"/>
-      <c r="K20" s="101"/>
-      <c r="L20" s="102"/>
-      <c r="N20" s="100"/>
-      <c r="O20" s="101"/>
-      <c r="P20" s="101"/>
-      <c r="Q20" s="101"/>
-      <c r="R20" s="102"/>
-      <c r="T20" s="100"/>
-      <c r="U20" s="101"/>
-      <c r="V20" s="101"/>
-      <c r="W20" s="101"/>
-      <c r="X20" s="102"/>
+    <row r="17" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="100"/>
+      <c r="C17" s="101"/>
+      <c r="D17" s="101"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="102"/>
+      <c r="G17" s="100"/>
+      <c r="H17" s="101"/>
+      <c r="I17" s="101"/>
+      <c r="J17" s="101"/>
+      <c r="K17" s="102"/>
+      <c r="L17" s="100"/>
+      <c r="M17" s="101"/>
+      <c r="N17" s="101"/>
+      <c r="O17" s="101"/>
+      <c r="P17" s="102"/>
+      <c r="Q17" s="100"/>
+      <c r="R17" s="101"/>
+      <c r="S17" s="101"/>
+      <c r="T17" s="101"/>
+      <c r="U17" s="102"/>
     </row>
-    <row r="21" spans="2:24" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="103"/>
-      <c r="C21" s="104"/>
-      <c r="D21" s="109" t="str">
+    <row r="18" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="138"/>
+      <c r="B18" s="103"/>
+      <c r="C18" s="104"/>
+      <c r="D18" s="109" t="str">
         <f>'Cards Src'!$A14</f>
         <v>BUT WAIT, THERE'S MORE</v>
       </c>
-      <c r="E21" s="104"/>
-      <c r="F21" s="106"/>
-      <c r="H21" s="103"/>
-      <c r="I21" s="104"/>
-      <c r="J21" s="115" t="str">
+      <c r="E18" s="104"/>
+      <c r="F18" s="106"/>
+      <c r="G18" s="103"/>
+      <c r="H18" s="104"/>
+      <c r="I18" s="115" t="str">
         <f>'Cards Src'!A15</f>
         <v>MANA SHIELD</v>
       </c>
-      <c r="K21" s="104"/>
-      <c r="L21" s="106"/>
-      <c r="N21" s="103"/>
-      <c r="O21" s="104"/>
-      <c r="P21" s="115" t="str">
+      <c r="J18" s="104"/>
+      <c r="K18" s="106"/>
+      <c r="L18" s="103"/>
+      <c r="M18" s="104"/>
+      <c r="N18" s="115" t="str">
         <f>'Cards Src'!A16</f>
         <v>RUNAWAY BULL</v>
       </c>
-      <c r="Q21" s="104"/>
-      <c r="R21" s="106"/>
-      <c r="T21" s="103"/>
-      <c r="U21" s="104"/>
-      <c r="V21" s="128" t="str">
+      <c r="O18" s="104"/>
+      <c r="P18" s="106"/>
+      <c r="Q18" s="103"/>
+      <c r="R18" s="104"/>
+      <c r="S18" s="128" t="str">
         <f>'Cards Src'!A17</f>
         <v>HOLY BLADE</v>
       </c>
-      <c r="W21" s="104"/>
-      <c r="X21" s="106"/>
+      <c r="T18" s="104"/>
+      <c r="U18" s="106"/>
+      <c r="V18" s="138"/>
     </row>
-    <row r="22" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="107"/>
-      <c r="C22" s="141" t="e" vm="13">
+    <row r="19" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="107"/>
+      <c r="C19" s="139" t="e" vm="13">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D22" s="141"/>
-      <c r="E22" s="141"/>
-      <c r="F22" s="108"/>
-      <c r="H22" s="107"/>
-      <c r="I22" s="141" t="e" vm="14">
+      <c r="D19" s="139"/>
+      <c r="E19" s="139"/>
+      <c r="F19" s="108"/>
+      <c r="G19" s="107"/>
+      <c r="H19" s="139" t="e" vm="14">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J22" s="141"/>
-      <c r="K22" s="141"/>
-      <c r="L22" s="108"/>
-      <c r="N22" s="107"/>
-      <c r="O22" s="141" t="e" vm="15">
+      <c r="I19" s="139"/>
+      <c r="J19" s="139"/>
+      <c r="K19" s="108"/>
+      <c r="L19" s="107"/>
+      <c r="M19" s="139" t="e" vm="15">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="P22" s="141"/>
-      <c r="Q22" s="141"/>
-      <c r="R22" s="108"/>
-      <c r="T22" s="107"/>
-      <c r="U22" s="141" t="e" vm="16">
+      <c r="N19" s="139"/>
+      <c r="O19" s="139"/>
+      <c r="P19" s="108"/>
+      <c r="Q19" s="107"/>
+      <c r="R19" s="139" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="V22" s="141"/>
-      <c r="W22" s="141"/>
-      <c r="X22" s="108"/>
+      <c r="S19" s="139"/>
+      <c r="T19" s="139"/>
+      <c r="U19" s="108"/>
     </row>
-    <row r="23" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="107"/>
-      <c r="C23" s="142" t="str">
+    <row r="20" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="107"/>
+      <c r="C20" s="140" t="str">
         <f>'Cards Src'!$C14</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D23" s="142"/>
-      <c r="E23" s="142"/>
-      <c r="F23" s="110"/>
-      <c r="H23" s="107"/>
-      <c r="I23" s="142" t="str">
+      <c r="D20" s="140"/>
+      <c r="E20" s="140"/>
+      <c r="F20" s="110"/>
+      <c r="G20" s="107"/>
+      <c r="H20" s="140" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="J23" s="142"/>
-      <c r="K23" s="142"/>
-      <c r="L23" s="110"/>
-      <c r="N23" s="107"/>
-      <c r="O23" s="155" t="str">
+      <c r="I20" s="140"/>
+      <c r="J20" s="140"/>
+      <c r="K20" s="110"/>
+      <c r="L20" s="107"/>
+      <c r="M20" s="143" t="str">
         <f>'Cards Src'!C16</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="P23" s="155"/>
-      <c r="Q23" s="155"/>
-      <c r="R23" s="110"/>
-      <c r="T23" s="107"/>
-      <c r="U23" s="142" t="str">
+      <c r="N20" s="143"/>
+      <c r="O20" s="143"/>
+      <c r="P20" s="110"/>
+      <c r="Q20" s="107"/>
+      <c r="R20" s="140" t="str">
         <f>'Cards Src'!C17</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="V23" s="142"/>
-      <c r="W23" s="142"/>
-      <c r="X23" s="110"/>
+      <c r="S20" s="140"/>
+      <c r="T20" s="140"/>
+      <c r="U20" s="110"/>
     </row>
-    <row r="24" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="111"/>
-      <c r="C24" s="112"/>
-      <c r="D24" s="112"/>
-      <c r="E24" s="112"/>
-      <c r="F24" s="113"/>
-      <c r="H24" s="111"/>
-      <c r="I24" s="112"/>
-      <c r="J24" s="112"/>
-      <c r="K24" s="112"/>
-      <c r="L24" s="113"/>
-      <c r="N24" s="111"/>
-      <c r="O24" s="112"/>
-      <c r="P24" s="112"/>
-      <c r="Q24" s="112"/>
-      <c r="R24" s="113"/>
-      <c r="T24" s="111"/>
-      <c r="U24" s="112"/>
-      <c r="V24" s="112"/>
-      <c r="W24" s="112"/>
-      <c r="X24" s="113"/>
+    <row r="21" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="111"/>
+      <c r="C21" s="112"/>
+      <c r="D21" s="112"/>
+      <c r="E21" s="112"/>
+      <c r="F21" s="113"/>
+      <c r="G21" s="111"/>
+      <c r="H21" s="112"/>
+      <c r="I21" s="112"/>
+      <c r="J21" s="112"/>
+      <c r="K21" s="113"/>
+      <c r="L21" s="111"/>
+      <c r="M21" s="112"/>
+      <c r="N21" s="112"/>
+      <c r="O21" s="112"/>
+      <c r="P21" s="113"/>
+      <c r="Q21" s="111"/>
+      <c r="R21" s="112"/>
+      <c r="S21" s="112"/>
+      <c r="T21" s="112"/>
+      <c r="U21" s="113"/>
     </row>
-    <row r="25" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="2:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="100"/>
-      <c r="C26" s="101"/>
-      <c r="D26" s="101"/>
-      <c r="E26" s="101"/>
-      <c r="F26" s="102"/>
-      <c r="H26" s="100"/>
-      <c r="I26" s="101"/>
-      <c r="J26" s="101"/>
-      <c r="K26" s="101"/>
-      <c r="L26" s="102"/>
-      <c r="N26" s="87"/>
-      <c r="O26" s="88"/>
-      <c r="P26" s="88"/>
-      <c r="Q26" s="88"/>
-      <c r="R26" s="89"/>
-      <c r="T26" s="87"/>
-      <c r="U26" s="88"/>
-      <c r="V26" s="88"/>
-      <c r="W26" s="88"/>
-      <c r="X26" s="89"/>
+    <row r="22" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="100"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
+      <c r="E22" s="101"/>
+      <c r="F22" s="102"/>
+      <c r="G22" s="100"/>
+      <c r="H22" s="101"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="101"/>
+      <c r="K22" s="102"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="88"/>
+      <c r="N22" s="88"/>
+      <c r="O22" s="88"/>
+      <c r="P22" s="89"/>
+      <c r="Q22" s="87"/>
+      <c r="R22" s="88"/>
+      <c r="S22" s="88"/>
+      <c r="T22" s="88"/>
+      <c r="U22" s="89"/>
     </row>
-    <row r="27" spans="2:24" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="103"/>
-      <c r="C27" s="104"/>
-      <c r="D27" s="105" t="str">
+    <row r="23" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="138"/>
+      <c r="B23" s="103"/>
+      <c r="C23" s="104"/>
+      <c r="D23" s="105" t="str">
         <f>'Cards Src'!$A18</f>
         <v>RECALL</v>
       </c>
-      <c r="E27" s="104"/>
-      <c r="F27" s="106"/>
-      <c r="H27" s="103"/>
-      <c r="I27" s="104"/>
-      <c r="J27" s="105" t="str">
+      <c r="E23" s="104"/>
+      <c r="F23" s="106"/>
+      <c r="G23" s="103"/>
+      <c r="H23" s="104"/>
+      <c r="I23" s="105" t="str">
         <f>'Cards Src'!A19</f>
         <v>GREED</v>
       </c>
-      <c r="K27" s="104"/>
-      <c r="L27" s="106"/>
-      <c r="N27" s="90"/>
-      <c r="O27" s="91"/>
-      <c r="P27" s="92">
+      <c r="J23" s="104"/>
+      <c r="K23" s="106"/>
+      <c r="L23" s="90"/>
+      <c r="M23" s="91"/>
+      <c r="N23" s="92">
         <f>'Cards Src'!A20</f>
         <v>0</v>
       </c>
-      <c r="Q27" s="91"/>
-      <c r="R27" s="93"/>
-      <c r="T27" s="90"/>
-      <c r="U27" s="91"/>
-      <c r="V27" s="92">
+      <c r="O23" s="91"/>
+      <c r="P23" s="93"/>
+      <c r="Q23" s="90"/>
+      <c r="R23" s="91"/>
+      <c r="S23" s="92">
         <f>'Cards Src'!A21</f>
         <v>0</v>
       </c>
-      <c r="W27" s="91"/>
-      <c r="X27" s="93"/>
+      <c r="T23" s="91"/>
+      <c r="U23" s="93"/>
+      <c r="V23" s="138"/>
     </row>
-    <row r="28" spans="2:24" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="107"/>
-      <c r="C28" s="141" t="e" vm="17">
+    <row r="24" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="107"/>
+      <c r="C24" s="139" t="e" vm="17">
         <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D28" s="141"/>
-      <c r="E28" s="141"/>
-      <c r="F28" s="108"/>
-      <c r="H28" s="107"/>
-      <c r="I28" s="141" t="e" vm="18">
+      <c r="D24" s="139"/>
+      <c r="E24" s="139"/>
+      <c r="F24" s="108"/>
+      <c r="G24" s="107"/>
+      <c r="H24" s="139" t="e" vm="18">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="J28" s="141"/>
-      <c r="K28" s="141"/>
-      <c r="L28" s="108"/>
-      <c r="N28" s="94"/>
-      <c r="O28" s="157">
+      <c r="I24" s="139"/>
+      <c r="J24" s="139"/>
+      <c r="K24" s="108"/>
+      <c r="L24" s="94"/>
+      <c r="M24" s="142">
         <f>'Cards Src'!E20</f>
         <v>0</v>
       </c>
-      <c r="P28" s="157"/>
-      <c r="Q28" s="157"/>
-      <c r="R28" s="95"/>
-      <c r="T28" s="94"/>
-      <c r="U28" s="157">
+      <c r="N24" s="142"/>
+      <c r="O24" s="142"/>
+      <c r="P24" s="95"/>
+      <c r="Q24" s="94"/>
+      <c r="R24" s="142">
         <f xml:space="preserve"> 'Cards Src'!E21</f>
         <v>0</v>
       </c>
-      <c r="V28" s="157"/>
-      <c r="W28" s="157"/>
-      <c r="X28" s="95"/>
+      <c r="S24" s="142"/>
+      <c r="T24" s="142"/>
+      <c r="U24" s="95"/>
     </row>
-    <row r="29" spans="2:24" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="107"/>
-      <c r="C29" s="142" t="str">
+    <row r="25" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="107"/>
+      <c r="C25" s="140" t="str">
         <f>'Cards Src'!$C18</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D29" s="142"/>
-      <c r="E29" s="142"/>
-      <c r="F29" s="110"/>
-      <c r="H29" s="107"/>
-      <c r="I29" s="142" t="str">
+      <c r="D25" s="140"/>
+      <c r="E25" s="140"/>
+      <c r="F25" s="110"/>
+      <c r="G25" s="107"/>
+      <c r="H25" s="140" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="J29" s="142"/>
-      <c r="K29" s="142"/>
-      <c r="L29" s="110"/>
-      <c r="N29" s="94"/>
-      <c r="O29" s="156">
+      <c r="I25" s="140"/>
+      <c r="J25" s="140"/>
+      <c r="K25" s="110"/>
+      <c r="L25" s="94"/>
+      <c r="M25" s="141">
         <f>'Cards Src'!C20</f>
         <v>0</v>
       </c>
-      <c r="P29" s="156"/>
-      <c r="Q29" s="156"/>
-      <c r="R29" s="96"/>
-      <c r="T29" s="94"/>
-      <c r="U29" s="156">
+      <c r="N25" s="141"/>
+      <c r="O25" s="141"/>
+      <c r="P25" s="96"/>
+      <c r="Q25" s="94"/>
+      <c r="R25" s="141">
         <f>'Cards Src'!C21</f>
         <v>0</v>
       </c>
-      <c r="V29" s="156"/>
-      <c r="W29" s="156"/>
-      <c r="X29" s="96"/>
+      <c r="S25" s="141"/>
+      <c r="T25" s="141"/>
+      <c r="U25" s="96"/>
     </row>
-    <row r="30" spans="2:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="111"/>
-      <c r="C30" s="112"/>
-      <c r="D30" s="112"/>
-      <c r="E30" s="112"/>
-      <c r="F30" s="113"/>
-      <c r="H30" s="111"/>
-      <c r="I30" s="112"/>
-      <c r="J30" s="112"/>
-      <c r="K30" s="112"/>
-      <c r="L30" s="113"/>
-      <c r="N30" s="97"/>
-      <c r="O30" s="98"/>
-      <c r="P30" s="98"/>
-      <c r="Q30" s="98"/>
-      <c r="R30" s="99"/>
-      <c r="T30" s="97"/>
-      <c r="U30" s="98"/>
-      <c r="V30" s="98"/>
-      <c r="W30" s="98"/>
-      <c r="X30" s="99"/>
+    <row r="26" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="111"/>
+      <c r="C26" s="112"/>
+      <c r="D26" s="112"/>
+      <c r="E26" s="112"/>
+      <c r="F26" s="113"/>
+      <c r="G26" s="111"/>
+      <c r="H26" s="112"/>
+      <c r="I26" s="112"/>
+      <c r="J26" s="112"/>
+      <c r="K26" s="113"/>
+      <c r="L26" s="97"/>
+      <c r="M26" s="98"/>
+      <c r="N26" s="98"/>
+      <c r="O26" s="98"/>
+      <c r="P26" s="99"/>
+      <c r="Q26" s="97"/>
+      <c r="R26" s="98"/>
+      <c r="S26" s="98"/>
+      <c r="T26" s="98"/>
+      <c r="U26" s="99"/>
     </row>
+    <row r="27" spans="1:22" s="137" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="U29:W29"/>
-    <mergeCell ref="I28:K28"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="U28:W28"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="U23:W23"/>
-    <mergeCell ref="I22:K22"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="U22:W22"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="U17:W17"/>
-    <mergeCell ref="I16:K16"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="U16:W16"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="O11:Q11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="O10:Q10"/>
-    <mergeCell ref="U10:W10"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="O5:Q5"/>
-    <mergeCell ref="U5:W5"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="U4:W4"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="R5:T5"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="M4:O4"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="R10:T10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="R9:T9"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="R15:T15"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="R14:T14"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="R20:T20"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="R25:T25"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="R24:T24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -7047,68 +6114,113 @@
   <sheetPr>
     <tabColor theme="4" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.42578125" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="55.42578125" style="131" customWidth="1"/>
+    <col min="4" max="12" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="98.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="130"/>
-      <c r="D1" s="21"/>
+      <c r="D1" s="21" t="e" vm="64">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E1" t="e" vm="65">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F1" s="21" t="e" vm="66">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G1" t="e" vm="67">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H1" s="21" t="e" vm="68">
+        <v>#VALUE!</v>
+      </c>
+      <c r="I1" t="e" vm="69">
+        <v>#VALUE!</v>
+      </c>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
     </row>
-    <row r="2" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="e" vm="64">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C2" s="131" t="e" vm="65">
+    <row r="2" spans="1:12" ht="393" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="e" vm="70">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C2" s="131" t="e" vm="71">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>55</v>
       </c>
       <c r="C3" s="130"/>
       <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
     </row>
-    <row r="4" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" t="e" vm="66">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C4" s="131" t="e" vm="67">
+    <row r="4" spans="1:12" ht="393" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="e" vm="72">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C4" s="131" t="e" vm="73">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C5" s="130"/>
       <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
     </row>
-    <row r="6" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" t="e" vm="68">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C6" s="131" t="e" vm="69">
+    <row r="6" spans="1:12" ht="393" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="e" vm="74">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C6" s="131" t="e" vm="75">
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
         <v>58</v>
       </c>
       <c r="C7" s="130"/>
       <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
     </row>
-    <row r="8" spans="1:4" ht="393" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="e" vm="70">
+    <row r="8" spans="1:12" ht="393" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="e" vm="76">
         <v>#VALUE!</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Art - Tidal Wave
Art for the Tidal Wave attack card
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA34AD08-B85F-4F96-AB2E-4E65F65B978D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E20631-CBD2-4F03-A256-8CB329EF09FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1585,67 +1585,67 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2807,7 +2807,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26099"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26115"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2872,7 +2872,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26100"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26116"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2937,7 +2937,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26101"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26117"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3002,7 +3002,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26102"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26118"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3067,7 +3067,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26103"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26119"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3132,7 +3132,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26104"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26120"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3197,7 +3197,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26105"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26121"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3262,7 +3262,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26106"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26122"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3327,7 +3327,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26107"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26123"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3392,7 +3392,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26108"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26124"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3457,7 +3457,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26109"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26125"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3522,7 +3522,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26110"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26126"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3587,7 +3587,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26111"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26127"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3652,7 +3652,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26112"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26128"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3761,7 +3761,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26113"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26129"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3826,7 +3826,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26114"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26130"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -4821,70 +4821,70 @@
     </row>
     <row r="4" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
-      <c r="C4" s="152" t="e" vm="1">
+      <c r="C4" s="139" t="e" vm="1">
         <f>'Cards Src'!E2</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="152"/>
-      <c r="E4" s="152"/>
+      <c r="D4" s="139"/>
+      <c r="E4" s="139"/>
       <c r="F4" s="42"/>
       <c r="G4" s="53"/>
-      <c r="H4" s="157" t="e" vm="2">
+      <c r="H4" s="144" t="e" vm="2">
         <f>'Cards Src'!E3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I4" s="157"/>
-      <c r="J4" s="157"/>
+      <c r="I4" s="144"/>
+      <c r="J4" s="144"/>
       <c r="K4" s="54"/>
       <c r="L4" s="116"/>
-      <c r="M4" s="158" t="e" vm="3">
+      <c r="M4" s="145" t="e" vm="3">
         <f>'Cards Src'!E4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N4" s="158"/>
-      <c r="O4" s="158"/>
+      <c r="N4" s="145"/>
+      <c r="O4" s="145"/>
       <c r="P4" s="64"/>
       <c r="Q4" s="7"/>
-      <c r="R4" s="159" t="e" vm="4">
+      <c r="R4" s="146" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S4" s="159"/>
-      <c r="T4" s="159"/>
+      <c r="S4" s="146"/>
+      <c r="T4" s="146"/>
       <c r="U4" s="29"/>
     </row>
     <row r="5" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
-      <c r="C5" s="153" t="str">
+      <c r="C5" s="140" t="str">
         <f>'Cards Src'!$C2</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="153"/>
-      <c r="E5" s="153"/>
+      <c r="D5" s="140"/>
+      <c r="E5" s="140"/>
       <c r="F5" s="43"/>
       <c r="G5" s="53"/>
-      <c r="H5" s="154" t="str">
+      <c r="H5" s="141" t="str">
         <f>'Cards Src'!$C3</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="I5" s="154"/>
-      <c r="J5" s="154"/>
+      <c r="I5" s="141"/>
+      <c r="J5" s="141"/>
       <c r="K5" s="55"/>
       <c r="L5" s="3"/>
-      <c r="M5" s="155" t="str">
+      <c r="M5" s="142" t="str">
         <f>'Cards Src'!C4</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="N5" s="155"/>
-      <c r="O5" s="155"/>
+      <c r="N5" s="142"/>
+      <c r="O5" s="142"/>
       <c r="P5" s="65"/>
       <c r="Q5" s="7"/>
-      <c r="R5" s="156" t="str">
+      <c r="R5" s="143" t="str">
         <f>'Cards Src'!C5</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="S5" s="156"/>
-      <c r="T5" s="156"/>
+      <c r="S5" s="143"/>
+      <c r="T5" s="143"/>
       <c r="U5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4985,12 +4985,12 @@
       <c r="J9" s="151"/>
       <c r="K9" s="72"/>
       <c r="L9" s="19"/>
-      <c r="M9" s="144" t="e" vm="7">
+      <c r="M9" s="152" t="e" vm="7">
         <f>'Cards Src'!E8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N9" s="144"/>
-      <c r="O9" s="144"/>
+      <c r="N9" s="152"/>
+      <c r="O9" s="152"/>
       <c r="P9" s="81"/>
       <c r="Q9" s="11"/>
       <c r="R9" s="147" t="e" vm="8">
@@ -5117,70 +5117,70 @@
     </row>
     <row r="14" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="19"/>
-      <c r="C14" s="144" t="e" vm="9">
+      <c r="C14" s="152" t="e" vm="9">
         <f>'Cards Src'!E10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D14" s="144"/>
-      <c r="E14" s="144"/>
+      <c r="D14" s="152"/>
+      <c r="E14" s="152"/>
       <c r="F14" s="81"/>
       <c r="G14" s="107"/>
-      <c r="H14" s="146" t="e" vm="10">
+      <c r="H14" s="155" t="e" vm="10">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I14" s="146"/>
-      <c r="J14" s="146"/>
+      <c r="I14" s="155"/>
+      <c r="J14" s="155"/>
       <c r="K14" s="108"/>
       <c r="L14" s="107"/>
-      <c r="M14" s="139" t="e" vm="11">
+      <c r="M14" s="156" t="e" vm="11">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N14" s="139"/>
-      <c r="O14" s="139"/>
+      <c r="N14" s="156"/>
+      <c r="O14" s="156"/>
       <c r="P14" s="108"/>
       <c r="Q14" s="107"/>
-      <c r="R14" s="139" t="e" vm="12">
+      <c r="R14" s="156" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S14" s="139"/>
-      <c r="T14" s="139"/>
+      <c r="S14" s="156"/>
+      <c r="T14" s="156"/>
       <c r="U14" s="108"/>
     </row>
     <row r="15" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="19"/>
-      <c r="C15" s="145" t="str">
+      <c r="C15" s="153" t="str">
         <f>'Cards Src'!$C10</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D15" s="145"/>
-      <c r="E15" s="145"/>
+      <c r="D15" s="153"/>
+      <c r="E15" s="153"/>
       <c r="F15" s="82"/>
       <c r="G15" s="107"/>
-      <c r="H15" s="140" t="str">
+      <c r="H15" s="154" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="I15" s="140"/>
-      <c r="J15" s="140"/>
+      <c r="I15" s="154"/>
+      <c r="J15" s="154"/>
       <c r="K15" s="110"/>
       <c r="L15" s="107"/>
-      <c r="M15" s="140" t="str">
+      <c r="M15" s="154" t="str">
         <f>'Cards Src'!C12</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="N15" s="140"/>
-      <c r="O15" s="140"/>
+      <c r="N15" s="154"/>
+      <c r="O15" s="154"/>
       <c r="P15" s="110"/>
       <c r="Q15" s="107"/>
-      <c r="R15" s="140" t="str">
+      <c r="R15" s="154" t="str">
         <f>'Cards Src'!C13</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="S15" s="140"/>
-      <c r="T15" s="140"/>
+      <c r="S15" s="154"/>
+      <c r="T15" s="154"/>
       <c r="U15" s="110"/>
     </row>
     <row r="16" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5265,70 +5265,70 @@
     </row>
     <row r="19" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="107"/>
-      <c r="C19" s="139" t="e" vm="13">
+      <c r="C19" s="156" t="e" vm="13">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D19" s="139"/>
-      <c r="E19" s="139"/>
+      <c r="D19" s="156"/>
+      <c r="E19" s="156"/>
       <c r="F19" s="108"/>
       <c r="G19" s="107"/>
-      <c r="H19" s="139" t="e" vm="14">
+      <c r="H19" s="156" t="e" vm="14">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I19" s="139"/>
-      <c r="J19" s="139"/>
+      <c r="I19" s="156"/>
+      <c r="J19" s="156"/>
       <c r="K19" s="108"/>
       <c r="L19" s="107"/>
-      <c r="M19" s="139" t="e" vm="15">
+      <c r="M19" s="156" t="e" vm="15">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N19" s="139"/>
-      <c r="O19" s="139"/>
+      <c r="N19" s="156"/>
+      <c r="O19" s="156"/>
       <c r="P19" s="108"/>
       <c r="Q19" s="107"/>
-      <c r="R19" s="139" t="e" vm="16">
+      <c r="R19" s="156" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S19" s="139"/>
-      <c r="T19" s="139"/>
+      <c r="S19" s="156"/>
+      <c r="T19" s="156"/>
       <c r="U19" s="108"/>
     </row>
     <row r="20" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="107"/>
-      <c r="C20" s="140" t="str">
+      <c r="C20" s="154" t="str">
         <f>'Cards Src'!$C14</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D20" s="140"/>
-      <c r="E20" s="140"/>
+      <c r="D20" s="154"/>
+      <c r="E20" s="154"/>
       <c r="F20" s="110"/>
       <c r="G20" s="107"/>
-      <c r="H20" s="140" t="str">
+      <c r="H20" s="154" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="I20" s="140"/>
-      <c r="J20" s="140"/>
+      <c r="I20" s="154"/>
+      <c r="J20" s="154"/>
       <c r="K20" s="110"/>
       <c r="L20" s="107"/>
-      <c r="M20" s="143" t="str">
+      <c r="M20" s="157" t="str">
         <f>'Cards Src'!C16</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="N20" s="143"/>
-      <c r="O20" s="143"/>
+      <c r="N20" s="157"/>
+      <c r="O20" s="157"/>
       <c r="P20" s="110"/>
       <c r="Q20" s="107"/>
-      <c r="R20" s="140" t="str">
+      <c r="R20" s="154" t="str">
         <f>'Cards Src'!C17</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="S20" s="140"/>
-      <c r="T20" s="140"/>
+      <c r="S20" s="154"/>
+      <c r="T20" s="154"/>
       <c r="U20" s="110"/>
     </row>
     <row r="21" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5413,70 +5413,70 @@
     </row>
     <row r="24" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="107"/>
-      <c r="C24" s="139" t="e" vm="17">
+      <c r="C24" s="156" t="e" vm="17">
         <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D24" s="139"/>
-      <c r="E24" s="139"/>
+      <c r="D24" s="156"/>
+      <c r="E24" s="156"/>
       <c r="F24" s="108"/>
       <c r="G24" s="107"/>
-      <c r="H24" s="139" t="e" vm="18">
+      <c r="H24" s="156" t="e" vm="18">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I24" s="139"/>
-      <c r="J24" s="139"/>
+      <c r="I24" s="156"/>
+      <c r="J24" s="156"/>
       <c r="K24" s="108"/>
       <c r="L24" s="94"/>
-      <c r="M24" s="142">
+      <c r="M24" s="159">
         <f>'Cards Src'!E20</f>
         <v>0</v>
       </c>
-      <c r="N24" s="142"/>
-      <c r="O24" s="142"/>
+      <c r="N24" s="159"/>
+      <c r="O24" s="159"/>
       <c r="P24" s="95"/>
       <c r="Q24" s="94"/>
-      <c r="R24" s="142">
+      <c r="R24" s="159">
         <f xml:space="preserve"> 'Cards Src'!E21</f>
         <v>0</v>
       </c>
-      <c r="S24" s="142"/>
-      <c r="T24" s="142"/>
+      <c r="S24" s="159"/>
+      <c r="T24" s="159"/>
       <c r="U24" s="95"/>
     </row>
     <row r="25" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="107"/>
-      <c r="C25" s="140" t="str">
+      <c r="C25" s="154" t="str">
         <f>'Cards Src'!$C18</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D25" s="140"/>
-      <c r="E25" s="140"/>
+      <c r="D25" s="154"/>
+      <c r="E25" s="154"/>
       <c r="F25" s="110"/>
       <c r="G25" s="107"/>
-      <c r="H25" s="140" t="str">
+      <c r="H25" s="154" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="I25" s="140"/>
-      <c r="J25" s="140"/>
+      <c r="I25" s="154"/>
+      <c r="J25" s="154"/>
       <c r="K25" s="110"/>
       <c r="L25" s="94"/>
-      <c r="M25" s="141">
+      <c r="M25" s="158">
         <f>'Cards Src'!C20</f>
         <v>0</v>
       </c>
-      <c r="N25" s="141"/>
-      <c r="O25" s="141"/>
+      <c r="N25" s="158"/>
+      <c r="O25" s="158"/>
       <c r="P25" s="96"/>
       <c r="Q25" s="94"/>
-      <c r="R25" s="141">
+      <c r="R25" s="158">
         <f>'Cards Src'!C21</f>
         <v>0</v>
       </c>
-      <c r="S25" s="141"/>
-      <c r="T25" s="141"/>
+      <c r="S25" s="158"/>
+      <c r="T25" s="158"/>
       <c r="U25" s="96"/>
     </row>
     <row r="26" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5504,6 +5504,38 @@
     <row r="27" spans="1:22" s="137" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="R25:T25"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="R24:T24"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="R20:T20"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="R15:T15"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="R14:T14"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="R10:T10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="R9:T9"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="H5:J5"/>
@@ -5512,38 +5544,6 @@
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="M4:O4"/>
     <mergeCell ref="R4:T4"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="R10:T10"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="R9:T9"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="R15:T15"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="R14:T14"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="R20:T20"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="R19:T19"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="R25:T25"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="R24:T24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Art - Bramble Snare
Art for Bramble Snare attack card
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91E20631-CBD2-4F03-A256-8CB329EF09FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E695512A-317D-4DE7-B005-3D017996C2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2807,7 +2807,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26115"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26147"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2872,7 +2872,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26116"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26148"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2937,7 +2937,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26117"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26149"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3002,7 +3002,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26118"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26150"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3067,7 +3067,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26119"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26151"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3132,7 +3132,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26120"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26152"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3197,7 +3197,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26121"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26153"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3262,7 +3262,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26122"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26154"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3327,7 +3327,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26123"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26155"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3392,7 +3392,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26124"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26156"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3457,7 +3457,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26125"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26157"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3522,7 +3522,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26126"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26158"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3587,7 +3587,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26127"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26159"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3652,7 +3652,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26128"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26160"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3761,7 +3761,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26129"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26161"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3826,7 +3826,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26130"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26162"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>

</xml_diff>

<commit_message>
Icons - New Art
Added Card Icons for Tidal Wave, Bramble Snare, and Mana Shield
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E695512A-317D-4DE7-B005-3D017996C2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085CAB31-42EF-4942-9366-2BAE543F62FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="15" r:id="rId1"/>
@@ -2807,7 +2807,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26147"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26163"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2872,7 +2872,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26148"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26164"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2937,7 +2937,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26149"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26165"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3002,7 +3002,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26150"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26166"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3067,7 +3067,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26151"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26167"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3132,7 +3132,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26152"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26168"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3197,7 +3197,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26153"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26169"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3262,7 +3262,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26154"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26170"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3327,7 +3327,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26155"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26171"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3392,7 +3392,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26156"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26172"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3457,7 +3457,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26157"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26173"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3522,7 +3522,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26158"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26174"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3587,7 +3587,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26159"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26175"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3652,7 +3652,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26160"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26176"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3761,7 +3761,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26161"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26177"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3826,7 +3826,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26162"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26178"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>

</xml_diff>

<commit_message>
Art - Black Hole
Art for Black Hole attack card
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085CAB31-42EF-4942-9366-2BAE543F62FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109F8892-5680-4920-AA05-AEDE15AB2098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="15" r:id="rId1"/>
@@ -1585,6 +1585,45 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1607,45 +1646,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2807,7 +2807,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26163"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26233"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2872,7 +2872,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26164"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26234"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2937,7 +2937,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26165"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26235"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3002,7 +3002,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26166"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26236"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3067,7 +3067,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26167"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26237"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3132,7 +3132,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26168"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26238"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3197,7 +3197,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26169"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26239"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3262,7 +3262,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26170"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26240"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3327,7 +3327,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26171"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26241"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3392,7 +3392,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26172"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26242"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3457,7 +3457,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26173"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26243"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3522,7 +3522,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26174"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26244"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3587,7 +3587,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26175"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26245"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3652,7 +3652,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26176"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26246"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3761,7 +3761,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26177"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26247"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3826,7 +3826,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26178"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26248"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -4821,70 +4821,70 @@
     </row>
     <row r="4" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
-      <c r="C4" s="139" t="e" vm="1">
+      <c r="C4" s="152" t="e" vm="1">
         <f>'Cards Src'!E2</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="139"/>
-      <c r="E4" s="139"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
       <c r="F4" s="42"/>
       <c r="G4" s="53"/>
-      <c r="H4" s="144" t="e" vm="2">
+      <c r="H4" s="157" t="e" vm="2">
         <f>'Cards Src'!E3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I4" s="144"/>
-      <c r="J4" s="144"/>
+      <c r="I4" s="157"/>
+      <c r="J4" s="157"/>
       <c r="K4" s="54"/>
       <c r="L4" s="116"/>
-      <c r="M4" s="145" t="e" vm="3">
+      <c r="M4" s="158" t="e" vm="3">
         <f>'Cards Src'!E4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N4" s="145"/>
-      <c r="O4" s="145"/>
+      <c r="N4" s="158"/>
+      <c r="O4" s="158"/>
       <c r="P4" s="64"/>
       <c r="Q4" s="7"/>
-      <c r="R4" s="146" t="e" vm="4">
+      <c r="R4" s="159" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S4" s="146"/>
-      <c r="T4" s="146"/>
+      <c r="S4" s="159"/>
+      <c r="T4" s="159"/>
       <c r="U4" s="29"/>
     </row>
     <row r="5" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
-      <c r="C5" s="140" t="str">
+      <c r="C5" s="153" t="str">
         <f>'Cards Src'!$C2</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="140"/>
-      <c r="E5" s="140"/>
+      <c r="D5" s="153"/>
+      <c r="E5" s="153"/>
       <c r="F5" s="43"/>
       <c r="G5" s="53"/>
-      <c r="H5" s="141" t="str">
+      <c r="H5" s="154" t="str">
         <f>'Cards Src'!$C3</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="I5" s="141"/>
-      <c r="J5" s="141"/>
+      <c r="I5" s="154"/>
+      <c r="J5" s="154"/>
       <c r="K5" s="55"/>
       <c r="L5" s="3"/>
-      <c r="M5" s="142" t="str">
+      <c r="M5" s="155" t="str">
         <f>'Cards Src'!C4</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="N5" s="142"/>
-      <c r="O5" s="142"/>
+      <c r="N5" s="155"/>
+      <c r="O5" s="155"/>
       <c r="P5" s="65"/>
       <c r="Q5" s="7"/>
-      <c r="R5" s="143" t="str">
+      <c r="R5" s="156" t="str">
         <f>'Cards Src'!C5</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="S5" s="143"/>
-      <c r="T5" s="143"/>
+      <c r="S5" s="156"/>
+      <c r="T5" s="156"/>
       <c r="U5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4985,12 +4985,12 @@
       <c r="J9" s="151"/>
       <c r="K9" s="72"/>
       <c r="L9" s="19"/>
-      <c r="M9" s="152" t="e" vm="7">
+      <c r="M9" s="144" t="e" vm="7">
         <f>'Cards Src'!E8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N9" s="152"/>
-      <c r="O9" s="152"/>
+      <c r="N9" s="144"/>
+      <c r="O9" s="144"/>
       <c r="P9" s="81"/>
       <c r="Q9" s="11"/>
       <c r="R9" s="147" t="e" vm="8">
@@ -5117,70 +5117,70 @@
     </row>
     <row r="14" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="19"/>
-      <c r="C14" s="152" t="e" vm="9">
+      <c r="C14" s="144" t="e" vm="9">
         <f>'Cards Src'!E10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D14" s="152"/>
-      <c r="E14" s="152"/>
+      <c r="D14" s="144"/>
+      <c r="E14" s="144"/>
       <c r="F14" s="81"/>
       <c r="G14" s="107"/>
-      <c r="H14" s="155" t="e" vm="10">
+      <c r="H14" s="146" t="e" vm="10">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I14" s="155"/>
-      <c r="J14" s="155"/>
+      <c r="I14" s="146"/>
+      <c r="J14" s="146"/>
       <c r="K14" s="108"/>
       <c r="L14" s="107"/>
-      <c r="M14" s="156" t="e" vm="11">
+      <c r="M14" s="139" t="e" vm="11">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N14" s="156"/>
-      <c r="O14" s="156"/>
+      <c r="N14" s="139"/>
+      <c r="O14" s="139"/>
       <c r="P14" s="108"/>
       <c r="Q14" s="107"/>
-      <c r="R14" s="156" t="e" vm="12">
+      <c r="R14" s="139" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S14" s="156"/>
-      <c r="T14" s="156"/>
+      <c r="S14" s="139"/>
+      <c r="T14" s="139"/>
       <c r="U14" s="108"/>
     </row>
     <row r="15" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="19"/>
-      <c r="C15" s="153" t="str">
+      <c r="C15" s="145" t="str">
         <f>'Cards Src'!$C10</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D15" s="153"/>
-      <c r="E15" s="153"/>
+      <c r="D15" s="145"/>
+      <c r="E15" s="145"/>
       <c r="F15" s="82"/>
       <c r="G15" s="107"/>
-      <c r="H15" s="154" t="str">
+      <c r="H15" s="140" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="I15" s="154"/>
-      <c r="J15" s="154"/>
+      <c r="I15" s="140"/>
+      <c r="J15" s="140"/>
       <c r="K15" s="110"/>
       <c r="L15" s="107"/>
-      <c r="M15" s="154" t="str">
+      <c r="M15" s="140" t="str">
         <f>'Cards Src'!C12</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="N15" s="154"/>
-      <c r="O15" s="154"/>
+      <c r="N15" s="140"/>
+      <c r="O15" s="140"/>
       <c r="P15" s="110"/>
       <c r="Q15" s="107"/>
-      <c r="R15" s="154" t="str">
+      <c r="R15" s="140" t="str">
         <f>'Cards Src'!C13</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="S15" s="154"/>
-      <c r="T15" s="154"/>
+      <c r="S15" s="140"/>
+      <c r="T15" s="140"/>
       <c r="U15" s="110"/>
     </row>
     <row r="16" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5265,70 +5265,70 @@
     </row>
     <row r="19" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="107"/>
-      <c r="C19" s="156" t="e" vm="13">
+      <c r="C19" s="139" t="e" vm="13">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D19" s="156"/>
-      <c r="E19" s="156"/>
+      <c r="D19" s="139"/>
+      <c r="E19" s="139"/>
       <c r="F19" s="108"/>
       <c r="G19" s="107"/>
-      <c r="H19" s="156" t="e" vm="14">
+      <c r="H19" s="139" t="e" vm="14">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I19" s="156"/>
-      <c r="J19" s="156"/>
+      <c r="I19" s="139"/>
+      <c r="J19" s="139"/>
       <c r="K19" s="108"/>
       <c r="L19" s="107"/>
-      <c r="M19" s="156" t="e" vm="15">
+      <c r="M19" s="139" t="e" vm="15">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N19" s="156"/>
-      <c r="O19" s="156"/>
+      <c r="N19" s="139"/>
+      <c r="O19" s="139"/>
       <c r="P19" s="108"/>
       <c r="Q19" s="107"/>
-      <c r="R19" s="156" t="e" vm="16">
+      <c r="R19" s="139" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S19" s="156"/>
-      <c r="T19" s="156"/>
+      <c r="S19" s="139"/>
+      <c r="T19" s="139"/>
       <c r="U19" s="108"/>
     </row>
     <row r="20" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="107"/>
-      <c r="C20" s="154" t="str">
+      <c r="C20" s="140" t="str">
         <f>'Cards Src'!$C14</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D20" s="154"/>
-      <c r="E20" s="154"/>
+      <c r="D20" s="140"/>
+      <c r="E20" s="140"/>
       <c r="F20" s="110"/>
       <c r="G20" s="107"/>
-      <c r="H20" s="154" t="str">
+      <c r="H20" s="140" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="I20" s="154"/>
-      <c r="J20" s="154"/>
+      <c r="I20" s="140"/>
+      <c r="J20" s="140"/>
       <c r="K20" s="110"/>
       <c r="L20" s="107"/>
-      <c r="M20" s="157" t="str">
+      <c r="M20" s="143" t="str">
         <f>'Cards Src'!C16</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="N20" s="157"/>
-      <c r="O20" s="157"/>
+      <c r="N20" s="143"/>
+      <c r="O20" s="143"/>
       <c r="P20" s="110"/>
       <c r="Q20" s="107"/>
-      <c r="R20" s="154" t="str">
+      <c r="R20" s="140" t="str">
         <f>'Cards Src'!C17</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="S20" s="154"/>
-      <c r="T20" s="154"/>
+      <c r="S20" s="140"/>
+      <c r="T20" s="140"/>
       <c r="U20" s="110"/>
     </row>
     <row r="21" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5413,70 +5413,70 @@
     </row>
     <row r="24" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="107"/>
-      <c r="C24" s="156" t="e" vm="17">
+      <c r="C24" s="139" t="e" vm="17">
         <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D24" s="156"/>
-      <c r="E24" s="156"/>
+      <c r="D24" s="139"/>
+      <c r="E24" s="139"/>
       <c r="F24" s="108"/>
       <c r="G24" s="107"/>
-      <c r="H24" s="156" t="e" vm="18">
+      <c r="H24" s="139" t="e" vm="18">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I24" s="156"/>
-      <c r="J24" s="156"/>
+      <c r="I24" s="139"/>
+      <c r="J24" s="139"/>
       <c r="K24" s="108"/>
       <c r="L24" s="94"/>
-      <c r="M24" s="159">
+      <c r="M24" s="142">
         <f>'Cards Src'!E20</f>
         <v>0</v>
       </c>
-      <c r="N24" s="159"/>
-      <c r="O24" s="159"/>
+      <c r="N24" s="142"/>
+      <c r="O24" s="142"/>
       <c r="P24" s="95"/>
       <c r="Q24" s="94"/>
-      <c r="R24" s="159">
+      <c r="R24" s="142">
         <f xml:space="preserve"> 'Cards Src'!E21</f>
         <v>0</v>
       </c>
-      <c r="S24" s="159"/>
-      <c r="T24" s="159"/>
+      <c r="S24" s="142"/>
+      <c r="T24" s="142"/>
       <c r="U24" s="95"/>
     </row>
     <row r="25" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="107"/>
-      <c r="C25" s="154" t="str">
+      <c r="C25" s="140" t="str">
         <f>'Cards Src'!$C18</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D25" s="154"/>
-      <c r="E25" s="154"/>
+      <c r="D25" s="140"/>
+      <c r="E25" s="140"/>
       <c r="F25" s="110"/>
       <c r="G25" s="107"/>
-      <c r="H25" s="154" t="str">
+      <c r="H25" s="140" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="I25" s="154"/>
-      <c r="J25" s="154"/>
+      <c r="I25" s="140"/>
+      <c r="J25" s="140"/>
       <c r="K25" s="110"/>
       <c r="L25" s="94"/>
-      <c r="M25" s="158">
+      <c r="M25" s="141">
         <f>'Cards Src'!C20</f>
         <v>0</v>
       </c>
-      <c r="N25" s="158"/>
-      <c r="O25" s="158"/>
+      <c r="N25" s="141"/>
+      <c r="O25" s="141"/>
       <c r="P25" s="96"/>
       <c r="Q25" s="94"/>
-      <c r="R25" s="158">
+      <c r="R25" s="141">
         <f>'Cards Src'!C21</f>
         <v>0</v>
       </c>
-      <c r="S25" s="158"/>
-      <c r="T25" s="158"/>
+      <c r="S25" s="141"/>
+      <c r="T25" s="141"/>
       <c r="U25" s="96"/>
     </row>
     <row r="26" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5504,6 +5504,38 @@
     <row r="27" spans="1:22" s="137" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="R5:T5"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="M4:O4"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="R10:T10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="R9:T9"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="R15:T15"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="R14:T14"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="R20:T20"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="R19:T19"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="C25:E25"/>
     <mergeCell ref="H25:J25"/>
@@ -5512,38 +5544,6 @@
     <mergeCell ref="H24:J24"/>
     <mergeCell ref="M24:O24"/>
     <mergeCell ref="R24:T24"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="R20:T20"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="R19:T19"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="R15:T15"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="R14:T14"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="R10:T10"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="R9:T9"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="M5:O5"/>
-    <mergeCell ref="R5:T5"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="M4:O4"/>
-    <mergeCell ref="R4:T4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Art - Runaway Bull
Art for the Runaway Bull modifier card
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\Card Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109F8892-5680-4920-AA05-AEDE15AB2098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6365232F-CA78-478A-9FAF-C88479B96E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1585,67 +1585,67 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2807,7 +2807,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26233"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26249"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2872,7 +2872,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26234"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26250"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2937,7 +2937,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26235"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26251"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3002,7 +3002,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26236"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26252"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3067,7 +3067,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26237"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26253"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3132,7 +3132,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26238"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26254"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3197,7 +3197,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26239"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26255"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3262,7 +3262,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26240"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26256"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3327,7 +3327,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26241"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26257"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3392,7 +3392,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26242"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26258"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3457,7 +3457,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26243"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26259"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3522,7 +3522,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26244"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26260"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3587,7 +3587,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26245"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26261"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3652,7 +3652,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26246"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26262"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3761,7 +3761,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26247"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26263"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3826,7 +3826,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26248"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26264"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -4821,70 +4821,70 @@
     </row>
     <row r="4" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
-      <c r="C4" s="152" t="e" vm="1">
+      <c r="C4" s="139" t="e" vm="1">
         <f>'Cards Src'!E2</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D4" s="152"/>
-      <c r="E4" s="152"/>
+      <c r="D4" s="139"/>
+      <c r="E4" s="139"/>
       <c r="F4" s="42"/>
       <c r="G4" s="53"/>
-      <c r="H4" s="157" t="e" vm="2">
+      <c r="H4" s="144" t="e" vm="2">
         <f>'Cards Src'!E3</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I4" s="157"/>
-      <c r="J4" s="157"/>
+      <c r="I4" s="144"/>
+      <c r="J4" s="144"/>
       <c r="K4" s="54"/>
       <c r="L4" s="116"/>
-      <c r="M4" s="158" t="e" vm="3">
+      <c r="M4" s="145" t="e" vm="3">
         <f>'Cards Src'!E4</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N4" s="158"/>
-      <c r="O4" s="158"/>
+      <c r="N4" s="145"/>
+      <c r="O4" s="145"/>
       <c r="P4" s="64"/>
       <c r="Q4" s="7"/>
-      <c r="R4" s="159" t="e" vm="4">
+      <c r="R4" s="146" t="e" vm="4">
         <f xml:space="preserve"> 'Cards Src'!E5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S4" s="159"/>
-      <c r="T4" s="159"/>
+      <c r="S4" s="146"/>
+      <c r="T4" s="146"/>
       <c r="U4" s="29"/>
     </row>
     <row r="5" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
-      <c r="C5" s="153" t="str">
+      <c r="C5" s="140" t="str">
         <f>'Cards Src'!$C2</f>
         <v>Deals damage on contact. Explodes against surfaces</v>
       </c>
-      <c r="D5" s="153"/>
-      <c r="E5" s="153"/>
+      <c r="D5" s="140"/>
+      <c r="E5" s="140"/>
       <c r="F5" s="43"/>
       <c r="G5" s="53"/>
-      <c r="H5" s="154" t="str">
+      <c r="H5" s="141" t="str">
         <f>'Cards Src'!$C3</f>
         <v>Explodes on contact and freezes enemies. Frozen enemies take 1.5x damage</v>
       </c>
-      <c r="I5" s="154"/>
-      <c r="J5" s="154"/>
+      <c r="I5" s="141"/>
+      <c r="J5" s="141"/>
       <c r="K5" s="55"/>
       <c r="L5" s="3"/>
-      <c r="M5" s="155" t="str">
+      <c r="M5" s="142" t="str">
         <f>'Cards Src'!C4</f>
         <v>Summons a wave that pushes back all enemies it hits, accumulating damage</v>
       </c>
-      <c r="N5" s="155"/>
-      <c r="O5" s="155"/>
+      <c r="N5" s="142"/>
+      <c r="O5" s="142"/>
       <c r="P5" s="65"/>
       <c r="Q5" s="7"/>
-      <c r="R5" s="156" t="str">
+      <c r="R5" s="143" t="str">
         <f>'Cards Src'!C5</f>
         <v>Creates a trap area that slows + damages enemies as they move through it</v>
       </c>
-      <c r="S5" s="156"/>
-      <c r="T5" s="156"/>
+      <c r="S5" s="143"/>
+      <c r="T5" s="143"/>
       <c r="U5" s="30"/>
     </row>
     <row r="6" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4985,12 +4985,12 @@
       <c r="J9" s="151"/>
       <c r="K9" s="72"/>
       <c r="L9" s="19"/>
-      <c r="M9" s="144" t="e" vm="7">
+      <c r="M9" s="152" t="e" vm="7">
         <f>'Cards Src'!E8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N9" s="144"/>
-      <c r="O9" s="144"/>
+      <c r="N9" s="152"/>
+      <c r="O9" s="152"/>
       <c r="P9" s="81"/>
       <c r="Q9" s="11"/>
       <c r="R9" s="147" t="e" vm="8">
@@ -5117,70 +5117,70 @@
     </row>
     <row r="14" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="19"/>
-      <c r="C14" s="144" t="e" vm="9">
+      <c r="C14" s="152" t="e" vm="9">
         <f>'Cards Src'!E10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D14" s="144"/>
-      <c r="E14" s="144"/>
+      <c r="D14" s="152"/>
+      <c r="E14" s="152"/>
       <c r="F14" s="81"/>
       <c r="G14" s="107"/>
-      <c r="H14" s="146" t="e" vm="10">
+      <c r="H14" s="155" t="e" vm="10">
         <f>'Cards Src'!E11</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I14" s="146"/>
-      <c r="J14" s="146"/>
+      <c r="I14" s="155"/>
+      <c r="J14" s="155"/>
       <c r="K14" s="108"/>
       <c r="L14" s="107"/>
-      <c r="M14" s="139" t="e" vm="11">
+      <c r="M14" s="156" t="e" vm="11">
         <f>'Cards Src'!E12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N14" s="139"/>
-      <c r="O14" s="139"/>
+      <c r="N14" s="156"/>
+      <c r="O14" s="156"/>
       <c r="P14" s="108"/>
       <c r="Q14" s="107"/>
-      <c r="R14" s="139" t="e" vm="12">
+      <c r="R14" s="156" t="e" vm="12">
         <f xml:space="preserve"> 'Cards Src'!E13</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S14" s="139"/>
-      <c r="T14" s="139"/>
+      <c r="S14" s="156"/>
+      <c r="T14" s="156"/>
       <c r="U14" s="108"/>
     </row>
     <row r="15" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="19"/>
-      <c r="C15" s="145" t="str">
+      <c r="C15" s="153" t="str">
         <f>'Cards Src'!$C10</f>
         <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
       </c>
-      <c r="D15" s="145"/>
-      <c r="E15" s="145"/>
+      <c r="D15" s="153"/>
+      <c r="E15" s="153"/>
       <c r="F15" s="82"/>
       <c r="G15" s="107"/>
-      <c r="H15" s="140" t="str">
+      <c r="H15" s="154" t="str">
         <f>'Cards Src'!$C11</f>
         <v>Increases player movement speed for a set duration</v>
       </c>
-      <c r="I15" s="140"/>
-      <c r="J15" s="140"/>
+      <c r="I15" s="154"/>
+      <c r="J15" s="154"/>
       <c r="K15" s="110"/>
       <c r="L15" s="107"/>
-      <c r="M15" s="140" t="str">
+      <c r="M15" s="154" t="str">
         <f>'Cards Src'!C12</f>
         <v>Enemies are temporarily slowed on hit for a set duration.</v>
       </c>
-      <c r="N15" s="140"/>
-      <c r="O15" s="140"/>
+      <c r="N15" s="154"/>
+      <c r="O15" s="154"/>
       <c r="P15" s="110"/>
       <c r="Q15" s="107"/>
-      <c r="R15" s="140" t="str">
+      <c r="R15" s="154" t="str">
         <f>'Cards Src'!C13</f>
         <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
-      <c r="S15" s="140"/>
-      <c r="T15" s="140"/>
+      <c r="S15" s="154"/>
+      <c r="T15" s="154"/>
       <c r="U15" s="110"/>
     </row>
     <row r="16" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5265,70 +5265,70 @@
     </row>
     <row r="19" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="107"/>
-      <c r="C19" s="139" t="e" vm="13">
+      <c r="C19" s="156" t="e" vm="13">
         <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D19" s="139"/>
-      <c r="E19" s="139"/>
+      <c r="D19" s="156"/>
+      <c r="E19" s="156"/>
       <c r="F19" s="108"/>
       <c r="G19" s="107"/>
-      <c r="H19" s="139" t="e" vm="14">
+      <c r="H19" s="156" t="e" vm="14">
         <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I19" s="139"/>
-      <c r="J19" s="139"/>
+      <c r="I19" s="156"/>
+      <c r="J19" s="156"/>
       <c r="K19" s="108"/>
       <c r="L19" s="107"/>
-      <c r="M19" s="139" t="e" vm="15">
+      <c r="M19" s="156" t="e" vm="15">
         <f>'Cards Src'!E16</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N19" s="139"/>
-      <c r="O19" s="139"/>
+      <c r="N19" s="156"/>
+      <c r="O19" s="156"/>
       <c r="P19" s="108"/>
       <c r="Q19" s="107"/>
-      <c r="R19" s="139" t="e" vm="16">
+      <c r="R19" s="156" t="e" vm="16">
         <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S19" s="139"/>
-      <c r="T19" s="139"/>
+      <c r="S19" s="156"/>
+      <c r="T19" s="156"/>
       <c r="U19" s="108"/>
     </row>
     <row r="20" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="107"/>
-      <c r="C20" s="140" t="str">
+      <c r="C20" s="154" t="str">
         <f>'Cards Src'!$C14</f>
         <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
-      <c r="D20" s="140"/>
-      <c r="E20" s="140"/>
+      <c r="D20" s="154"/>
+      <c r="E20" s="154"/>
       <c r="F20" s="110"/>
       <c r="G20" s="107"/>
-      <c r="H20" s="140" t="str">
+      <c r="H20" s="154" t="str">
         <f>'Cards Src'!$C15</f>
         <v>Negate x number of hits</v>
       </c>
-      <c r="I20" s="140"/>
-      <c r="J20" s="140"/>
+      <c r="I20" s="154"/>
+      <c r="J20" s="154"/>
       <c r="K20" s="110"/>
       <c r="L20" s="107"/>
-      <c r="M20" s="143" t="str">
+      <c r="M20" s="157" t="str">
         <f>'Cards Src'!C16</f>
         <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
       </c>
-      <c r="N20" s="143"/>
-      <c r="O20" s="143"/>
+      <c r="N20" s="157"/>
+      <c r="O20" s="157"/>
       <c r="P20" s="110"/>
       <c r="Q20" s="107"/>
-      <c r="R20" s="140" t="str">
+      <c r="R20" s="154" t="str">
         <f>'Cards Src'!C17</f>
         <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
-      <c r="S20" s="140"/>
-      <c r="T20" s="140"/>
+      <c r="S20" s="154"/>
+      <c r="T20" s="154"/>
       <c r="U20" s="110"/>
     </row>
     <row r="21" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5413,70 +5413,70 @@
     </row>
     <row r="24" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="107"/>
-      <c r="C24" s="139" t="e" vm="17">
+      <c r="C24" s="156" t="e" vm="17">
         <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D24" s="139"/>
-      <c r="E24" s="139"/>
+      <c r="D24" s="156"/>
+      <c r="E24" s="156"/>
       <c r="F24" s="108"/>
       <c r="G24" s="107"/>
-      <c r="H24" s="139" t="e" vm="18">
+      <c r="H24" s="156" t="e" vm="18">
         <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I24" s="139"/>
-      <c r="J24" s="139"/>
+      <c r="I24" s="156"/>
+      <c r="J24" s="156"/>
       <c r="K24" s="108"/>
       <c r="L24" s="94"/>
-      <c r="M24" s="142">
+      <c r="M24" s="159">
         <f>'Cards Src'!E20</f>
         <v>0</v>
       </c>
-      <c r="N24" s="142"/>
-      <c r="O24" s="142"/>
+      <c r="N24" s="159"/>
+      <c r="O24" s="159"/>
       <c r="P24" s="95"/>
       <c r="Q24" s="94"/>
-      <c r="R24" s="142">
+      <c r="R24" s="159">
         <f xml:space="preserve"> 'Cards Src'!E21</f>
         <v>0</v>
       </c>
-      <c r="S24" s="142"/>
-      <c r="T24" s="142"/>
+      <c r="S24" s="159"/>
+      <c r="T24" s="159"/>
       <c r="U24" s="95"/>
     </row>
     <row r="25" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="107"/>
-      <c r="C25" s="140" t="str">
+      <c r="C25" s="154" t="str">
         <f>'Cards Src'!$C18</f>
         <v>Recall last used card into deck</v>
       </c>
-      <c r="D25" s="140"/>
-      <c r="E25" s="140"/>
+      <c r="D25" s="154"/>
+      <c r="E25" s="154"/>
       <c r="F25" s="110"/>
       <c r="G25" s="107"/>
-      <c r="H25" s="140" t="str">
+      <c r="H25" s="154" t="str">
         <f>'Cards Src'!$C19</f>
         <v>Draw 2 cards</v>
       </c>
-      <c r="I25" s="140"/>
-      <c r="J25" s="140"/>
+      <c r="I25" s="154"/>
+      <c r="J25" s="154"/>
       <c r="K25" s="110"/>
       <c r="L25" s="94"/>
-      <c r="M25" s="141">
+      <c r="M25" s="158">
         <f>'Cards Src'!C20</f>
         <v>0</v>
       </c>
-      <c r="N25" s="141"/>
-      <c r="O25" s="141"/>
+      <c r="N25" s="158"/>
+      <c r="O25" s="158"/>
       <c r="P25" s="96"/>
       <c r="Q25" s="94"/>
-      <c r="R25" s="141">
+      <c r="R25" s="158">
         <f>'Cards Src'!C21</f>
         <v>0</v>
       </c>
-      <c r="S25" s="141"/>
-      <c r="T25" s="141"/>
+      <c r="S25" s="158"/>
+      <c r="T25" s="158"/>
       <c r="U25" s="96"/>
     </row>
     <row r="26" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5504,6 +5504,38 @@
     <row r="27" spans="1:22" s="137" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="M25:O25"/>
+    <mergeCell ref="R25:T25"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="M24:O24"/>
+    <mergeCell ref="R24:T24"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="M20:O20"/>
+    <mergeCell ref="R20:T20"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="R15:T15"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="R14:T14"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="M10:O10"/>
+    <mergeCell ref="R10:T10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="M9:O9"/>
+    <mergeCell ref="R9:T9"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="H5:J5"/>
@@ -5512,38 +5544,6 @@
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="M4:O4"/>
     <mergeCell ref="R4:T4"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="M10:O10"/>
-    <mergeCell ref="R10:T10"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="M9:O9"/>
-    <mergeCell ref="R9:T9"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="M15:O15"/>
-    <mergeCell ref="R15:T15"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="M14:O14"/>
-    <mergeCell ref="R14:T14"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="M20:O20"/>
-    <mergeCell ref="R20:T20"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="R19:T19"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="R25:T25"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="R24:T24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Art - Divine Judgement
Added the last card art, Divine Judgement
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\Card Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6365232F-CA78-478A-9FAF-C88479B96E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1B3B34-0E18-41D8-BAFB-3E970CB0A55A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1683,860 +1683,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="56" name="Picture 55">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6643A80E-1E86-43F0-A209-C1D50216F722}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="609600" y="16287750"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="57" name="Picture 56">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6E4D18E-8A8E-450E-9786-783FDD5E9176}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4914900" y="16287750"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="58" name="Picture 57">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37A6EFF8-4851-4285-81EF-A040AC6311C1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9220200" y="16287750"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="59" name="Picture 58">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1184FE64-8B56-433D-BBF5-2BB9046EEC7B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13525500" y="16287750"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="60" name="Picture 59">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1E8C2D1-BE90-4701-A257-39737621BDF1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="609600" y="21650325"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="61" name="Picture 60">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94E4EFA5-2E34-4FC3-8A05-36E8EAB45292}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4914900" y="21650325"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="54" name="Picture 53">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA45D086-D230-4AA1-9245-BE67E5F173D0}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13525500" y="10925175"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="53" name="Picture 52">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3EF0721-4DDE-4F40-987C-1C816DC4241E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9220200" y="10925175"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="52" name="Picture 51">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F7DAF7DC-C28D-B648-A1F5-9051912EDC0A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4914900" y="10925175"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="47" name="Picture 46">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49043CFD-EA61-4065-882F-869A50F62868}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="609600" y="10925175"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="46" name="Picture 45">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0BCCACA-3FFB-42EA-85C5-1F7808814533}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="13525500" y="5562600"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="45" name="Picture 44">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5541008-5B1A-4E98-9BF9-323D3A316D73}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="9220200" y="5562600"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="44" name="Picture 43">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3CA5460E-7BB0-46BB-A7D2-173FA277090E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="4914900" y="5562600"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="43" name="Picture 42">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E43082E8-05A2-42EC-96D7-B4898EC02DC5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="609600" y="5562600"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
@@ -2562,7 +1708,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2623,7 +1769,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2684,7 +1830,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2745,7 +1891,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2783,136 +1929,6 @@
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>6</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>3</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="2" name="Picture 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C521C7F4-671D-0A45-9735-836567FFA2B9}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26249"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="5562600"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>16</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>6</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>18</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="10" name="Picture 9">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A36F1FB-D023-B2AA-5081-52E889897827}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26250"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="13525500" y="5562600"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
           <xdr:col>6</xdr:col>
           <xdr:colOff>0</xdr:colOff>
           <xdr:row>1</xdr:row>
@@ -2937,13 +1953,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26251"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26430"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3002,13 +2018,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26252"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26431"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -3017,656 +2033,6 @@
           <xdr:spPr bwMode="auto">
             <a:xfrm>
               <a:off x="13525500" y="200025"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>6</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>6</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="14" name="Picture 13">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B576719D-8BA6-9858-BC7D-10FA133C864D}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26253"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="5562600"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>11</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>6</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="15" name="Picture 14">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C669489D-FE2E-74CB-12BA-FCF3F27D6F5A}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26254"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="5562600"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>11</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>3</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>12</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="25" name="Picture 24">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{543F4BF1-000E-35C7-3B25-6A370D72B0A5}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26255"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="10925175"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>6</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>11</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>12</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="26" name="Picture 25">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6DF1518-9F16-3EEB-4E52-B419760BD6D3}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26256"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="10925175"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>11</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>11</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>12</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="28" name="Picture 27">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3072FAA5-7CA2-2185-B433-53847D82E0AD}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26257"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="10925175"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>11</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>16</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>13</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>17</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="33" name="Picture 32">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1502DDBA-04CF-508A-A772-199391C15073}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26258"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="9220200" y="16287750"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>6</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>16</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>17</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="34" name="Picture 33">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C71F4324-8F91-5E8B-B2FB-CA0D2990ECD4}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26259"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="16287750"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>16</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>16</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>18</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>17</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="35" name="Picture 34">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBF4878E-BFFD-9114-3CC9-B741BD0495CD}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26260"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="13525500" y="16287750"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>16</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>11</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>18</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>12</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="38" name="Picture 37">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA47B8F5-192C-52AC-48C5-1ADA10A2B02D}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26261"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="13525500" y="10925175"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>16</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>3</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>17</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="39" name="Picture 38">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43F4E71F-5074-6D90-70F8-B48999ECF183}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26262"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="16287750"/>
               <a:ext cx="1038225" cy="1038225"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -3716,7 +2082,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3733,136 +2099,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>21</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>3</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>22</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="29" name="Picture 28">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{292D765A-E3FA-4B39-AADB-BE88A55C8C15}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26263"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="609600" y="21650325"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>6</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>21</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>8</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
-          <xdr:row>22</xdr:row>
-          <xdr:rowOff>876300</xdr:rowOff>
-        </xdr:to>
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="30" name="Picture 29">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{432560D0-7668-43F9-B2B0-01C69C0E123B}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr>
-              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-              <a:extLst>
-                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26264"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPicPr>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
-            <a:srcRect/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="4914900" y="21650325"/>
-              <a:ext cx="1038225" cy="1038225"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:pic>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
@@ -3890,7 +2126,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -3926,23 +2162,1708 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>26</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="20" name="Picture 19">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D012A3C-9297-C268-573B-B28B633BBB5A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A71C0859-748B-40A1-AF8F-048E3D6C1207}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="14963775" y="200025"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>21</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>1</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>23</xdr:col>
+          <xdr:colOff>47625</xdr:colOff>
+          <xdr:row>2</xdr:row>
+          <xdr:rowOff>876300</xdr:rowOff>
+        </xdr:to>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="21" name="Picture 20">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D05AA74C-1375-4635-9EF3-8A6ECE87ED45}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26432"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="14963775" y="200025"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Picture 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75DA29EE-1622-45F4-B677-F343527E6558}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3876675" y="5181600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="23" name="Picture 22">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DEF6EF0A-558E-4682-A701-D1975B62C892}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26433"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="3876675" y="5181600"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Picture 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6D32FFB-0C04-4B8E-BCEE-014ED603EAFE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="7572375" y="5181600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="27" name="Picture 26">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6ECFA43-E163-4C9F-8CA6-E1EB1D0FB09C}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26434"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="7572375" y="5181600"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Picture 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0870AB32-E262-4097-80F4-10D376F2FBBE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11268075" y="5181600"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>11</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="36" name="Picture 35">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A3B0DFA-D994-4FF4-B417-D94D9918455A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26435"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="11268075" y="5181600"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Picture 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D947106A-7FAA-4306-A7EE-C77EB39A401B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="180975" y="10163175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>16</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="49" name="Picture 48">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{152A3A5B-1FA2-4664-994E-BFE6E37663E5}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26436"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="180975" y="10163175"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="50" name="Picture 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B549E9C-CA58-41FC-899F-319E6EC60568}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3876675" y="10163175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>21</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>6</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="51" name="Picture 50">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E6C0BF71-4CB4-415F-81CB-9BDD1CF38B0D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26437"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="3876675" y="10163175"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="55" name="Picture 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{097E0E90-07B4-4036-AC53-9D85F561112D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="7572375" y="10163175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>11</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="62" name="Picture 61">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F32765B2-F198-4C62-BE05-1B0D51274376}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26438"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="7572375" y="10163175"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="63" name="Picture 62">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B68CD4FA-5825-4E13-B80B-C903AF6E150D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11268075" y="10163175"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>11</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="64" name="Picture 63">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E403313-31DC-4060-AAD4-9440B68842FC}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26439"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="11268075" y="10163175"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="65" name="Picture 64">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EF552AC-1CEA-4D5A-BE3E-776A6F739A4D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="180975" y="15144750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>11</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>11</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="66" name="Picture 65">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7152206-5B93-42D7-A66E-7C5A2F24AAD3}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26440"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="180975" y="15144750"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="67" name="Picture 66">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5BE251F9-8DD4-4039-9F40-35A92DAFB568}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3876675" y="15144750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>16</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>11</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="68" name="Picture 67">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1472319F-59BC-4B85-AC0D-5F25C5121797}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26441"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="3876675" y="15144750"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="69" name="Picture 68">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9DF6A63-9FC3-441E-8515-56F3B7809565}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="7572375" y="15144750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>21</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>11</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="70" name="Picture 69">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7F692EA-6D4C-4E81-A63C-E54B99B4E724}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26442"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="7572375" y="15144750"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="71" name="Picture 70">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE40E61F-1F53-4596-A8EE-093D81C723DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11268075" y="15144750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>1</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>16</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="73" name="Picture 72">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9021CDE6-10E9-4FBD-BDC9-06E44288A02D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26443"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="11268075" y="15144750"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="76" name="Picture 75">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4527763F-236F-4702-8875-6362D3BF554E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="180975" y="20126325"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>16</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="77" name="Picture 76">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57A23A8C-976D-4522-920E-423F25E9D048}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26444"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="180975" y="20126325"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="78" name="Picture 77">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4AE1C048-89D5-4BCC-BC21-67E44A82D6B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3876675" y="20126325"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>11</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>16</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1038225" cy="1038225"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="79" name="Picture 78">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F21664C-F923-4DFB-9962-F970960F2974}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26445"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="3876675" y="20126325"/>
+              <a:ext cx="1038225" cy="1038225"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="80" name="Picture 79">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95EC237F-51FD-4FE0-8C85-E9003EF6A07A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11268075" y="15144750"/>
+          <a:ext cx="3705225" cy="5000625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3705225" cy="5000625"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="81" name="Picture 80">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{89790AB7-0203-4DD1-9C5F-AD875CABE92B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3965,7 +3886,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="7391400" y="19926300"/>
+          <a:off x="11268075" y="20126325"/>
           <a:ext cx="3705225" cy="5000625"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3984,68 +3905,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE9ED85E-3DA5-B5A1-932D-D8944C0DEEC1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11087100" y="19926300"/>
-          <a:ext cx="3705225" cy="5000625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4736,7 +4596,7 @@
   <sheetPr>
     <tabColor theme="7"/>
   </sheetPr>
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:AA22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="137" customWidth="1"/>
@@ -4756,12 +4616,16 @@
     <col min="18" max="18" width="10.85546875" customWidth="1"/>
     <col min="19" max="19" width="25.7109375" customWidth="1"/>
     <col min="20" max="20" width="10.85546875" customWidth="1"/>
-    <col min="21" max="21" width="4" customWidth="1"/>
-    <col min="22" max="22" width="2.7109375" style="137" customWidth="1"/>
+    <col min="21" max="22" width="4" customWidth="1"/>
+    <col min="23" max="23" width="10.85546875" customWidth="1"/>
+    <col min="24" max="24" width="25.7109375" customWidth="1"/>
+    <col min="25" max="25" width="10.85546875" customWidth="1"/>
+    <col min="26" max="26" width="4" customWidth="1"/>
+    <col min="27" max="27" width="2.7109375" style="137" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="137" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="137" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="35"/>
       <c r="C2" s="36"/>
       <c r="D2" s="36"/>
@@ -4782,8 +4646,13 @@
       <c r="S2" s="6"/>
       <c r="T2" s="6"/>
       <c r="U2" s="25"/>
+      <c r="V2" s="9"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10"/>
+      <c r="Z2" s="117"/>
     </row>
-    <row r="3" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="138"/>
       <c r="B3" s="38"/>
       <c r="C3" s="39"/>
@@ -4817,9 +4686,17 @@
       </c>
       <c r="T3" s="27"/>
       <c r="U3" s="28"/>
-      <c r="V3" s="138"/>
+      <c r="V3" s="118"/>
+      <c r="W3" s="119"/>
+      <c r="X3" s="120" t="str">
+        <f>'Cards Src'!$A6</f>
+        <v>LIGHTNING BOLT</v>
+      </c>
+      <c r="Y3" s="119"/>
+      <c r="Z3" s="121"/>
+      <c r="AA3" s="138"/>
     </row>
-    <row r="4" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="41"/>
       <c r="C4" s="139" t="e" vm="1">
         <f>'Cards Src'!E2</f>
@@ -4852,8 +4729,16 @@
       <c r="S4" s="146"/>
       <c r="T4" s="146"/>
       <c r="U4" s="29"/>
+      <c r="V4" s="11"/>
+      <c r="W4" s="147" t="e" vm="5">
+        <f>'Cards Src'!E6</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="X4" s="147"/>
+      <c r="Y4" s="147"/>
+      <c r="Z4" s="126"/>
     </row>
-    <row r="5" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="41"/>
       <c r="C5" s="140" t="str">
         <f>'Cards Src'!$C2</f>
@@ -4886,8 +4771,16 @@
       <c r="S5" s="143"/>
       <c r="T5" s="143"/>
       <c r="U5" s="30"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="148" t="str">
+        <f>'Cards Src'!$C6</f>
+        <v>Casts a bolt of lightning</v>
+      </c>
+      <c r="X5" s="148"/>
+      <c r="Y5" s="148"/>
+      <c r="Z5" s="123"/>
     </row>
-    <row r="6" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="44"/>
       <c r="C6" s="45"/>
       <c r="D6" s="45"/>
@@ -4908,161 +4801,200 @@
       <c r="S6" s="31"/>
       <c r="T6" s="31"/>
       <c r="U6" s="32"/>
+      <c r="V6" s="12"/>
+      <c r="W6" s="124"/>
+      <c r="X6" s="124"/>
+      <c r="Y6" s="124"/>
+      <c r="Z6" s="125"/>
     </row>
-    <row r="7" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="9"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="117"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="68"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="18"/>
-      <c r="P7" s="76"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="117"/>
+    <row r="7" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="13"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="76"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="117"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="18"/>
+      <c r="U7" s="76"/>
+      <c r="V7" s="100"/>
+      <c r="W7" s="101"/>
+      <c r="X7" s="101"/>
+      <c r="Y7" s="101"/>
+      <c r="Z7" s="102"/>
     </row>
-    <row r="8" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="138"/>
-      <c r="B8" s="118"/>
-      <c r="C8" s="119"/>
-      <c r="D8" s="120" t="str">
-        <f>'Cards Src'!$A6</f>
-        <v>LIGHTNING BOLT</v>
-      </c>
-      <c r="E8" s="119"/>
-      <c r="F8" s="121"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="86" t="str">
+      <c r="B8" s="69"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="86" t="str">
         <f>'Cards Src'!A7</f>
         <v>BLACK HOLE</v>
       </c>
-      <c r="J8" s="70"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="77"/>
-      <c r="M8" s="78"/>
-      <c r="N8" s="79" t="str">
+      <c r="E8" s="70"/>
+      <c r="F8" s="71"/>
+      <c r="G8" s="77"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="79" t="str">
         <f>'Cards Src'!A8</f>
         <v>ASTRAL DAGGER</v>
       </c>
-      <c r="O8" s="78"/>
-      <c r="P8" s="80"/>
-      <c r="Q8" s="118"/>
-      <c r="R8" s="119"/>
-      <c r="S8" s="120" t="str">
+      <c r="J8" s="78"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="118"/>
+      <c r="M8" s="119"/>
+      <c r="N8" s="120" t="str">
         <f>'Cards Src'!A9</f>
         <v>CHAIN LIGHTNING</v>
       </c>
-      <c r="T8" s="119"/>
-      <c r="U8" s="121"/>
-      <c r="V8" s="138"/>
+      <c r="O8" s="119"/>
+      <c r="P8" s="121"/>
+      <c r="Q8" s="77"/>
+      <c r="R8" s="78"/>
+      <c r="S8" s="79" t="str">
+        <f>'Cards Src'!$A10</f>
+        <v>DIVINE JUDGEMENT</v>
+      </c>
+      <c r="T8" s="78"/>
+      <c r="U8" s="80"/>
+      <c r="V8" s="103"/>
+      <c r="W8" s="104"/>
+      <c r="X8" s="105" t="str">
+        <f>'Cards Src'!A11</f>
+        <v>HASTE</v>
+      </c>
+      <c r="Y8" s="104"/>
+      <c r="Z8" s="106"/>
+      <c r="AA8" s="138"/>
     </row>
-    <row r="9" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="11"/>
-      <c r="C9" s="147" t="e" vm="5">
-        <f>'Cards Src'!E6</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D9" s="147"/>
-      <c r="E9" s="147"/>
-      <c r="F9" s="126"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="151" t="e" vm="6">
+    <row r="9" spans="1:27" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="15"/>
+      <c r="C9" s="151" t="e" vm="6">
         <f>'Cards Src'!E7</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I9" s="151"/>
-      <c r="J9" s="151"/>
-      <c r="K9" s="72"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="152" t="e" vm="7">
+      <c r="D9" s="151"/>
+      <c r="E9" s="151"/>
+      <c r="F9" s="72"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="152" t="e" vm="7">
         <f>'Cards Src'!E8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="N9" s="152"/>
-      <c r="O9" s="152"/>
-      <c r="P9" s="81"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="147" t="e" vm="8">
+      <c r="I9" s="152"/>
+      <c r="J9" s="152"/>
+      <c r="K9" s="81"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="147" t="e" vm="8">
         <f>'Cards Src'!E9</f>
         <v>#VALUE!</v>
       </c>
-      <c r="S9" s="147"/>
-      <c r="T9" s="147"/>
-      <c r="U9" s="122"/>
+      <c r="N9" s="147"/>
+      <c r="O9" s="147"/>
+      <c r="P9" s="122"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="152" t="e" vm="9">
+        <f>'Cards Src'!E10</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="S9" s="152"/>
+      <c r="T9" s="152"/>
+      <c r="U9" s="81"/>
+      <c r="V9" s="107"/>
+      <c r="W9" s="155" t="e" vm="10">
+        <f>'Cards Src'!E11</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="X9" s="155"/>
+      <c r="Y9" s="155"/>
+      <c r="Z9" s="108"/>
     </row>
-    <row r="10" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="11"/>
-      <c r="C10" s="148" t="str">
-        <f>'Cards Src'!$C6</f>
-        <v>Casts a bolt of lightning</v>
-      </c>
-      <c r="D10" s="148"/>
-      <c r="E10" s="148"/>
-      <c r="F10" s="123"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="149" t="str">
+    <row r="10" spans="1:27" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="15"/>
+      <c r="C10" s="149" t="str">
         <f>'Cards Src'!$C7</f>
         <v>Vacuums in nearby enemies</v>
       </c>
-      <c r="I10" s="149"/>
-      <c r="J10" s="149"/>
-      <c r="K10" s="73"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="150" t="str">
+      <c r="D10" s="149"/>
+      <c r="E10" s="149"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="150" t="str">
         <f>'Cards Src'!C8</f>
         <v>Flies to the nearest enemy in vision</v>
       </c>
-      <c r="N10" s="150"/>
-      <c r="O10" s="150"/>
-      <c r="P10" s="82"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="148" t="str">
+      <c r="I10" s="150"/>
+      <c r="J10" s="150"/>
+      <c r="K10" s="82"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="148" t="str">
         <f>'Cards Src'!C9</f>
         <v>Casts a tracking bolt of lightning that can chain to close enemies</v>
       </c>
-      <c r="S10" s="148"/>
-      <c r="T10" s="148"/>
-      <c r="U10" s="123"/>
+      <c r="N10" s="148"/>
+      <c r="O10" s="148"/>
+      <c r="P10" s="123"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="153" t="str">
+        <f>'Cards Src'!$C10</f>
+        <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
+      </c>
+      <c r="S10" s="153"/>
+      <c r="T10" s="153"/>
+      <c r="U10" s="82"/>
+      <c r="V10" s="107"/>
+      <c r="W10" s="154" t="str">
+        <f>'Cards Src'!$C11</f>
+        <v>Increases player movement speed for a set duration</v>
+      </c>
+      <c r="X10" s="154"/>
+      <c r="Y10" s="154"/>
+      <c r="Z10" s="110"/>
     </row>
-    <row r="11" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="12"/>
-      <c r="C11" s="124"/>
-      <c r="D11" s="124"/>
-      <c r="E11" s="124"/>
-      <c r="F11" s="125"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="74"/>
-      <c r="I11" s="74"/>
-      <c r="J11" s="74"/>
-      <c r="K11" s="75"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="83"/>
-      <c r="N11" s="83"/>
-      <c r="O11" s="83"/>
-      <c r="P11" s="84"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="124"/>
-      <c r="S11" s="124"/>
-      <c r="T11" s="124"/>
-      <c r="U11" s="125"/>
+    <row r="11" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="16"/>
+      <c r="C11" s="74"/>
+      <c r="D11" s="74"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="75"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="83"/>
+      <c r="I11" s="83"/>
+      <c r="J11" s="83"/>
+      <c r="K11" s="84"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="124"/>
+      <c r="N11" s="124"/>
+      <c r="O11" s="124"/>
+      <c r="P11" s="125"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="83"/>
+      <c r="S11" s="83"/>
+      <c r="T11" s="83"/>
+      <c r="U11" s="84"/>
+      <c r="V11" s="111"/>
+      <c r="W11" s="112"/>
+      <c r="X11" s="112"/>
+      <c r="Y11" s="112"/>
+      <c r="Z11" s="113"/>
     </row>
-    <row r="12" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="17"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="76"/>
+    <row r="12" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="100"/>
+      <c r="C12" s="101"/>
+      <c r="D12" s="101"/>
+      <c r="E12" s="101"/>
+      <c r="F12" s="102"/>
       <c r="G12" s="100"/>
       <c r="H12" s="101"/>
       <c r="I12" s="101"/>
@@ -5078,117 +5010,146 @@
       <c r="S12" s="101"/>
       <c r="T12" s="101"/>
       <c r="U12" s="102"/>
+      <c r="V12" s="100"/>
+      <c r="W12" s="101"/>
+      <c r="X12" s="101"/>
+      <c r="Y12" s="101"/>
+      <c r="Z12" s="102"/>
     </row>
-    <row r="13" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="138"/>
-      <c r="B13" s="77"/>
-      <c r="C13" s="78"/>
-      <c r="D13" s="79" t="str">
-        <f>'Cards Src'!$A10</f>
-        <v>DIVINE JUDGEMENT</v>
-      </c>
-      <c r="E13" s="78"/>
-      <c r="F13" s="80"/>
+      <c r="B13" s="103"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="105" t="str">
+        <f>'Cards Src'!A12</f>
+        <v>HINDER</v>
+      </c>
+      <c r="E13" s="104"/>
+      <c r="F13" s="106"/>
       <c r="G13" s="103"/>
       <c r="H13" s="104"/>
-      <c r="I13" s="105" t="str">
-        <f>'Cards Src'!A11</f>
-        <v>HASTE</v>
+      <c r="I13" s="114" t="str">
+        <f>'Cards Src'!A13</f>
+        <v>MULLIGAN</v>
       </c>
       <c r="J13" s="104"/>
       <c r="K13" s="106"/>
       <c r="L13" s="103"/>
       <c r="M13" s="104"/>
-      <c r="N13" s="105" t="str">
-        <f>'Cards Src'!A12</f>
-        <v>HINDER</v>
+      <c r="N13" s="109" t="str">
+        <f>'Cards Src'!$A14</f>
+        <v>BUT WAIT, THERE'S MORE</v>
       </c>
       <c r="O13" s="104"/>
       <c r="P13" s="106"/>
       <c r="Q13" s="103"/>
       <c r="R13" s="104"/>
-      <c r="S13" s="114" t="str">
-        <f>'Cards Src'!A13</f>
-        <v>MULLIGAN</v>
+      <c r="S13" s="115" t="str">
+        <f>'Cards Src'!A15</f>
+        <v>MANA SHIELD</v>
       </c>
       <c r="T13" s="104"/>
       <c r="U13" s="106"/>
-      <c r="V13" s="138"/>
+      <c r="V13" s="103"/>
+      <c r="W13" s="104"/>
+      <c r="X13" s="115" t="str">
+        <f>'Cards Src'!A16</f>
+        <v>RUNAWAY BULL</v>
+      </c>
+      <c r="Y13" s="104"/>
+      <c r="Z13" s="106"/>
+      <c r="AA13" s="138"/>
     </row>
-    <row r="14" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="19"/>
-      <c r="C14" s="152" t="e" vm="9">
-        <f>'Cards Src'!E10</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D14" s="152"/>
-      <c r="E14" s="152"/>
-      <c r="F14" s="81"/>
+    <row r="14" spans="1:27" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="107"/>
+      <c r="C14" s="156" t="e" vm="11">
+        <f>'Cards Src'!E12</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D14" s="156"/>
+      <c r="E14" s="156"/>
+      <c r="F14" s="108"/>
       <c r="G14" s="107"/>
-      <c r="H14" s="155" t="e" vm="10">
-        <f>'Cards Src'!E11</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I14" s="155"/>
-      <c r="J14" s="155"/>
+      <c r="H14" s="156" t="e" vm="12">
+        <f xml:space="preserve"> 'Cards Src'!E13</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I14" s="156"/>
+      <c r="J14" s="156"/>
       <c r="K14" s="108"/>
       <c r="L14" s="107"/>
-      <c r="M14" s="156" t="e" vm="11">
-        <f>'Cards Src'!E12</f>
+      <c r="M14" s="156" t="e" vm="13">
+        <f>'Cards Src'!E14</f>
         <v>#VALUE!</v>
       </c>
       <c r="N14" s="156"/>
       <c r="O14" s="156"/>
       <c r="P14" s="108"/>
       <c r="Q14" s="107"/>
-      <c r="R14" s="156" t="e" vm="12">
-        <f xml:space="preserve"> 'Cards Src'!E13</f>
+      <c r="R14" s="156" t="e" vm="14">
+        <f>'Cards Src'!E15</f>
         <v>#VALUE!</v>
       </c>
       <c r="S14" s="156"/>
       <c r="T14" s="156"/>
       <c r="U14" s="108"/>
+      <c r="V14" s="107"/>
+      <c r="W14" s="156" t="e" vm="15">
+        <f>'Cards Src'!E16</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="X14" s="156"/>
+      <c r="Y14" s="156"/>
+      <c r="Z14" s="108"/>
     </row>
-    <row r="15" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="19"/>
-      <c r="C15" s="153" t="str">
-        <f>'Cards Src'!$C10</f>
-        <v>Creates an area on the ground that damages to enemies within it. Mark any enemy to deal damage to the enemy proportional to the time spent once finishes</v>
-      </c>
-      <c r="D15" s="153"/>
-      <c r="E15" s="153"/>
-      <c r="F15" s="82"/>
+    <row r="15" spans="1:27" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="107"/>
+      <c r="C15" s="154" t="str">
+        <f>'Cards Src'!C12</f>
+        <v>Enemies are temporarily slowed on hit for a set duration.</v>
+      </c>
+      <c r="D15" s="154"/>
+      <c r="E15" s="154"/>
+      <c r="F15" s="110"/>
       <c r="G15" s="107"/>
       <c r="H15" s="154" t="str">
-        <f>'Cards Src'!$C11</f>
-        <v>Increases player movement speed for a set duration</v>
+        <f>'Cards Src'!C13</f>
+        <v>Randomly swap two cards in the current hand with cards in the deck</v>
       </c>
       <c r="I15" s="154"/>
       <c r="J15" s="154"/>
       <c r="K15" s="110"/>
       <c r="L15" s="107"/>
       <c r="M15" s="154" t="str">
-        <f>'Cards Src'!C12</f>
-        <v>Enemies are temporarily slowed on hit for a set duration.</v>
+        <f>'Cards Src'!$C14</f>
+        <v>Randomly shuffle two cards from the discard pile back into the deck</v>
       </c>
       <c r="N15" s="154"/>
       <c r="O15" s="154"/>
       <c r="P15" s="110"/>
       <c r="Q15" s="107"/>
       <c r="R15" s="154" t="str">
-        <f>'Cards Src'!C13</f>
-        <v>Randomly swap two cards in the current hand with cards in the deck</v>
+        <f>'Cards Src'!$C15</f>
+        <v>Negate x number of hits</v>
       </c>
       <c r="S15" s="154"/>
       <c r="T15" s="154"/>
       <c r="U15" s="110"/>
+      <c r="V15" s="107"/>
+      <c r="W15" s="157" t="str">
+        <f>'Cards Src'!C16</f>
+        <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
+      </c>
+      <c r="X15" s="157"/>
+      <c r="Y15" s="157"/>
+      <c r="Z15" s="110"/>
     </row>
-    <row r="16" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="20"/>
-      <c r="C16" s="83"/>
-      <c r="D16" s="83"/>
-      <c r="E16" s="83"/>
-      <c r="F16" s="84"/>
+    <row r="16" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="111"/>
+      <c r="C16" s="112"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="112"/>
+      <c r="F16" s="113"/>
       <c r="G16" s="111"/>
       <c r="H16" s="112"/>
       <c r="I16" s="112"/>
@@ -5204,8 +5165,13 @@
       <c r="S16" s="112"/>
       <c r="T16" s="112"/>
       <c r="U16" s="113"/>
+      <c r="V16" s="111"/>
+      <c r="W16" s="112"/>
+      <c r="X16" s="112"/>
+      <c r="Y16" s="112"/>
+      <c r="Z16" s="113"/>
     </row>
-    <row r="17" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="100"/>
       <c r="C17" s="101"/>
       <c r="D17" s="101"/>
@@ -5221,117 +5187,146 @@
       <c r="N17" s="101"/>
       <c r="O17" s="101"/>
       <c r="P17" s="102"/>
-      <c r="Q17" s="100"/>
-      <c r="R17" s="101"/>
-      <c r="S17" s="101"/>
-      <c r="T17" s="101"/>
-      <c r="U17" s="102"/>
+      <c r="Q17" s="87"/>
+      <c r="R17" s="88"/>
+      <c r="S17" s="88"/>
+      <c r="T17" s="88"/>
+      <c r="U17" s="89"/>
+      <c r="V17" s="87"/>
+      <c r="W17" s="88"/>
+      <c r="X17" s="88"/>
+      <c r="Y17" s="88"/>
+      <c r="Z17" s="89"/>
     </row>
-    <row r="18" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="138"/>
       <c r="B18" s="103"/>
       <c r="C18" s="104"/>
-      <c r="D18" s="109" t="str">
-        <f>'Cards Src'!$A14</f>
-        <v>BUT WAIT, THERE'S MORE</v>
+      <c r="D18" s="128" t="str">
+        <f>'Cards Src'!A17</f>
+        <v>HOLY BLADE</v>
       </c>
       <c r="E18" s="104"/>
       <c r="F18" s="106"/>
       <c r="G18" s="103"/>
       <c r="H18" s="104"/>
-      <c r="I18" s="115" t="str">
-        <f>'Cards Src'!A15</f>
-        <v>MANA SHIELD</v>
+      <c r="I18" s="105" t="str">
+        <f>'Cards Src'!$A18</f>
+        <v>RECALL</v>
       </c>
       <c r="J18" s="104"/>
       <c r="K18" s="106"/>
       <c r="L18" s="103"/>
       <c r="M18" s="104"/>
-      <c r="N18" s="115" t="str">
-        <f>'Cards Src'!A16</f>
-        <v>RUNAWAY BULL</v>
+      <c r="N18" s="105" t="str">
+        <f>'Cards Src'!A19</f>
+        <v>GREED</v>
       </c>
       <c r="O18" s="104"/>
       <c r="P18" s="106"/>
-      <c r="Q18" s="103"/>
-      <c r="R18" s="104"/>
-      <c r="S18" s="128" t="str">
-        <f>'Cards Src'!A17</f>
-        <v>HOLY BLADE</v>
-      </c>
-      <c r="T18" s="104"/>
-      <c r="U18" s="106"/>
-      <c r="V18" s="138"/>
+      <c r="Q18" s="90"/>
+      <c r="R18" s="91"/>
+      <c r="S18" s="92">
+        <f>'Cards Src'!F15</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="91"/>
+      <c r="U18" s="93"/>
+      <c r="V18" s="90"/>
+      <c r="W18" s="91"/>
+      <c r="X18" s="92">
+        <f>'Cards Src'!F16</f>
+        <v>0</v>
+      </c>
+      <c r="Y18" s="91"/>
+      <c r="Z18" s="93"/>
+      <c r="AA18" s="138"/>
     </row>
-    <row r="19" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="107"/>
-      <c r="C19" s="156" t="e" vm="13">
-        <f>'Cards Src'!E14</f>
+      <c r="C19" s="156" t="e" vm="16">
+        <f xml:space="preserve"> 'Cards Src'!E17</f>
         <v>#VALUE!</v>
       </c>
       <c r="D19" s="156"/>
       <c r="E19" s="156"/>
       <c r="F19" s="108"/>
       <c r="G19" s="107"/>
-      <c r="H19" s="156" t="e" vm="14">
-        <f>'Cards Src'!E15</f>
+      <c r="H19" s="156" t="e" vm="17">
+        <f>'Cards Src'!E18</f>
         <v>#VALUE!</v>
       </c>
       <c r="I19" s="156"/>
       <c r="J19" s="156"/>
       <c r="K19" s="108"/>
       <c r="L19" s="107"/>
-      <c r="M19" s="156" t="e" vm="15">
-        <f>'Cards Src'!E16</f>
+      <c r="M19" s="156" t="e" vm="18">
+        <f>'Cards Src'!E19</f>
         <v>#VALUE!</v>
       </c>
       <c r="N19" s="156"/>
       <c r="O19" s="156"/>
       <c r="P19" s="108"/>
-      <c r="Q19" s="107"/>
-      <c r="R19" s="156" t="e" vm="16">
-        <f xml:space="preserve"> 'Cards Src'!E17</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="S19" s="156"/>
-      <c r="T19" s="156"/>
-      <c r="U19" s="108"/>
+      <c r="Q19" s="94"/>
+      <c r="R19" s="159">
+        <f>'Cards Src'!J15</f>
+        <v>0</v>
+      </c>
+      <c r="S19" s="159"/>
+      <c r="T19" s="159"/>
+      <c r="U19" s="95"/>
+      <c r="V19" s="94"/>
+      <c r="W19" s="159">
+        <f xml:space="preserve"> 'Cards Src'!J16</f>
+        <v>0</v>
+      </c>
+      <c r="X19" s="159"/>
+      <c r="Y19" s="159"/>
+      <c r="Z19" s="95"/>
     </row>
-    <row r="20" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="107"/>
       <c r="C20" s="154" t="str">
-        <f>'Cards Src'!$C14</f>
-        <v>Randomly shuffle two cards from the discard pile back into the deck</v>
+        <f>'Cards Src'!C17</f>
+        <v>Increase damage of your weapon by x for a certain amount of time</v>
       </c>
       <c r="D20" s="154"/>
       <c r="E20" s="154"/>
       <c r="F20" s="110"/>
       <c r="G20" s="107"/>
       <c r="H20" s="154" t="str">
-        <f>'Cards Src'!$C15</f>
-        <v>Negate x number of hits</v>
+        <f>'Cards Src'!$C18</f>
+        <v>Recall last used card into deck</v>
       </c>
       <c r="I20" s="154"/>
       <c r="J20" s="154"/>
       <c r="K20" s="110"/>
       <c r="L20" s="107"/>
-      <c r="M20" s="157" t="str">
-        <f>'Cards Src'!C16</f>
-        <v>For a temporary amount of time, causes the player's dashes to push enemies away slightly and inflict damage</v>
-      </c>
-      <c r="N20" s="157"/>
-      <c r="O20" s="157"/>
+      <c r="M20" s="154" t="str">
+        <f>'Cards Src'!$C19</f>
+        <v>Draw 2 cards</v>
+      </c>
+      <c r="N20" s="154"/>
+      <c r="O20" s="154"/>
       <c r="P20" s="110"/>
-      <c r="Q20" s="107"/>
-      <c r="R20" s="154" t="str">
-        <f>'Cards Src'!C17</f>
-        <v>Increase damage of your weapon by x for a certain amount of time</v>
-      </c>
-      <c r="S20" s="154"/>
-      <c r="T20" s="154"/>
-      <c r="U20" s="110"/>
+      <c r="Q20" s="94"/>
+      <c r="R20" s="158">
+        <f>'Cards Src'!H15</f>
+        <v>0</v>
+      </c>
+      <c r="S20" s="158"/>
+      <c r="T20" s="158"/>
+      <c r="U20" s="96"/>
+      <c r="V20" s="94"/>
+      <c r="W20" s="158">
+        <f>'Cards Src'!H16</f>
+        <v>0</v>
+      </c>
+      <c r="X20" s="158"/>
+      <c r="Y20" s="158"/>
+      <c r="Z20" s="96"/>
     </row>
-    <row r="21" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="111"/>
       <c r="C21" s="112"/>
       <c r="D21" s="112"/>
@@ -5347,171 +5342,28 @@
       <c r="N21" s="112"/>
       <c r="O21" s="112"/>
       <c r="P21" s="113"/>
-      <c r="Q21" s="111"/>
-      <c r="R21" s="112"/>
-      <c r="S21" s="112"/>
-      <c r="T21" s="112"/>
-      <c r="U21" s="113"/>
+      <c r="Q21" s="97"/>
+      <c r="R21" s="98"/>
+      <c r="S21" s="98"/>
+      <c r="T21" s="98"/>
+      <c r="U21" s="99"/>
+      <c r="V21" s="97"/>
+      <c r="W21" s="98"/>
+      <c r="X21" s="98"/>
+      <c r="Y21" s="98"/>
+      <c r="Z21" s="99"/>
     </row>
-    <row r="22" spans="1:22" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="100"/>
-      <c r="C22" s="101"/>
-      <c r="D22" s="101"/>
-      <c r="E22" s="101"/>
-      <c r="F22" s="102"/>
-      <c r="G22" s="100"/>
-      <c r="H22" s="101"/>
-      <c r="I22" s="101"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="87"/>
-      <c r="M22" s="88"/>
-      <c r="N22" s="88"/>
-      <c r="O22" s="88"/>
-      <c r="P22" s="89"/>
-      <c r="Q22" s="87"/>
-      <c r="R22" s="88"/>
-      <c r="S22" s="88"/>
-      <c r="T22" s="88"/>
-      <c r="U22" s="89"/>
-    </row>
-    <row r="23" spans="1:22" s="21" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="138"/>
-      <c r="B23" s="103"/>
-      <c r="C23" s="104"/>
-      <c r="D23" s="105" t="str">
-        <f>'Cards Src'!$A18</f>
-        <v>RECALL</v>
-      </c>
-      <c r="E23" s="104"/>
-      <c r="F23" s="106"/>
-      <c r="G23" s="103"/>
-      <c r="H23" s="104"/>
-      <c r="I23" s="105" t="str">
-        <f>'Cards Src'!A19</f>
-        <v>GREED</v>
-      </c>
-      <c r="J23" s="104"/>
-      <c r="K23" s="106"/>
-      <c r="L23" s="90"/>
-      <c r="M23" s="91"/>
-      <c r="N23" s="92">
-        <f>'Cards Src'!A20</f>
-        <v>0</v>
-      </c>
-      <c r="O23" s="91"/>
-      <c r="P23" s="93"/>
-      <c r="Q23" s="90"/>
-      <c r="R23" s="91"/>
-      <c r="S23" s="92">
-        <f>'Cards Src'!A21</f>
-        <v>0</v>
-      </c>
-      <c r="T23" s="91"/>
-      <c r="U23" s="93"/>
-      <c r="V23" s="138"/>
-    </row>
-    <row r="24" spans="1:22" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="107"/>
-      <c r="C24" s="156" t="e" vm="17">
-        <f>'Cards Src'!E18</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D24" s="156"/>
-      <c r="E24" s="156"/>
-      <c r="F24" s="108"/>
-      <c r="G24" s="107"/>
-      <c r="H24" s="156" t="e" vm="18">
-        <f>'Cards Src'!E19</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="156"/>
-      <c r="J24" s="156"/>
-      <c r="K24" s="108"/>
-      <c r="L24" s="94"/>
-      <c r="M24" s="159">
-        <f>'Cards Src'!E20</f>
-        <v>0</v>
-      </c>
-      <c r="N24" s="159"/>
-      <c r="O24" s="159"/>
-      <c r="P24" s="95"/>
-      <c r="Q24" s="94"/>
-      <c r="R24" s="159">
-        <f xml:space="preserve"> 'Cards Src'!E21</f>
-        <v>0</v>
-      </c>
-      <c r="S24" s="159"/>
-      <c r="T24" s="159"/>
-      <c r="U24" s="95"/>
-    </row>
-    <row r="25" spans="1:22" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="107"/>
-      <c r="C25" s="154" t="str">
-        <f>'Cards Src'!$C18</f>
-        <v>Recall last used card into deck</v>
-      </c>
-      <c r="D25" s="154"/>
-      <c r="E25" s="154"/>
-      <c r="F25" s="110"/>
-      <c r="G25" s="107"/>
-      <c r="H25" s="154" t="str">
-        <f>'Cards Src'!$C19</f>
-        <v>Draw 2 cards</v>
-      </c>
-      <c r="I25" s="154"/>
-      <c r="J25" s="154"/>
-      <c r="K25" s="110"/>
-      <c r="L25" s="94"/>
-      <c r="M25" s="158">
-        <f>'Cards Src'!C20</f>
-        <v>0</v>
-      </c>
-      <c r="N25" s="158"/>
-      <c r="O25" s="158"/>
-      <c r="P25" s="96"/>
-      <c r="Q25" s="94"/>
-      <c r="R25" s="158">
-        <f>'Cards Src'!C21</f>
-        <v>0</v>
-      </c>
-      <c r="S25" s="158"/>
-      <c r="T25" s="158"/>
-      <c r="U25" s="96"/>
-    </row>
-    <row r="26" spans="1:22" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="111"/>
-      <c r="C26" s="112"/>
-      <c r="D26" s="112"/>
-      <c r="E26" s="112"/>
-      <c r="F26" s="113"/>
-      <c r="G26" s="111"/>
-      <c r="H26" s="112"/>
-      <c r="I26" s="112"/>
-      <c r="J26" s="112"/>
-      <c r="K26" s="113"/>
-      <c r="L26" s="97"/>
-      <c r="M26" s="98"/>
-      <c r="N26" s="98"/>
-      <c r="O26" s="98"/>
-      <c r="P26" s="99"/>
-      <c r="Q26" s="97"/>
-      <c r="R26" s="98"/>
-      <c r="S26" s="98"/>
-      <c r="T26" s="98"/>
-      <c r="U26" s="99"/>
-    </row>
-    <row r="27" spans="1:22" s="137" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:27" s="137" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="M25:O25"/>
-    <mergeCell ref="R25:T25"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="M24:O24"/>
-    <mergeCell ref="R24:T24"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="W19:Y19"/>
+    <mergeCell ref="W20:Y20"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="W5:Y5"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="W14:Y14"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="H20:J20"/>

</xml_diff>

<commit_message>
Icons - Last batch of art
Added card icons for Black Hole, Divine Judgement, and Runaway Bull
</commit_message>
<xml_diff>
--- a/Assets/Documents/Concept Art/Cards by Layer.xlsx
+++ b/Assets/Documents/Concept Art/Cards by Layer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\willc\My Stuff\School\CSC 486C\Assets\Card Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1B3B34-0E18-41D8-BAFB-3E970CB0A55A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C2EAEC-CE59-49F8-B00D-741B1E958272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1953,7 +1953,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26430"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26462"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2018,7 +2018,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26431"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26463"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2249,7 +2249,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26432"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26464"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2365,7 +2365,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26433"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26465"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2481,7 +2481,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26434"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26466"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2597,7 +2597,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26435"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26467"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2713,7 +2713,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26436"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26468"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2829,7 +2829,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26437"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26469"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -2945,7 +2945,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26438"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26470"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3061,7 +3061,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26439"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26471"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3177,7 +3177,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26440"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26472"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3293,7 +3293,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26441"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26473"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3409,7 +3409,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26442"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26474"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3525,7 +3525,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26443"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26475"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3641,7 +3641,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26444"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26476"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -3757,7 +3757,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26445"/>
+                  <a14:cameraTool cellRange="'Cards Src'!#REF!" spid="_x0000_s26477"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>

</xml_diff>